<commit_message>
Planogram: empty zones are STOCK areas (labelled STOCK on screen and PNG); Excel status 'Zona STOCK'
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGHS9u6kQyg6PXbaVYikDd
</commit_message>
<xml_diff>
--- a/data_planogram_terisi.xlsx
+++ b/data_planogram_terisi.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>OK / Zona kosong / Belum ditempatkan / CEK + penyebab. Semua baris yang ditempatkan harus OK sebelum diimpor.</t>
+          <t>OK / Zona STOCK (tanpa item) / Belum ditempatkan / CEK + penyebab. Semua baris yang ditempatkan harus OK sebelum diimpor.</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>4. Baris yang hanya berisi ID FIXTURE + ZONA NO (SKU kosong) = zona dibiarkan kosong.</t>
+          <t>4. Zona yang tidak berisi item (baris ID FIXTURE + ZONA NO tanpa SKU, atau zona yang tidak ditulis sama sekali) dianggap tempat STOCK dan ditulis STOCK di planogram.</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
         <v/>
       </c>
       <c r="M2" s="12">
-        <f>IF(AND(A2="",F2=""),"",IF(F2="","Belum ditempatkan",IF(I2="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G2="","CEK ZONA NO kosong",IF(K2="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H2&lt;&gt;K2,"CEK JENIS ZONA",IF(A2="","Zona kosong",IF(B2="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A2="",F2=""),"",IF(F2="","Belum ditempatkan",IF(I2="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G2="","CEK ZONA NO kosong",IF(K2="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H2&lt;&gt;K2,"CEK JENIS ZONA",IF(A2="","Zona STOCK",IF(B2="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
         <v/>
       </c>
       <c r="M3" s="12">
-        <f>IF(AND(A3="",F3=""),"",IF(F3="","Belum ditempatkan",IF(I3="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G3="","CEK ZONA NO kosong",IF(K3="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H3&lt;&gt;K3,"CEK JENIS ZONA",IF(A3="","Zona kosong",IF(B3="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A3="",F3=""),"",IF(F3="","Belum ditempatkan",IF(I3="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G3="","CEK ZONA NO kosong",IF(K3="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H3&lt;&gt;K3,"CEK JENIS ZONA",IF(A3="","Zona STOCK",IF(B3="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
         <v/>
       </c>
       <c r="M4" s="12">
-        <f>IF(AND(A4="",F4=""),"",IF(F4="","Belum ditempatkan",IF(I4="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G4="","CEK ZONA NO kosong",IF(K4="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H4&lt;&gt;K4,"CEK JENIS ZONA",IF(A4="","Zona kosong",IF(B4="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A4="",F4=""),"",IF(F4="","Belum ditempatkan",IF(I4="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G4="","CEK ZONA NO kosong",IF(K4="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H4&lt;&gt;K4,"CEK JENIS ZONA",IF(A4="","Zona STOCK",IF(B4="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
         <v/>
       </c>
       <c r="M5" s="12">
-        <f>IF(AND(A5="",F5=""),"",IF(F5="","Belum ditempatkan",IF(I5="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G5="","CEK ZONA NO kosong",IF(K5="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H5&lt;&gt;K5,"CEK JENIS ZONA",IF(A5="","Zona kosong",IF(B5="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A5="",F5=""),"",IF(F5="","Belum ditempatkan",IF(I5="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G5="","CEK ZONA NO kosong",IF(K5="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H5&lt;&gt;K5,"CEK JENIS ZONA",IF(A5="","Zona STOCK",IF(B5="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
         <v/>
       </c>
       <c r="M6" s="12">
-        <f>IF(AND(A6="",F6=""),"",IF(F6="","Belum ditempatkan",IF(I6="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G6="","CEK ZONA NO kosong",IF(K6="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H6&lt;&gt;K6,"CEK JENIS ZONA",IF(A6="","Zona kosong",IF(B6="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A6="",F6=""),"",IF(F6="","Belum ditempatkan",IF(I6="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G6="","CEK ZONA NO kosong",IF(K6="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H6&lt;&gt;K6,"CEK JENIS ZONA",IF(A6="","Zona STOCK",IF(B6="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
         <v/>
       </c>
       <c r="M7" s="12">
-        <f>IF(AND(A7="",F7=""),"",IF(F7="","Belum ditempatkan",IF(I7="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G7="","CEK ZONA NO kosong",IF(K7="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H7&lt;&gt;K7,"CEK JENIS ZONA",IF(A7="","Zona kosong",IF(B7="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A7="",F7=""),"",IF(F7="","Belum ditempatkan",IF(I7="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G7="","CEK ZONA NO kosong",IF(K7="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H7&lt;&gt;K7,"CEK JENIS ZONA",IF(A7="","Zona STOCK",IF(B7="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
         <v/>
       </c>
       <c r="M8" s="12">
-        <f>IF(AND(A8="",F8=""),"",IF(F8="","Belum ditempatkan",IF(I8="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G8="","CEK ZONA NO kosong",IF(K8="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H8&lt;&gt;K8,"CEK JENIS ZONA",IF(A8="","Zona kosong",IF(B8="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A8="",F8=""),"",IF(F8="","Belum ditempatkan",IF(I8="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G8="","CEK ZONA NO kosong",IF(K8="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H8&lt;&gt;K8,"CEK JENIS ZONA",IF(A8="","Zona STOCK",IF(B8="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
         <v/>
       </c>
       <c r="M9" s="12">
-        <f>IF(AND(A9="",F9=""),"",IF(F9="","Belum ditempatkan",IF(I9="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G9="","CEK ZONA NO kosong",IF(K9="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H9&lt;&gt;K9,"CEK JENIS ZONA",IF(A9="","Zona kosong",IF(B9="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A9="",F9=""),"",IF(F9="","Belum ditempatkan",IF(I9="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G9="","CEK ZONA NO kosong",IF(K9="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H9&lt;&gt;K9,"CEK JENIS ZONA",IF(A9="","Zona STOCK",IF(B9="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
         <v/>
       </c>
       <c r="M10" s="12">
-        <f>IF(AND(A10="",F10=""),"",IF(F10="","Belum ditempatkan",IF(I10="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G10="","CEK ZONA NO kosong",IF(K10="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H10&lt;&gt;K10,"CEK JENIS ZONA",IF(A10="","Zona kosong",IF(B10="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A10="",F10=""),"",IF(F10="","Belum ditempatkan",IF(I10="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G10="","CEK ZONA NO kosong",IF(K10="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H10&lt;&gt;K10,"CEK JENIS ZONA",IF(A10="","Zona STOCK",IF(B10="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="M11" s="12">
-        <f>IF(AND(A11="",F11=""),"",IF(F11="","Belum ditempatkan",IF(I11="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G11="","CEK ZONA NO kosong",IF(K11="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H11&lt;&gt;K11,"CEK JENIS ZONA",IF(A11="","Zona kosong",IF(B11="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A11="",F11=""),"",IF(F11="","Belum ditempatkan",IF(I11="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G11="","CEK ZONA NO kosong",IF(K11="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H11&lt;&gt;K11,"CEK JENIS ZONA",IF(A11="","Zona STOCK",IF(B11="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="M12" s="12">
-        <f>IF(AND(A12="",F12=""),"",IF(F12="","Belum ditempatkan",IF(I12="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G12="","CEK ZONA NO kosong",IF(K12="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H12&lt;&gt;K12,"CEK JENIS ZONA",IF(A12="","Zona kosong",IF(B12="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A12="",F12=""),"",IF(F12="","Belum ditempatkan",IF(I12="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G12="","CEK ZONA NO kosong",IF(K12="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H12&lt;&gt;K12,"CEK JENIS ZONA",IF(A12="","Zona STOCK",IF(B12="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
         <v/>
       </c>
       <c r="M13" s="12">
-        <f>IF(AND(A13="",F13=""),"",IF(F13="","Belum ditempatkan",IF(I13="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G13="","CEK ZONA NO kosong",IF(K13="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H13&lt;&gt;K13,"CEK JENIS ZONA",IF(A13="","Zona kosong",IF(B13="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A13="",F13=""),"",IF(F13="","Belum ditempatkan",IF(I13="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G13="","CEK ZONA NO kosong",IF(K13="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H13&lt;&gt;K13,"CEK JENIS ZONA",IF(A13="","Zona STOCK",IF(B13="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="M14" s="12">
-        <f>IF(AND(A14="",F14=""),"",IF(F14="","Belum ditempatkan",IF(I14="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G14="","CEK ZONA NO kosong",IF(K14="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H14&lt;&gt;K14,"CEK JENIS ZONA",IF(A14="","Zona kosong",IF(B14="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A14="",F14=""),"",IF(F14="","Belum ditempatkan",IF(I14="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G14="","CEK ZONA NO kosong",IF(K14="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H14&lt;&gt;K14,"CEK JENIS ZONA",IF(A14="","Zona STOCK",IF(B14="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
         <v/>
       </c>
       <c r="M15" s="12">
-        <f>IF(AND(A15="",F15=""),"",IF(F15="","Belum ditempatkan",IF(I15="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G15="","CEK ZONA NO kosong",IF(K15="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H15&lt;&gt;K15,"CEK JENIS ZONA",IF(A15="","Zona kosong",IF(B15="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A15="",F15=""),"",IF(F15="","Belum ditempatkan",IF(I15="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G15="","CEK ZONA NO kosong",IF(K15="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H15&lt;&gt;K15,"CEK JENIS ZONA",IF(A15="","Zona STOCK",IF(B15="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
         <v/>
       </c>
       <c r="M16" s="12">
-        <f>IF(AND(A16="",F16=""),"",IF(F16="","Belum ditempatkan",IF(I16="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G16="","CEK ZONA NO kosong",IF(K16="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H16&lt;&gt;K16,"CEK JENIS ZONA",IF(A16="","Zona kosong",IF(B16="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A16="",F16=""),"",IF(F16="","Belum ditempatkan",IF(I16="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G16="","CEK ZONA NO kosong",IF(K16="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H16&lt;&gt;K16,"CEK JENIS ZONA",IF(A16="","Zona STOCK",IF(B16="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
         <v/>
       </c>
       <c r="M17" s="12">
-        <f>IF(AND(A17="",F17=""),"",IF(F17="","Belum ditempatkan",IF(I17="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G17="","CEK ZONA NO kosong",IF(K17="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H17&lt;&gt;K17,"CEK JENIS ZONA",IF(A17="","Zona kosong",IF(B17="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A17="",F17=""),"",IF(F17="","Belum ditempatkan",IF(I17="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G17="","CEK ZONA NO kosong",IF(K17="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H17&lt;&gt;K17,"CEK JENIS ZONA",IF(A17="","Zona STOCK",IF(B17="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
         <v/>
       </c>
       <c r="M18" s="12">
-        <f>IF(AND(A18="",F18=""),"",IF(F18="","Belum ditempatkan",IF(I18="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G18="","CEK ZONA NO kosong",IF(K18="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H18&lt;&gt;K18,"CEK JENIS ZONA",IF(A18="","Zona kosong",IF(B18="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A18="",F18=""),"",IF(F18="","Belum ditempatkan",IF(I18="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G18="","CEK ZONA NO kosong",IF(K18="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H18&lt;&gt;K18,"CEK JENIS ZONA",IF(A18="","Zona STOCK",IF(B18="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
         <v/>
       </c>
       <c r="M19" s="12">
-        <f>IF(AND(A19="",F19=""),"",IF(F19="","Belum ditempatkan",IF(I19="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G19="","CEK ZONA NO kosong",IF(K19="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H19&lt;&gt;K19,"CEK JENIS ZONA",IF(A19="","Zona kosong",IF(B19="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A19="",F19=""),"",IF(F19="","Belum ditempatkan",IF(I19="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G19="","CEK ZONA NO kosong",IF(K19="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H19&lt;&gt;K19,"CEK JENIS ZONA",IF(A19="","Zona STOCK",IF(B19="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1819,7 +1819,7 @@
         <v/>
       </c>
       <c r="M20" s="12">
-        <f>IF(AND(A20="",F20=""),"",IF(F20="","Belum ditempatkan",IF(I20="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G20="","CEK ZONA NO kosong",IF(K20="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H20&lt;&gt;K20,"CEK JENIS ZONA",IF(A20="","Zona kosong",IF(B20="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A20="",F20=""),"",IF(F20="","Belum ditempatkan",IF(I20="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G20="","CEK ZONA NO kosong",IF(K20="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H20&lt;&gt;K20,"CEK JENIS ZONA",IF(A20="","Zona STOCK",IF(B20="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
         <v/>
       </c>
       <c r="M21" s="12">
-        <f>IF(AND(A21="",F21=""),"",IF(F21="","Belum ditempatkan",IF(I21="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G21="","CEK ZONA NO kosong",IF(K21="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H21&lt;&gt;K21,"CEK JENIS ZONA",IF(A21="","Zona kosong",IF(B21="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A21="",F21=""),"",IF(F21="","Belum ditempatkan",IF(I21="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G21="","CEK ZONA NO kosong",IF(K21="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H21&lt;&gt;K21,"CEK JENIS ZONA",IF(A21="","Zona STOCK",IF(B21="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
         <v/>
       </c>
       <c r="M22" s="12">
-        <f>IF(AND(A22="",F22=""),"",IF(F22="","Belum ditempatkan",IF(I22="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G22="","CEK ZONA NO kosong",IF(K22="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H22&lt;&gt;K22,"CEK JENIS ZONA",IF(A22="","Zona kosong",IF(B22="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A22="",F22=""),"",IF(F22="","Belum ditempatkan",IF(I22="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G22="","CEK ZONA NO kosong",IF(K22="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H22&lt;&gt;K22,"CEK JENIS ZONA",IF(A22="","Zona STOCK",IF(B22="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         <v/>
       </c>
       <c r="M23" s="12">
-        <f>IF(AND(A23="",F23=""),"",IF(F23="","Belum ditempatkan",IF(I23="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G23="","CEK ZONA NO kosong",IF(K23="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H23&lt;&gt;K23,"CEK JENIS ZONA",IF(A23="","Zona kosong",IF(B23="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A23="",F23=""),"",IF(F23="","Belum ditempatkan",IF(I23="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G23="","CEK ZONA NO kosong",IF(K23="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H23&lt;&gt;K23,"CEK JENIS ZONA",IF(A23="","Zona STOCK",IF(B23="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         <v/>
       </c>
       <c r="M24" s="12">
-        <f>IF(AND(A24="",F24=""),"",IF(F24="","Belum ditempatkan",IF(I24="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G24="","CEK ZONA NO kosong",IF(K24="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H24&lt;&gt;K24,"CEK JENIS ZONA",IF(A24="","Zona kosong",IF(B24="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A24="",F24=""),"",IF(F24="","Belum ditempatkan",IF(I24="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G24="","CEK ZONA NO kosong",IF(K24="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H24&lt;&gt;K24,"CEK JENIS ZONA",IF(A24="","Zona STOCK",IF(B24="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="M25" s="12">
-        <f>IF(AND(A25="",F25=""),"",IF(F25="","Belum ditempatkan",IF(I25="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G25="","CEK ZONA NO kosong",IF(K25="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H25&lt;&gt;K25,"CEK JENIS ZONA",IF(A25="","Zona kosong",IF(B25="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A25="",F25=""),"",IF(F25="","Belum ditempatkan",IF(I25="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G25="","CEK ZONA NO kosong",IF(K25="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H25&lt;&gt;K25,"CEK JENIS ZONA",IF(A25="","Zona STOCK",IF(B25="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
         <v/>
       </c>
       <c r="M26" s="12">
-        <f>IF(AND(A26="",F26=""),"",IF(F26="","Belum ditempatkan",IF(I26="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G26="","CEK ZONA NO kosong",IF(K26="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H26&lt;&gt;K26,"CEK JENIS ZONA",IF(A26="","Zona kosong",IF(B26="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A26="",F26=""),"",IF(F26="","Belum ditempatkan",IF(I26="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G26="","CEK ZONA NO kosong",IF(K26="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H26&lt;&gt;K26,"CEK JENIS ZONA",IF(A26="","Zona STOCK",IF(B26="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
         <v/>
       </c>
       <c r="M27" s="12">
-        <f>IF(AND(A27="",F27=""),"",IF(F27="","Belum ditempatkan",IF(I27="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G27="","CEK ZONA NO kosong",IF(K27="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H27&lt;&gt;K27,"CEK JENIS ZONA",IF(A27="","Zona kosong",IF(B27="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A27="",F27=""),"",IF(F27="","Belum ditempatkan",IF(I27="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G27="","CEK ZONA NO kosong",IF(K27="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H27&lt;&gt;K27,"CEK JENIS ZONA",IF(A27="","Zona STOCK",IF(B27="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
         <v/>
       </c>
       <c r="M28" s="12">
-        <f>IF(AND(A28="",F28=""),"",IF(F28="","Belum ditempatkan",IF(I28="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G28="","CEK ZONA NO kosong",IF(K28="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H28&lt;&gt;K28,"CEK JENIS ZONA",IF(A28="","Zona kosong",IF(B28="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A28="",F28=""),"",IF(F28="","Belum ditempatkan",IF(I28="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G28="","CEK ZONA NO kosong",IF(K28="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H28&lt;&gt;K28,"CEK JENIS ZONA",IF(A28="","Zona STOCK",IF(B28="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
         <v/>
       </c>
       <c r="M29" s="12">
-        <f>IF(AND(A29="",F29=""),"",IF(F29="","Belum ditempatkan",IF(I29="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G29="","CEK ZONA NO kosong",IF(K29="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H29&lt;&gt;K29,"CEK JENIS ZONA",IF(A29="","Zona kosong",IF(B29="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A29="",F29=""),"",IF(F29="","Belum ditempatkan",IF(I29="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G29="","CEK ZONA NO kosong",IF(K29="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H29&lt;&gt;K29,"CEK JENIS ZONA",IF(A29="","Zona STOCK",IF(B29="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
         <v/>
       </c>
       <c r="M30" s="12">
-        <f>IF(AND(A30="",F30=""),"",IF(F30="","Belum ditempatkan",IF(I30="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G30="","CEK ZONA NO kosong",IF(K30="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H30&lt;&gt;K30,"CEK JENIS ZONA",IF(A30="","Zona kosong",IF(B30="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A30="",F30=""),"",IF(F30="","Belum ditempatkan",IF(I30="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G30="","CEK ZONA NO kosong",IF(K30="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H30&lt;&gt;K30,"CEK JENIS ZONA",IF(A30="","Zona STOCK",IF(B30="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
         <v/>
       </c>
       <c r="M31" s="12">
-        <f>IF(AND(A31="",F31=""),"",IF(F31="","Belum ditempatkan",IF(I31="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G31="","CEK ZONA NO kosong",IF(K31="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H31&lt;&gt;K31,"CEK JENIS ZONA",IF(A31="","Zona kosong",IF(B31="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A31="",F31=""),"",IF(F31="","Belum ditempatkan",IF(I31="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G31="","CEK ZONA NO kosong",IF(K31="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H31&lt;&gt;K31,"CEK JENIS ZONA",IF(A31="","Zona STOCK",IF(B31="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
         <v/>
       </c>
       <c r="M32" s="12">
-        <f>IF(AND(A32="",F32=""),"",IF(F32="","Belum ditempatkan",IF(I32="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G32="","CEK ZONA NO kosong",IF(K32="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H32&lt;&gt;K32,"CEK JENIS ZONA",IF(A32="","Zona kosong",IF(B32="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A32="",F32=""),"",IF(F32="","Belum ditempatkan",IF(I32="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G32="","CEK ZONA NO kosong",IF(K32="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H32&lt;&gt;K32,"CEK JENIS ZONA",IF(A32="","Zona STOCK",IF(B32="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
         <v/>
       </c>
       <c r="M33" s="12">
-        <f>IF(AND(A33="",F33=""),"",IF(F33="","Belum ditempatkan",IF(I33="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G33="","CEK ZONA NO kosong",IF(K33="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H33&lt;&gt;K33,"CEK JENIS ZONA",IF(A33="","Zona kosong",IF(B33="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A33="",F33=""),"",IF(F33="","Belum ditempatkan",IF(I33="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G33="","CEK ZONA NO kosong",IF(K33="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H33&lt;&gt;K33,"CEK JENIS ZONA",IF(A33="","Zona STOCK",IF(B33="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
         <v/>
       </c>
       <c r="M34" s="12">
-        <f>IF(AND(A34="",F34=""),"",IF(F34="","Belum ditempatkan",IF(I34="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G34="","CEK ZONA NO kosong",IF(K34="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H34&lt;&gt;K34,"CEK JENIS ZONA",IF(A34="","Zona kosong",IF(B34="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A34="",F34=""),"",IF(F34="","Belum ditempatkan",IF(I34="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G34="","CEK ZONA NO kosong",IF(K34="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H34&lt;&gt;K34,"CEK JENIS ZONA",IF(A34="","Zona STOCK",IF(B34="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2515,7 +2515,7 @@
         <v/>
       </c>
       <c r="M35" s="12">
-        <f>IF(AND(A35="",F35=""),"",IF(F35="","Belum ditempatkan",IF(I35="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G35="","CEK ZONA NO kosong",IF(K35="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H35&lt;&gt;K35,"CEK JENIS ZONA",IF(A35="","Zona kosong",IF(B35="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A35="",F35=""),"",IF(F35="","Belum ditempatkan",IF(I35="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G35="","CEK ZONA NO kosong",IF(K35="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H35&lt;&gt;K35,"CEK JENIS ZONA",IF(A35="","Zona STOCK",IF(B35="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
         <v/>
       </c>
       <c r="M36" s="12">
-        <f>IF(AND(A36="",F36=""),"",IF(F36="","Belum ditempatkan",IF(I36="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G36="","CEK ZONA NO kosong",IF(K36="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H36&lt;&gt;K36,"CEK JENIS ZONA",IF(A36="","Zona kosong",IF(B36="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A36="",F36=""),"",IF(F36="","Belum ditempatkan",IF(I36="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G36="","CEK ZONA NO kosong",IF(K36="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H36&lt;&gt;K36,"CEK JENIS ZONA",IF(A36="","Zona STOCK",IF(B36="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
         <v/>
       </c>
       <c r="M37" s="12">
-        <f>IF(AND(A37="",F37=""),"",IF(F37="","Belum ditempatkan",IF(I37="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G37="","CEK ZONA NO kosong",IF(K37="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H37&lt;&gt;K37,"CEK JENIS ZONA",IF(A37="","Zona kosong",IF(B37="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A37="",F37=""),"",IF(F37="","Belum ditempatkan",IF(I37="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G37="","CEK ZONA NO kosong",IF(K37="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H37&lt;&gt;K37,"CEK JENIS ZONA",IF(A37="","Zona STOCK",IF(B37="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
         <v/>
       </c>
       <c r="M38" s="12">
-        <f>IF(AND(A38="",F38=""),"",IF(F38="","Belum ditempatkan",IF(I38="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G38="","CEK ZONA NO kosong",IF(K38="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H38&lt;&gt;K38,"CEK JENIS ZONA",IF(A38="","Zona kosong",IF(B38="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A38="",F38=""),"",IF(F38="","Belum ditempatkan",IF(I38="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G38="","CEK ZONA NO kosong",IF(K38="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H38&lt;&gt;K38,"CEK JENIS ZONA",IF(A38="","Zona STOCK",IF(B38="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
         <v/>
       </c>
       <c r="M39" s="12">
-        <f>IF(AND(A39="",F39=""),"",IF(F39="","Belum ditempatkan",IF(I39="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G39="","CEK ZONA NO kosong",IF(K39="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H39&lt;&gt;K39,"CEK JENIS ZONA",IF(A39="","Zona kosong",IF(B39="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A39="",F39=""),"",IF(F39="","Belum ditempatkan",IF(I39="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G39="","CEK ZONA NO kosong",IF(K39="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H39&lt;&gt;K39,"CEK JENIS ZONA",IF(A39="","Zona STOCK",IF(B39="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2747,7 +2747,7 @@
         <v/>
       </c>
       <c r="M40" s="12">
-        <f>IF(AND(A40="",F40=""),"",IF(F40="","Belum ditempatkan",IF(I40="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G40="","CEK ZONA NO kosong",IF(K40="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H40&lt;&gt;K40,"CEK JENIS ZONA",IF(A40="","Zona kosong",IF(B40="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A40="",F40=""),"",IF(F40="","Belum ditempatkan",IF(I40="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G40="","CEK ZONA NO kosong",IF(K40="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H40&lt;&gt;K40,"CEK JENIS ZONA",IF(A40="","Zona STOCK",IF(B40="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2795,7 +2795,7 @@
         <v/>
       </c>
       <c r="M41" s="12">
-        <f>IF(AND(A41="",F41=""),"",IF(F41="","Belum ditempatkan",IF(I41="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G41="","CEK ZONA NO kosong",IF(K41="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H41&lt;&gt;K41,"CEK JENIS ZONA",IF(A41="","Zona kosong",IF(B41="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A41="",F41=""),"",IF(F41="","Belum ditempatkan",IF(I41="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G41="","CEK ZONA NO kosong",IF(K41="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H41&lt;&gt;K41,"CEK JENIS ZONA",IF(A41="","Zona STOCK",IF(B41="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
         <v/>
       </c>
       <c r="M42" s="12">
-        <f>IF(AND(A42="",F42=""),"",IF(F42="","Belum ditempatkan",IF(I42="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G42="","CEK ZONA NO kosong",IF(K42="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H42&lt;&gt;K42,"CEK JENIS ZONA",IF(A42="","Zona kosong",IF(B42="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A42="",F42=""),"",IF(F42="","Belum ditempatkan",IF(I42="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G42="","CEK ZONA NO kosong",IF(K42="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H42&lt;&gt;K42,"CEK JENIS ZONA",IF(A42="","Zona STOCK",IF(B42="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="M43" s="12">
-        <f>IF(AND(A43="",F43=""),"",IF(F43="","Belum ditempatkan",IF(I43="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G43="","CEK ZONA NO kosong",IF(K43="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H43&lt;&gt;K43,"CEK JENIS ZONA",IF(A43="","Zona kosong",IF(B43="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A43="",F43=""),"",IF(F43="","Belum ditempatkan",IF(I43="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G43="","CEK ZONA NO kosong",IF(K43="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H43&lt;&gt;K43,"CEK JENIS ZONA",IF(A43="","Zona STOCK",IF(B43="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="M44" s="12">
-        <f>IF(AND(A44="",F44=""),"",IF(F44="","Belum ditempatkan",IF(I44="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G44="","CEK ZONA NO kosong",IF(K44="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H44&lt;&gt;K44,"CEK JENIS ZONA",IF(A44="","Zona kosong",IF(B44="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A44="",F44=""),"",IF(F44="","Belum ditempatkan",IF(I44="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G44="","CEK ZONA NO kosong",IF(K44="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H44&lt;&gt;K44,"CEK JENIS ZONA",IF(A44="","Zona STOCK",IF(B44="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
         <v/>
       </c>
       <c r="M45" s="12">
-        <f>IF(AND(A45="",F45=""),"",IF(F45="","Belum ditempatkan",IF(I45="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G45="","CEK ZONA NO kosong",IF(K45="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H45&lt;&gt;K45,"CEK JENIS ZONA",IF(A45="","Zona kosong",IF(B45="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A45="",F45=""),"",IF(F45="","Belum ditempatkan",IF(I45="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G45="","CEK ZONA NO kosong",IF(K45="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H45&lt;&gt;K45,"CEK JENIS ZONA",IF(A45="","Zona STOCK",IF(B45="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
         <v/>
       </c>
       <c r="M46" s="12">
-        <f>IF(AND(A46="",F46=""),"",IF(F46="","Belum ditempatkan",IF(I46="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G46="","CEK ZONA NO kosong",IF(K46="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H46&lt;&gt;K46,"CEK JENIS ZONA",IF(A46="","Zona kosong",IF(B46="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A46="",F46=""),"",IF(F46="","Belum ditempatkan",IF(I46="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G46="","CEK ZONA NO kosong",IF(K46="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H46&lt;&gt;K46,"CEK JENIS ZONA",IF(A46="","Zona STOCK",IF(B46="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
         <v/>
       </c>
       <c r="M47" s="12">
-        <f>IF(AND(A47="",F47=""),"",IF(F47="","Belum ditempatkan",IF(I47="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G47="","CEK ZONA NO kosong",IF(K47="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H47&lt;&gt;K47,"CEK JENIS ZONA",IF(A47="","Zona kosong",IF(B47="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A47="",F47=""),"",IF(F47="","Belum ditempatkan",IF(I47="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G47="","CEK ZONA NO kosong",IF(K47="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H47&lt;&gt;K47,"CEK JENIS ZONA",IF(A47="","Zona STOCK",IF(B47="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
         <v/>
       </c>
       <c r="M48" s="12">
-        <f>IF(AND(A48="",F48=""),"",IF(F48="","Belum ditempatkan",IF(I48="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G48="","CEK ZONA NO kosong",IF(K48="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H48&lt;&gt;K48,"CEK JENIS ZONA",IF(A48="","Zona kosong",IF(B48="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A48="",F48=""),"",IF(F48="","Belum ditempatkan",IF(I48="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G48="","CEK ZONA NO kosong",IF(K48="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H48&lt;&gt;K48,"CEK JENIS ZONA",IF(A48="","Zona STOCK",IF(B48="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
         <v/>
       </c>
       <c r="M49" s="12">
-        <f>IF(AND(A49="",F49=""),"",IF(F49="","Belum ditempatkan",IF(I49="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G49="","CEK ZONA NO kosong",IF(K49="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H49&lt;&gt;K49,"CEK JENIS ZONA",IF(A49="","Zona kosong",IF(B49="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A49="",F49=""),"",IF(F49="","Belum ditempatkan",IF(I49="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G49="","CEK ZONA NO kosong",IF(K49="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H49&lt;&gt;K49,"CEK JENIS ZONA",IF(A49="","Zona STOCK",IF(B49="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
         <v/>
       </c>
       <c r="M50" s="12">
-        <f>IF(AND(A50="",F50=""),"",IF(F50="","Belum ditempatkan",IF(I50="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G50="","CEK ZONA NO kosong",IF(K50="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H50&lt;&gt;K50,"CEK JENIS ZONA",IF(A50="","Zona kosong",IF(B50="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A50="",F50=""),"",IF(F50="","Belum ditempatkan",IF(I50="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G50="","CEK ZONA NO kosong",IF(K50="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H50&lt;&gt;K50,"CEK JENIS ZONA",IF(A50="","Zona STOCK",IF(B50="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
         <v/>
       </c>
       <c r="M51" s="12">
-        <f>IF(AND(A51="",F51=""),"",IF(F51="","Belum ditempatkan",IF(I51="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G51="","CEK ZONA NO kosong",IF(K51="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H51&lt;&gt;K51,"CEK JENIS ZONA",IF(A51="","Zona kosong",IF(B51="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A51="",F51=""),"",IF(F51="","Belum ditempatkan",IF(I51="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G51="","CEK ZONA NO kosong",IF(K51="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H51&lt;&gt;K51,"CEK JENIS ZONA",IF(A51="","Zona STOCK",IF(B51="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
         <v/>
       </c>
       <c r="M52" s="12">
-        <f>IF(AND(A52="",F52=""),"",IF(F52="","Belum ditempatkan",IF(I52="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G52="","CEK ZONA NO kosong",IF(K52="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H52&lt;&gt;K52,"CEK JENIS ZONA",IF(A52="","Zona kosong",IF(B52="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A52="",F52=""),"",IF(F52="","Belum ditempatkan",IF(I52="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G52="","CEK ZONA NO kosong",IF(K52="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H52&lt;&gt;K52,"CEK JENIS ZONA",IF(A52="","Zona STOCK",IF(B52="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
         <v/>
       </c>
       <c r="M53" s="12">
-        <f>IF(AND(A53="",F53=""),"",IF(F53="","Belum ditempatkan",IF(I53="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G53="","CEK ZONA NO kosong",IF(K53="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H53&lt;&gt;K53,"CEK JENIS ZONA",IF(A53="","Zona kosong",IF(B53="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A53="",F53=""),"",IF(F53="","Belum ditempatkan",IF(I53="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G53="","CEK ZONA NO kosong",IF(K53="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H53&lt;&gt;K53,"CEK JENIS ZONA",IF(A53="","Zona STOCK",IF(B53="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
         <v/>
       </c>
       <c r="M54" s="12">
-        <f>IF(AND(A54="",F54=""),"",IF(F54="","Belum ditempatkan",IF(I54="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G54="","CEK ZONA NO kosong",IF(K54="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H54&lt;&gt;K54,"CEK JENIS ZONA",IF(A54="","Zona kosong",IF(B54="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A54="",F54=""),"",IF(F54="","Belum ditempatkan",IF(I54="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G54="","CEK ZONA NO kosong",IF(K54="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H54&lt;&gt;K54,"CEK JENIS ZONA",IF(A54="","Zona STOCK",IF(B54="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
         <v/>
       </c>
       <c r="M55" s="12">
-        <f>IF(AND(A55="",F55=""),"",IF(F55="","Belum ditempatkan",IF(I55="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G55="","CEK ZONA NO kosong",IF(K55="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H55&lt;&gt;K55,"CEK JENIS ZONA",IF(A55="","Zona kosong",IF(B55="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A55="",F55=""),"",IF(F55="","Belum ditempatkan",IF(I55="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G55="","CEK ZONA NO kosong",IF(K55="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H55&lt;&gt;K55,"CEK JENIS ZONA",IF(A55="","Zona STOCK",IF(B55="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
         <v/>
       </c>
       <c r="M56" s="12">
-        <f>IF(AND(A56="",F56=""),"",IF(F56="","Belum ditempatkan",IF(I56="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G56="","CEK ZONA NO kosong",IF(K56="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H56&lt;&gt;K56,"CEK JENIS ZONA",IF(A56="","Zona kosong",IF(B56="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A56="",F56=""),"",IF(F56="","Belum ditempatkan",IF(I56="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G56="","CEK ZONA NO kosong",IF(K56="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H56&lt;&gt;K56,"CEK JENIS ZONA",IF(A56="","Zona STOCK",IF(B56="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3547,7 +3547,7 @@
         <v/>
       </c>
       <c r="M57" s="12">
-        <f>IF(AND(A57="",F57=""),"",IF(F57="","Belum ditempatkan",IF(I57="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G57="","CEK ZONA NO kosong",IF(K57="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H57&lt;&gt;K57,"CEK JENIS ZONA",IF(A57="","Zona kosong",IF(B57="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A57="",F57=""),"",IF(F57="","Belum ditempatkan",IF(I57="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G57="","CEK ZONA NO kosong",IF(K57="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H57&lt;&gt;K57,"CEK JENIS ZONA",IF(A57="","Zona STOCK",IF(B57="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
         <v/>
       </c>
       <c r="M58" s="12">
-        <f>IF(AND(A58="",F58=""),"",IF(F58="","Belum ditempatkan",IF(I58="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G58="","CEK ZONA NO kosong",IF(K58="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H58&lt;&gt;K58,"CEK JENIS ZONA",IF(A58="","Zona kosong",IF(B58="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A58="",F58=""),"",IF(F58="","Belum ditempatkan",IF(I58="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G58="","CEK ZONA NO kosong",IF(K58="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H58&lt;&gt;K58,"CEK JENIS ZONA",IF(A58="","Zona STOCK",IF(B58="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
         <v/>
       </c>
       <c r="M59" s="12">
-        <f>IF(AND(A59="",F59=""),"",IF(F59="","Belum ditempatkan",IF(I59="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G59="","CEK ZONA NO kosong",IF(K59="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H59&lt;&gt;K59,"CEK JENIS ZONA",IF(A59="","Zona kosong",IF(B59="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A59="",F59=""),"",IF(F59="","Belum ditempatkan",IF(I59="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G59="","CEK ZONA NO kosong",IF(K59="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H59&lt;&gt;K59,"CEK JENIS ZONA",IF(A59="","Zona STOCK",IF(B59="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
         <v/>
       </c>
       <c r="M60" s="12">
-        <f>IF(AND(A60="",F60=""),"",IF(F60="","Belum ditempatkan",IF(I60="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G60="","CEK ZONA NO kosong",IF(K60="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H60&lt;&gt;K60,"CEK JENIS ZONA",IF(A60="","Zona kosong",IF(B60="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A60="",F60=""),"",IF(F60="","Belum ditempatkan",IF(I60="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G60="","CEK ZONA NO kosong",IF(K60="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H60&lt;&gt;K60,"CEK JENIS ZONA",IF(A60="","Zona STOCK",IF(B60="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
         <v/>
       </c>
       <c r="M61" s="12">
-        <f>IF(AND(A61="",F61=""),"",IF(F61="","Belum ditempatkan",IF(I61="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G61="","CEK ZONA NO kosong",IF(K61="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H61&lt;&gt;K61,"CEK JENIS ZONA",IF(A61="","Zona kosong",IF(B61="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A61="",F61=""),"",IF(F61="","Belum ditempatkan",IF(I61="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G61="","CEK ZONA NO kosong",IF(K61="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H61&lt;&gt;K61,"CEK JENIS ZONA",IF(A61="","Zona STOCK",IF(B61="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
         <v/>
       </c>
       <c r="M62" s="12">
-        <f>IF(AND(A62="",F62=""),"",IF(F62="","Belum ditempatkan",IF(I62="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G62="","CEK ZONA NO kosong",IF(K62="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H62&lt;&gt;K62,"CEK JENIS ZONA",IF(A62="","Zona kosong",IF(B62="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A62="",F62=""),"",IF(F62="","Belum ditempatkan",IF(I62="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G62="","CEK ZONA NO kosong",IF(K62="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H62&lt;&gt;K62,"CEK JENIS ZONA",IF(A62="","Zona STOCK",IF(B62="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
         <v/>
       </c>
       <c r="M63" s="12">
-        <f>IF(AND(A63="",F63=""),"",IF(F63="","Belum ditempatkan",IF(I63="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G63="","CEK ZONA NO kosong",IF(K63="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H63&lt;&gt;K63,"CEK JENIS ZONA",IF(A63="","Zona kosong",IF(B63="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A63="",F63=""),"",IF(F63="","Belum ditempatkan",IF(I63="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G63="","CEK ZONA NO kosong",IF(K63="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H63&lt;&gt;K63,"CEK JENIS ZONA",IF(A63="","Zona STOCK",IF(B63="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
         <v/>
       </c>
       <c r="M64" s="12">
-        <f>IF(AND(A64="",F64=""),"",IF(F64="","Belum ditempatkan",IF(I64="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G64="","CEK ZONA NO kosong",IF(K64="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H64&lt;&gt;K64,"CEK JENIS ZONA",IF(A64="","Zona kosong",IF(B64="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A64="",F64=""),"",IF(F64="","Belum ditempatkan",IF(I64="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G64="","CEK ZONA NO kosong",IF(K64="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H64&lt;&gt;K64,"CEK JENIS ZONA",IF(A64="","Zona STOCK",IF(B64="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
         <v/>
       </c>
       <c r="M65" s="12">
-        <f>IF(AND(A65="",F65=""),"",IF(F65="","Belum ditempatkan",IF(I65="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G65="","CEK ZONA NO kosong",IF(K65="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H65&lt;&gt;K65,"CEK JENIS ZONA",IF(A65="","Zona kosong",IF(B65="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A65="",F65=""),"",IF(F65="","Belum ditempatkan",IF(I65="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G65="","CEK ZONA NO kosong",IF(K65="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H65&lt;&gt;K65,"CEK JENIS ZONA",IF(A65="","Zona STOCK",IF(B65="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
         <v/>
       </c>
       <c r="M66" s="12">
-        <f>IF(AND(A66="",F66=""),"",IF(F66="","Belum ditempatkan",IF(I66="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G66="","CEK ZONA NO kosong",IF(K66="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H66&lt;&gt;K66,"CEK JENIS ZONA",IF(A66="","Zona kosong",IF(B66="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A66="",F66=""),"",IF(F66="","Belum ditempatkan",IF(I66="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G66="","CEK ZONA NO kosong",IF(K66="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H66&lt;&gt;K66,"CEK JENIS ZONA",IF(A66="","Zona STOCK",IF(B66="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
         <v/>
       </c>
       <c r="M67" s="12">
-        <f>IF(AND(A67="",F67=""),"",IF(F67="","Belum ditempatkan",IF(I67="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G67="","CEK ZONA NO kosong",IF(K67="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H67&lt;&gt;K67,"CEK JENIS ZONA",IF(A67="","Zona kosong",IF(B67="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A67="",F67=""),"",IF(F67="","Belum ditempatkan",IF(I67="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G67="","CEK ZONA NO kosong",IF(K67="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H67&lt;&gt;K67,"CEK JENIS ZONA",IF(A67="","Zona STOCK",IF(B67="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
         <v/>
       </c>
       <c r="M68" s="12">
-        <f>IF(AND(A68="",F68=""),"",IF(F68="","Belum ditempatkan",IF(I68="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G68="","CEK ZONA NO kosong",IF(K68="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H68&lt;&gt;K68,"CEK JENIS ZONA",IF(A68="","Zona kosong",IF(B68="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A68="",F68=""),"",IF(F68="","Belum ditempatkan",IF(I68="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G68="","CEK ZONA NO kosong",IF(K68="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H68&lt;&gt;K68,"CEK JENIS ZONA",IF(A68="","Zona STOCK",IF(B68="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
         <v/>
       </c>
       <c r="M69" s="12">
-        <f>IF(AND(A69="",F69=""),"",IF(F69="","Belum ditempatkan",IF(I69="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G69="","CEK ZONA NO kosong",IF(K69="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H69&lt;&gt;K69,"CEK JENIS ZONA",IF(A69="","Zona kosong",IF(B69="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A69="",F69=""),"",IF(F69="","Belum ditempatkan",IF(I69="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G69="","CEK ZONA NO kosong",IF(K69="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H69&lt;&gt;K69,"CEK JENIS ZONA",IF(A69="","Zona STOCK",IF(B69="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
         <v/>
       </c>
       <c r="M70" s="12">
-        <f>IF(AND(A70="",F70=""),"",IF(F70="","Belum ditempatkan",IF(I70="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G70="","CEK ZONA NO kosong",IF(K70="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H70&lt;&gt;K70,"CEK JENIS ZONA",IF(A70="","Zona kosong",IF(B70="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A70="",F70=""),"",IF(F70="","Belum ditempatkan",IF(I70="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G70="","CEK ZONA NO kosong",IF(K70="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H70&lt;&gt;K70,"CEK JENIS ZONA",IF(A70="","Zona STOCK",IF(B70="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
         <v/>
       </c>
       <c r="M71" s="12">
-        <f>IF(AND(A71="",F71=""),"",IF(F71="","Belum ditempatkan",IF(I71="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G71="","CEK ZONA NO kosong",IF(K71="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H71&lt;&gt;K71,"CEK JENIS ZONA",IF(A71="","Zona kosong",IF(B71="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A71="",F71=""),"",IF(F71="","Belum ditempatkan",IF(I71="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G71="","CEK ZONA NO kosong",IF(K71="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H71&lt;&gt;K71,"CEK JENIS ZONA",IF(A71="","Zona STOCK",IF(B71="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
         <v/>
       </c>
       <c r="M72" s="12">
-        <f>IF(AND(A72="",F72=""),"",IF(F72="","Belum ditempatkan",IF(I72="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G72="","CEK ZONA NO kosong",IF(K72="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H72&lt;&gt;K72,"CEK JENIS ZONA",IF(A72="","Zona kosong",IF(B72="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A72="",F72=""),"",IF(F72="","Belum ditempatkan",IF(I72="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G72="","CEK ZONA NO kosong",IF(K72="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H72&lt;&gt;K72,"CEK JENIS ZONA",IF(A72="","Zona STOCK",IF(B72="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
         <v/>
       </c>
       <c r="M73" s="12">
-        <f>IF(AND(A73="",F73=""),"",IF(F73="","Belum ditempatkan",IF(I73="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G73="","CEK ZONA NO kosong",IF(K73="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H73&lt;&gt;K73,"CEK JENIS ZONA",IF(A73="","Zona kosong",IF(B73="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A73="",F73=""),"",IF(F73="","Belum ditempatkan",IF(I73="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G73="","CEK ZONA NO kosong",IF(K73="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H73&lt;&gt;K73,"CEK JENIS ZONA",IF(A73="","Zona STOCK",IF(B73="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
         <v/>
       </c>
       <c r="M74" s="12">
-        <f>IF(AND(A74="",F74=""),"",IF(F74="","Belum ditempatkan",IF(I74="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G74="","CEK ZONA NO kosong",IF(K74="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H74&lt;&gt;K74,"CEK JENIS ZONA",IF(A74="","Zona kosong",IF(B74="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A74="",F74=""),"",IF(F74="","Belum ditempatkan",IF(I74="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G74="","CEK ZONA NO kosong",IF(K74="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H74&lt;&gt;K74,"CEK JENIS ZONA",IF(A74="","Zona STOCK",IF(B74="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
         <v/>
       </c>
       <c r="M75" s="12">
-        <f>IF(AND(A75="",F75=""),"",IF(F75="","Belum ditempatkan",IF(I75="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G75="","CEK ZONA NO kosong",IF(K75="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H75&lt;&gt;K75,"CEK JENIS ZONA",IF(A75="","Zona kosong",IF(B75="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A75="",F75=""),"",IF(F75="","Belum ditempatkan",IF(I75="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G75="","CEK ZONA NO kosong",IF(K75="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H75&lt;&gt;K75,"CEK JENIS ZONA",IF(A75="","Zona STOCK",IF(B75="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4459,7 +4459,7 @@
         <v/>
       </c>
       <c r="M76" s="12">
-        <f>IF(AND(A76="",F76=""),"",IF(F76="","Belum ditempatkan",IF(I76="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G76="","CEK ZONA NO kosong",IF(K76="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H76&lt;&gt;K76,"CEK JENIS ZONA",IF(A76="","Zona kosong",IF(B76="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A76="",F76=""),"",IF(F76="","Belum ditempatkan",IF(I76="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G76="","CEK ZONA NO kosong",IF(K76="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H76&lt;&gt;K76,"CEK JENIS ZONA",IF(A76="","Zona STOCK",IF(B76="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4507,7 +4507,7 @@
         <v/>
       </c>
       <c r="M77" s="12">
-        <f>IF(AND(A77="",F77=""),"",IF(F77="","Belum ditempatkan",IF(I77="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G77="","CEK ZONA NO kosong",IF(K77="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H77&lt;&gt;K77,"CEK JENIS ZONA",IF(A77="","Zona kosong",IF(B77="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A77="",F77=""),"",IF(F77="","Belum ditempatkan",IF(I77="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G77="","CEK ZONA NO kosong",IF(K77="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H77&lt;&gt;K77,"CEK JENIS ZONA",IF(A77="","Zona STOCK",IF(B77="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
         <v/>
       </c>
       <c r="M78" s="12">
-        <f>IF(AND(A78="",F78=""),"",IF(F78="","Belum ditempatkan",IF(I78="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G78="","CEK ZONA NO kosong",IF(K78="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H78&lt;&gt;K78,"CEK JENIS ZONA",IF(A78="","Zona kosong",IF(B78="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A78="",F78=""),"",IF(F78="","Belum ditempatkan",IF(I78="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G78="","CEK ZONA NO kosong",IF(K78="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H78&lt;&gt;K78,"CEK JENIS ZONA",IF(A78="","Zona STOCK",IF(B78="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
         <v/>
       </c>
       <c r="M79" s="12">
-        <f>IF(AND(A79="",F79=""),"",IF(F79="","Belum ditempatkan",IF(I79="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G79="","CEK ZONA NO kosong",IF(K79="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H79&lt;&gt;K79,"CEK JENIS ZONA",IF(A79="","Zona kosong",IF(B79="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A79="",F79=""),"",IF(F79="","Belum ditempatkan",IF(I79="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G79="","CEK ZONA NO kosong",IF(K79="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H79&lt;&gt;K79,"CEK JENIS ZONA",IF(A79="","Zona STOCK",IF(B79="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
         <v/>
       </c>
       <c r="M80" s="12">
-        <f>IF(AND(A80="",F80=""),"",IF(F80="","Belum ditempatkan",IF(I80="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G80="","CEK ZONA NO kosong",IF(K80="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H80&lt;&gt;K80,"CEK JENIS ZONA",IF(A80="","Zona kosong",IF(B80="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A80="",F80=""),"",IF(F80="","Belum ditempatkan",IF(I80="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G80="","CEK ZONA NO kosong",IF(K80="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H80&lt;&gt;K80,"CEK JENIS ZONA",IF(A80="","Zona STOCK",IF(B80="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
         <v/>
       </c>
       <c r="M81" s="12">
-        <f>IF(AND(A81="",F81=""),"",IF(F81="","Belum ditempatkan",IF(I81="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G81="","CEK ZONA NO kosong",IF(K81="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H81&lt;&gt;K81,"CEK JENIS ZONA",IF(A81="","Zona kosong",IF(B81="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A81="",F81=""),"",IF(F81="","Belum ditempatkan",IF(I81="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G81="","CEK ZONA NO kosong",IF(K81="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H81&lt;&gt;K81,"CEK JENIS ZONA",IF(A81="","Zona STOCK",IF(B81="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4747,7 +4747,7 @@
         <v/>
       </c>
       <c r="M82" s="12">
-        <f>IF(AND(A82="",F82=""),"",IF(F82="","Belum ditempatkan",IF(I82="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G82="","CEK ZONA NO kosong",IF(K82="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H82&lt;&gt;K82,"CEK JENIS ZONA",IF(A82="","Zona kosong",IF(B82="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A82="",F82=""),"",IF(F82="","Belum ditempatkan",IF(I82="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G82="","CEK ZONA NO kosong",IF(K82="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H82&lt;&gt;K82,"CEK JENIS ZONA",IF(A82="","Zona STOCK",IF(B82="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="M83" s="12">
-        <f>IF(AND(A83="",F83=""),"",IF(F83="","Belum ditempatkan",IF(I83="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G83="","CEK ZONA NO kosong",IF(K83="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H83&lt;&gt;K83,"CEK JENIS ZONA",IF(A83="","Zona kosong",IF(B83="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A83="",F83=""),"",IF(F83="","Belum ditempatkan",IF(I83="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G83="","CEK ZONA NO kosong",IF(K83="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H83&lt;&gt;K83,"CEK JENIS ZONA",IF(A83="","Zona STOCK",IF(B83="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
         <v/>
       </c>
       <c r="M84" s="12">
-        <f>IF(AND(A84="",F84=""),"",IF(F84="","Belum ditempatkan",IF(I84="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G84="","CEK ZONA NO kosong",IF(K84="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H84&lt;&gt;K84,"CEK JENIS ZONA",IF(A84="","Zona kosong",IF(B84="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A84="",F84=""),"",IF(F84="","Belum ditempatkan",IF(I84="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G84="","CEK ZONA NO kosong",IF(K84="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H84&lt;&gt;K84,"CEK JENIS ZONA",IF(A84="","Zona STOCK",IF(B84="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
         <v/>
       </c>
       <c r="M85" s="12">
-        <f>IF(AND(A85="",F85=""),"",IF(F85="","Belum ditempatkan",IF(I85="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G85="","CEK ZONA NO kosong",IF(K85="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H85&lt;&gt;K85,"CEK JENIS ZONA",IF(A85="","Zona kosong",IF(B85="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A85="",F85=""),"",IF(F85="","Belum ditempatkan",IF(I85="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G85="","CEK ZONA NO kosong",IF(K85="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H85&lt;&gt;K85,"CEK JENIS ZONA",IF(A85="","Zona STOCK",IF(B85="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4939,7 +4939,7 @@
         <v/>
       </c>
       <c r="M86" s="12">
-        <f>IF(AND(A86="",F86=""),"",IF(F86="","Belum ditempatkan",IF(I86="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G86="","CEK ZONA NO kosong",IF(K86="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H86&lt;&gt;K86,"CEK JENIS ZONA",IF(A86="","Zona kosong",IF(B86="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A86="",F86=""),"",IF(F86="","Belum ditempatkan",IF(I86="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G86="","CEK ZONA NO kosong",IF(K86="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H86&lt;&gt;K86,"CEK JENIS ZONA",IF(A86="","Zona STOCK",IF(B86="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -4987,7 +4987,7 @@
         <v/>
       </c>
       <c r="M87" s="12">
-        <f>IF(AND(A87="",F87=""),"",IF(F87="","Belum ditempatkan",IF(I87="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G87="","CEK ZONA NO kosong",IF(K87="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H87&lt;&gt;K87,"CEK JENIS ZONA",IF(A87="","Zona kosong",IF(B87="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A87="",F87=""),"",IF(F87="","Belum ditempatkan",IF(I87="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G87="","CEK ZONA NO kosong",IF(K87="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H87&lt;&gt;K87,"CEK JENIS ZONA",IF(A87="","Zona STOCK",IF(B87="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
         <v/>
       </c>
       <c r="M88" s="12">
-        <f>IF(AND(A88="",F88=""),"",IF(F88="","Belum ditempatkan",IF(I88="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G88="","CEK ZONA NO kosong",IF(K88="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H88&lt;&gt;K88,"CEK JENIS ZONA",IF(A88="","Zona kosong",IF(B88="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A88="",F88=""),"",IF(F88="","Belum ditempatkan",IF(I88="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G88="","CEK ZONA NO kosong",IF(K88="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H88&lt;&gt;K88,"CEK JENIS ZONA",IF(A88="","Zona STOCK",IF(B88="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5083,7 +5083,7 @@
         <v/>
       </c>
       <c r="M89" s="12">
-        <f>IF(AND(A89="",F89=""),"",IF(F89="","Belum ditempatkan",IF(I89="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G89="","CEK ZONA NO kosong",IF(K89="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H89&lt;&gt;K89,"CEK JENIS ZONA",IF(A89="","Zona kosong",IF(B89="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A89="",F89=""),"",IF(F89="","Belum ditempatkan",IF(I89="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G89="","CEK ZONA NO kosong",IF(K89="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H89&lt;&gt;K89,"CEK JENIS ZONA",IF(A89="","Zona STOCK",IF(B89="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
         <v/>
       </c>
       <c r="M90" s="12">
-        <f>IF(AND(A90="",F90=""),"",IF(F90="","Belum ditempatkan",IF(I90="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G90="","CEK ZONA NO kosong",IF(K90="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H90&lt;&gt;K90,"CEK JENIS ZONA",IF(A90="","Zona kosong",IF(B90="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A90="",F90=""),"",IF(F90="","Belum ditempatkan",IF(I90="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G90="","CEK ZONA NO kosong",IF(K90="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H90&lt;&gt;K90,"CEK JENIS ZONA",IF(A90="","Zona STOCK",IF(B90="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
         <v/>
       </c>
       <c r="M91" s="12">
-        <f>IF(AND(A91="",F91=""),"",IF(F91="","Belum ditempatkan",IF(I91="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G91="","CEK ZONA NO kosong",IF(K91="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H91&lt;&gt;K91,"CEK JENIS ZONA",IF(A91="","Zona kosong",IF(B91="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A91="",F91=""),"",IF(F91="","Belum ditempatkan",IF(I91="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G91="","CEK ZONA NO kosong",IF(K91="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H91&lt;&gt;K91,"CEK JENIS ZONA",IF(A91="","Zona STOCK",IF(B91="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
         <v/>
       </c>
       <c r="M92" s="12">
-        <f>IF(AND(A92="",F92=""),"",IF(F92="","Belum ditempatkan",IF(I92="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G92="","CEK ZONA NO kosong",IF(K92="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H92&lt;&gt;K92,"CEK JENIS ZONA",IF(A92="","Zona kosong",IF(B92="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A92="",F92=""),"",IF(F92="","Belum ditempatkan",IF(I92="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G92="","CEK ZONA NO kosong",IF(K92="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H92&lt;&gt;K92,"CEK JENIS ZONA",IF(A92="","Zona STOCK",IF(B92="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5275,7 +5275,7 @@
         <v/>
       </c>
       <c r="M93" s="12">
-        <f>IF(AND(A93="",F93=""),"",IF(F93="","Belum ditempatkan",IF(I93="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G93="","CEK ZONA NO kosong",IF(K93="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H93&lt;&gt;K93,"CEK JENIS ZONA",IF(A93="","Zona kosong",IF(B93="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A93="",F93=""),"",IF(F93="","Belum ditempatkan",IF(I93="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G93="","CEK ZONA NO kosong",IF(K93="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H93&lt;&gt;K93,"CEK JENIS ZONA",IF(A93="","Zona STOCK",IF(B93="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
         <v/>
       </c>
       <c r="M94" s="12">
-        <f>IF(AND(A94="",F94=""),"",IF(F94="","Belum ditempatkan",IF(I94="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G94="","CEK ZONA NO kosong",IF(K94="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H94&lt;&gt;K94,"CEK JENIS ZONA",IF(A94="","Zona kosong",IF(B94="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A94="",F94=""),"",IF(F94="","Belum ditempatkan",IF(I94="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G94="","CEK ZONA NO kosong",IF(K94="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H94&lt;&gt;K94,"CEK JENIS ZONA",IF(A94="","Zona STOCK",IF(B94="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
         <v/>
       </c>
       <c r="M95" s="12">
-        <f>IF(AND(A95="",F95=""),"",IF(F95="","Belum ditempatkan",IF(I95="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G95="","CEK ZONA NO kosong",IF(K95="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H95&lt;&gt;K95,"CEK JENIS ZONA",IF(A95="","Zona kosong",IF(B95="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A95="",F95=""),"",IF(F95="","Belum ditempatkan",IF(I95="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G95="","CEK ZONA NO kosong",IF(K95="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H95&lt;&gt;K95,"CEK JENIS ZONA",IF(A95="","Zona STOCK",IF(B95="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
         <v/>
       </c>
       <c r="M96" s="12">
-        <f>IF(AND(A96="",F96=""),"",IF(F96="","Belum ditempatkan",IF(I96="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G96="","CEK ZONA NO kosong",IF(K96="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H96&lt;&gt;K96,"CEK JENIS ZONA",IF(A96="","Zona kosong",IF(B96="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A96="",F96=""),"",IF(F96="","Belum ditempatkan",IF(I96="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G96="","CEK ZONA NO kosong",IF(K96="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H96&lt;&gt;K96,"CEK JENIS ZONA",IF(A96="","Zona STOCK",IF(B96="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="M97" s="12">
-        <f>IF(AND(A97="",F97=""),"",IF(F97="","Belum ditempatkan",IF(I97="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G97="","CEK ZONA NO kosong",IF(K97="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H97&lt;&gt;K97,"CEK JENIS ZONA",IF(A97="","Zona kosong",IF(B97="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A97="",F97=""),"",IF(F97="","Belum ditempatkan",IF(I97="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G97="","CEK ZONA NO kosong",IF(K97="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H97&lt;&gt;K97,"CEK JENIS ZONA",IF(A97="","Zona STOCK",IF(B97="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5515,7 +5515,7 @@
         <v/>
       </c>
       <c r="M98" s="12">
-        <f>IF(AND(A98="",F98=""),"",IF(F98="","Belum ditempatkan",IF(I98="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G98="","CEK ZONA NO kosong",IF(K98="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H98&lt;&gt;K98,"CEK JENIS ZONA",IF(A98="","Zona kosong",IF(B98="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A98="",F98=""),"",IF(F98="","Belum ditempatkan",IF(I98="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G98="","CEK ZONA NO kosong",IF(K98="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H98&lt;&gt;K98,"CEK JENIS ZONA",IF(A98="","Zona STOCK",IF(B98="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
         <v/>
       </c>
       <c r="M99" s="12">
-        <f>IF(AND(A99="",F99=""),"",IF(F99="","Belum ditempatkan",IF(I99="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G99="","CEK ZONA NO kosong",IF(K99="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H99&lt;&gt;K99,"CEK JENIS ZONA",IF(A99="","Zona kosong",IF(B99="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A99="",F99=""),"",IF(F99="","Belum ditempatkan",IF(I99="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G99="","CEK ZONA NO kosong",IF(K99="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H99&lt;&gt;K99,"CEK JENIS ZONA",IF(A99="","Zona STOCK",IF(B99="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5611,7 +5611,7 @@
         <v/>
       </c>
       <c r="M100" s="12">
-        <f>IF(AND(A100="",F100=""),"",IF(F100="","Belum ditempatkan",IF(I100="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G100="","CEK ZONA NO kosong",IF(K100="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H100&lt;&gt;K100,"CEK JENIS ZONA",IF(A100="","Zona kosong",IF(B100="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A100="",F100=""),"",IF(F100="","Belum ditempatkan",IF(I100="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G100="","CEK ZONA NO kosong",IF(K100="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H100&lt;&gt;K100,"CEK JENIS ZONA",IF(A100="","Zona STOCK",IF(B100="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5659,7 +5659,7 @@
         <v/>
       </c>
       <c r="M101" s="12">
-        <f>IF(AND(A101="",F101=""),"",IF(F101="","Belum ditempatkan",IF(I101="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G101="","CEK ZONA NO kosong",IF(K101="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H101&lt;&gt;K101,"CEK JENIS ZONA",IF(A101="","Zona kosong",IF(B101="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A101="",F101=""),"",IF(F101="","Belum ditempatkan",IF(I101="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G101="","CEK ZONA NO kosong",IF(K101="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H101&lt;&gt;K101,"CEK JENIS ZONA",IF(A101="","Zona STOCK",IF(B101="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5707,7 +5707,7 @@
         <v/>
       </c>
       <c r="M102" s="12">
-        <f>IF(AND(A102="",F102=""),"",IF(F102="","Belum ditempatkan",IF(I102="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G102="","CEK ZONA NO kosong",IF(K102="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H102&lt;&gt;K102,"CEK JENIS ZONA",IF(A102="","Zona kosong",IF(B102="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A102="",F102=""),"",IF(F102="","Belum ditempatkan",IF(I102="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G102="","CEK ZONA NO kosong",IF(K102="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H102&lt;&gt;K102,"CEK JENIS ZONA",IF(A102="","Zona STOCK",IF(B102="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5755,7 +5755,7 @@
         <v/>
       </c>
       <c r="M103" s="12">
-        <f>IF(AND(A103="",F103=""),"",IF(F103="","Belum ditempatkan",IF(I103="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G103="","CEK ZONA NO kosong",IF(K103="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H103&lt;&gt;K103,"CEK JENIS ZONA",IF(A103="","Zona kosong",IF(B103="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A103="",F103=""),"",IF(F103="","Belum ditempatkan",IF(I103="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G103="","CEK ZONA NO kosong",IF(K103="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H103&lt;&gt;K103,"CEK JENIS ZONA",IF(A103="","Zona STOCK",IF(B103="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5803,7 +5803,7 @@
         <v/>
       </c>
       <c r="M104" s="12">
-        <f>IF(AND(A104="",F104=""),"",IF(F104="","Belum ditempatkan",IF(I104="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G104="","CEK ZONA NO kosong",IF(K104="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H104&lt;&gt;K104,"CEK JENIS ZONA",IF(A104="","Zona kosong",IF(B104="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A104="",F104=""),"",IF(F104="","Belum ditempatkan",IF(I104="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G104="","CEK ZONA NO kosong",IF(K104="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H104&lt;&gt;K104,"CEK JENIS ZONA",IF(A104="","Zona STOCK",IF(B104="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
         <v/>
       </c>
       <c r="M105" s="12">
-        <f>IF(AND(A105="",F105=""),"",IF(F105="","Belum ditempatkan",IF(I105="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G105="","CEK ZONA NO kosong",IF(K105="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H105&lt;&gt;K105,"CEK JENIS ZONA",IF(A105="","Zona kosong",IF(B105="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A105="",F105=""),"",IF(F105="","Belum ditempatkan",IF(I105="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G105="","CEK ZONA NO kosong",IF(K105="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H105&lt;&gt;K105,"CEK JENIS ZONA",IF(A105="","Zona STOCK",IF(B105="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5899,7 +5899,7 @@
         <v/>
       </c>
       <c r="M106" s="12">
-        <f>IF(AND(A106="",F106=""),"",IF(F106="","Belum ditempatkan",IF(I106="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G106="","CEK ZONA NO kosong",IF(K106="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H106&lt;&gt;K106,"CEK JENIS ZONA",IF(A106="","Zona kosong",IF(B106="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A106="",F106=""),"",IF(F106="","Belum ditempatkan",IF(I106="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G106="","CEK ZONA NO kosong",IF(K106="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H106&lt;&gt;K106,"CEK JENIS ZONA",IF(A106="","Zona STOCK",IF(B106="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
         <v/>
       </c>
       <c r="M107" s="12">
-        <f>IF(AND(A107="",F107=""),"",IF(F107="","Belum ditempatkan",IF(I107="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G107="","CEK ZONA NO kosong",IF(K107="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H107&lt;&gt;K107,"CEK JENIS ZONA",IF(A107="","Zona kosong",IF(B107="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A107="",F107=""),"",IF(F107="","Belum ditempatkan",IF(I107="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G107="","CEK ZONA NO kosong",IF(K107="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H107&lt;&gt;K107,"CEK JENIS ZONA",IF(A107="","Zona STOCK",IF(B107="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
         <v/>
       </c>
       <c r="M108" s="12">
-        <f>IF(AND(A108="",F108=""),"",IF(F108="","Belum ditempatkan",IF(I108="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G108="","CEK ZONA NO kosong",IF(K108="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H108&lt;&gt;K108,"CEK JENIS ZONA",IF(A108="","Zona kosong",IF(B108="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A108="",F108=""),"",IF(F108="","Belum ditempatkan",IF(I108="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G108="","CEK ZONA NO kosong",IF(K108="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H108&lt;&gt;K108,"CEK JENIS ZONA",IF(A108="","Zona STOCK",IF(B108="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6043,7 +6043,7 @@
         <v/>
       </c>
       <c r="M109" s="12">
-        <f>IF(AND(A109="",F109=""),"",IF(F109="","Belum ditempatkan",IF(I109="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G109="","CEK ZONA NO kosong",IF(K109="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H109&lt;&gt;K109,"CEK JENIS ZONA",IF(A109="","Zona kosong",IF(B109="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A109="",F109=""),"",IF(F109="","Belum ditempatkan",IF(I109="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G109="","CEK ZONA NO kosong",IF(K109="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H109&lt;&gt;K109,"CEK JENIS ZONA",IF(A109="","Zona STOCK",IF(B109="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6091,7 +6091,7 @@
         <v/>
       </c>
       <c r="M110" s="12">
-        <f>IF(AND(A110="",F110=""),"",IF(F110="","Belum ditempatkan",IF(I110="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G110="","CEK ZONA NO kosong",IF(K110="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H110&lt;&gt;K110,"CEK JENIS ZONA",IF(A110="","Zona kosong",IF(B110="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A110="",F110=""),"",IF(F110="","Belum ditempatkan",IF(I110="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G110="","CEK ZONA NO kosong",IF(K110="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H110&lt;&gt;K110,"CEK JENIS ZONA",IF(A110="","Zona STOCK",IF(B110="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
         <v/>
       </c>
       <c r="M111" s="12">
-        <f>IF(AND(A111="",F111=""),"",IF(F111="","Belum ditempatkan",IF(I111="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G111="","CEK ZONA NO kosong",IF(K111="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H111&lt;&gt;K111,"CEK JENIS ZONA",IF(A111="","Zona kosong",IF(B111="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A111="",F111=""),"",IF(F111="","Belum ditempatkan",IF(I111="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G111="","CEK ZONA NO kosong",IF(K111="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H111&lt;&gt;K111,"CEK JENIS ZONA",IF(A111="","Zona STOCK",IF(B111="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
         <v/>
       </c>
       <c r="M112" s="12">
-        <f>IF(AND(A112="",F112=""),"",IF(F112="","Belum ditempatkan",IF(I112="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G112="","CEK ZONA NO kosong",IF(K112="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H112&lt;&gt;K112,"CEK JENIS ZONA",IF(A112="","Zona kosong",IF(B112="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A112="",F112=""),"",IF(F112="","Belum ditempatkan",IF(I112="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G112="","CEK ZONA NO kosong",IF(K112="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H112&lt;&gt;K112,"CEK JENIS ZONA",IF(A112="","Zona STOCK",IF(B112="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6235,7 +6235,7 @@
         <v/>
       </c>
       <c r="M113" s="12">
-        <f>IF(AND(A113="",F113=""),"",IF(F113="","Belum ditempatkan",IF(I113="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G113="","CEK ZONA NO kosong",IF(K113="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H113&lt;&gt;K113,"CEK JENIS ZONA",IF(A113="","Zona kosong",IF(B113="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A113="",F113=""),"",IF(F113="","Belum ditempatkan",IF(I113="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G113="","CEK ZONA NO kosong",IF(K113="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H113&lt;&gt;K113,"CEK JENIS ZONA",IF(A113="","Zona STOCK",IF(B113="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6283,7 +6283,7 @@
         <v/>
       </c>
       <c r="M114" s="12">
-        <f>IF(AND(A114="",F114=""),"",IF(F114="","Belum ditempatkan",IF(I114="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G114="","CEK ZONA NO kosong",IF(K114="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H114&lt;&gt;K114,"CEK JENIS ZONA",IF(A114="","Zona kosong",IF(B114="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A114="",F114=""),"",IF(F114="","Belum ditempatkan",IF(I114="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G114="","CEK ZONA NO kosong",IF(K114="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H114&lt;&gt;K114,"CEK JENIS ZONA",IF(A114="","Zona STOCK",IF(B114="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6331,7 +6331,7 @@
         <v/>
       </c>
       <c r="M115" s="12">
-        <f>IF(AND(A115="",F115=""),"",IF(F115="","Belum ditempatkan",IF(I115="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G115="","CEK ZONA NO kosong",IF(K115="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H115&lt;&gt;K115,"CEK JENIS ZONA",IF(A115="","Zona kosong",IF(B115="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A115="",F115=""),"",IF(F115="","Belum ditempatkan",IF(I115="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G115="","CEK ZONA NO kosong",IF(K115="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H115&lt;&gt;K115,"CEK JENIS ZONA",IF(A115="","Zona STOCK",IF(B115="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
         <v/>
       </c>
       <c r="M116" s="12">
-        <f>IF(AND(A116="",F116=""),"",IF(F116="","Belum ditempatkan",IF(I116="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G116="","CEK ZONA NO kosong",IF(K116="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H116&lt;&gt;K116,"CEK JENIS ZONA",IF(A116="","Zona kosong",IF(B116="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A116="",F116=""),"",IF(F116="","Belum ditempatkan",IF(I116="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G116="","CEK ZONA NO kosong",IF(K116="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H116&lt;&gt;K116,"CEK JENIS ZONA",IF(A116="","Zona STOCK",IF(B116="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6427,7 +6427,7 @@
         <v/>
       </c>
       <c r="M117" s="12">
-        <f>IF(AND(A117="",F117=""),"",IF(F117="","Belum ditempatkan",IF(I117="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G117="","CEK ZONA NO kosong",IF(K117="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H117&lt;&gt;K117,"CEK JENIS ZONA",IF(A117="","Zona kosong",IF(B117="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A117="",F117=""),"",IF(F117="","Belum ditempatkan",IF(I117="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G117="","CEK ZONA NO kosong",IF(K117="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H117&lt;&gt;K117,"CEK JENIS ZONA",IF(A117="","Zona STOCK",IF(B117="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6457,7 +6457,7 @@
         <v/>
       </c>
       <c r="M118" s="12">
-        <f>IF(AND(A118="",F118=""),"",IF(F118="","Belum ditempatkan",IF(I118="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G118="","CEK ZONA NO kosong",IF(K118="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H118&lt;&gt;K118,"CEK JENIS ZONA",IF(A118="","Zona kosong",IF(B118="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A118="",F118=""),"",IF(F118="","Belum ditempatkan",IF(I118="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G118="","CEK ZONA NO kosong",IF(K118="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H118&lt;&gt;K118,"CEK JENIS ZONA",IF(A118="","Zona STOCK",IF(B118="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
         <v/>
       </c>
       <c r="M119" s="12">
-        <f>IF(AND(A119="",F119=""),"",IF(F119="","Belum ditempatkan",IF(I119="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G119="","CEK ZONA NO kosong",IF(K119="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H119&lt;&gt;K119,"CEK JENIS ZONA",IF(A119="","Zona kosong",IF(B119="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A119="",F119=""),"",IF(F119="","Belum ditempatkan",IF(I119="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G119="","CEK ZONA NO kosong",IF(K119="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H119&lt;&gt;K119,"CEK JENIS ZONA",IF(A119="","Zona STOCK",IF(B119="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6517,7 +6517,7 @@
         <v/>
       </c>
       <c r="M120" s="12">
-        <f>IF(AND(A120="",F120=""),"",IF(F120="","Belum ditempatkan",IF(I120="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G120="","CEK ZONA NO kosong",IF(K120="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H120&lt;&gt;K120,"CEK JENIS ZONA",IF(A120="","Zona kosong",IF(B120="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A120="",F120=""),"",IF(F120="","Belum ditempatkan",IF(I120="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G120="","CEK ZONA NO kosong",IF(K120="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H120&lt;&gt;K120,"CEK JENIS ZONA",IF(A120="","Zona STOCK",IF(B120="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6547,7 +6547,7 @@
         <v/>
       </c>
       <c r="M121" s="12">
-        <f>IF(AND(A121="",F121=""),"",IF(F121="","Belum ditempatkan",IF(I121="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G121="","CEK ZONA NO kosong",IF(K121="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H121&lt;&gt;K121,"CEK JENIS ZONA",IF(A121="","Zona kosong",IF(B121="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A121="",F121=""),"",IF(F121="","Belum ditempatkan",IF(I121="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G121="","CEK ZONA NO kosong",IF(K121="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H121&lt;&gt;K121,"CEK JENIS ZONA",IF(A121="","Zona STOCK",IF(B121="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6577,7 +6577,7 @@
         <v/>
       </c>
       <c r="M122" s="12">
-        <f>IF(AND(A122="",F122=""),"",IF(F122="","Belum ditempatkan",IF(I122="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G122="","CEK ZONA NO kosong",IF(K122="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H122&lt;&gt;K122,"CEK JENIS ZONA",IF(A122="","Zona kosong",IF(B122="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A122="",F122=""),"",IF(F122="","Belum ditempatkan",IF(I122="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G122="","CEK ZONA NO kosong",IF(K122="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H122&lt;&gt;K122,"CEK JENIS ZONA",IF(A122="","Zona STOCK",IF(B122="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
         <v/>
       </c>
       <c r="M123" s="12">
-        <f>IF(AND(A123="",F123=""),"",IF(F123="","Belum ditempatkan",IF(I123="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G123="","CEK ZONA NO kosong",IF(K123="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H123&lt;&gt;K123,"CEK JENIS ZONA",IF(A123="","Zona kosong",IF(B123="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A123="",F123=""),"",IF(F123="","Belum ditempatkan",IF(I123="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G123="","CEK ZONA NO kosong",IF(K123="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H123&lt;&gt;K123,"CEK JENIS ZONA",IF(A123="","Zona STOCK",IF(B123="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
         <v/>
       </c>
       <c r="M124" s="12">
-        <f>IF(AND(A124="",F124=""),"",IF(F124="","Belum ditempatkan",IF(I124="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G124="","CEK ZONA NO kosong",IF(K124="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H124&lt;&gt;K124,"CEK JENIS ZONA",IF(A124="","Zona kosong",IF(B124="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A124="",F124=""),"",IF(F124="","Belum ditempatkan",IF(I124="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G124="","CEK ZONA NO kosong",IF(K124="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H124&lt;&gt;K124,"CEK JENIS ZONA",IF(A124="","Zona STOCK",IF(B124="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6667,7 +6667,7 @@
         <v/>
       </c>
       <c r="M125" s="12">
-        <f>IF(AND(A125="",F125=""),"",IF(F125="","Belum ditempatkan",IF(I125="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G125="","CEK ZONA NO kosong",IF(K125="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H125&lt;&gt;K125,"CEK JENIS ZONA",IF(A125="","Zona kosong",IF(B125="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A125="",F125=""),"",IF(F125="","Belum ditempatkan",IF(I125="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G125="","CEK ZONA NO kosong",IF(K125="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H125&lt;&gt;K125,"CEK JENIS ZONA",IF(A125="","Zona STOCK",IF(B125="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
         <v/>
       </c>
       <c r="M126" s="12">
-        <f>IF(AND(A126="",F126=""),"",IF(F126="","Belum ditempatkan",IF(I126="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G126="","CEK ZONA NO kosong",IF(K126="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H126&lt;&gt;K126,"CEK JENIS ZONA",IF(A126="","Zona kosong",IF(B126="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A126="",F126=""),"",IF(F126="","Belum ditempatkan",IF(I126="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G126="","CEK ZONA NO kosong",IF(K126="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H126&lt;&gt;K126,"CEK JENIS ZONA",IF(A126="","Zona STOCK",IF(B126="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6727,7 +6727,7 @@
         <v/>
       </c>
       <c r="M127" s="12">
-        <f>IF(AND(A127="",F127=""),"",IF(F127="","Belum ditempatkan",IF(I127="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G127="","CEK ZONA NO kosong",IF(K127="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H127&lt;&gt;K127,"CEK JENIS ZONA",IF(A127="","Zona kosong",IF(B127="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A127="",F127=""),"",IF(F127="","Belum ditempatkan",IF(I127="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G127="","CEK ZONA NO kosong",IF(K127="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H127&lt;&gt;K127,"CEK JENIS ZONA",IF(A127="","Zona STOCK",IF(B127="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6757,7 +6757,7 @@
         <v/>
       </c>
       <c r="M128" s="12">
-        <f>IF(AND(A128="",F128=""),"",IF(F128="","Belum ditempatkan",IF(I128="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G128="","CEK ZONA NO kosong",IF(K128="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H128&lt;&gt;K128,"CEK JENIS ZONA",IF(A128="","Zona kosong",IF(B128="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A128="",F128=""),"",IF(F128="","Belum ditempatkan",IF(I128="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G128="","CEK ZONA NO kosong",IF(K128="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H128&lt;&gt;K128,"CEK JENIS ZONA",IF(A128="","Zona STOCK",IF(B128="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6787,7 +6787,7 @@
         <v/>
       </c>
       <c r="M129" s="12">
-        <f>IF(AND(A129="",F129=""),"",IF(F129="","Belum ditempatkan",IF(I129="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G129="","CEK ZONA NO kosong",IF(K129="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H129&lt;&gt;K129,"CEK JENIS ZONA",IF(A129="","Zona kosong",IF(B129="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A129="",F129=""),"",IF(F129="","Belum ditempatkan",IF(I129="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G129="","CEK ZONA NO kosong",IF(K129="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H129&lt;&gt;K129,"CEK JENIS ZONA",IF(A129="","Zona STOCK",IF(B129="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6817,7 +6817,7 @@
         <v/>
       </c>
       <c r="M130" s="12">
-        <f>IF(AND(A130="",F130=""),"",IF(F130="","Belum ditempatkan",IF(I130="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G130="","CEK ZONA NO kosong",IF(K130="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H130&lt;&gt;K130,"CEK JENIS ZONA",IF(A130="","Zona kosong",IF(B130="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A130="",F130=""),"",IF(F130="","Belum ditempatkan",IF(I130="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G130="","CEK ZONA NO kosong",IF(K130="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H130&lt;&gt;K130,"CEK JENIS ZONA",IF(A130="","Zona STOCK",IF(B130="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
         <v/>
       </c>
       <c r="M131" s="12">
-        <f>IF(AND(A131="",F131=""),"",IF(F131="","Belum ditempatkan",IF(I131="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G131="","CEK ZONA NO kosong",IF(K131="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H131&lt;&gt;K131,"CEK JENIS ZONA",IF(A131="","Zona kosong",IF(B131="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A131="",F131=""),"",IF(F131="","Belum ditempatkan",IF(I131="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G131="","CEK ZONA NO kosong",IF(K131="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H131&lt;&gt;K131,"CEK JENIS ZONA",IF(A131="","Zona STOCK",IF(B131="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6877,7 +6877,7 @@
         <v/>
       </c>
       <c r="M132" s="12">
-        <f>IF(AND(A132="",F132=""),"",IF(F132="","Belum ditempatkan",IF(I132="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G132="","CEK ZONA NO kosong",IF(K132="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H132&lt;&gt;K132,"CEK JENIS ZONA",IF(A132="","Zona kosong",IF(B132="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A132="",F132=""),"",IF(F132="","Belum ditempatkan",IF(I132="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G132="","CEK ZONA NO kosong",IF(K132="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H132&lt;&gt;K132,"CEK JENIS ZONA",IF(A132="","Zona STOCK",IF(B132="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6907,7 +6907,7 @@
         <v/>
       </c>
       <c r="M133" s="12">
-        <f>IF(AND(A133="",F133=""),"",IF(F133="","Belum ditempatkan",IF(I133="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G133="","CEK ZONA NO kosong",IF(K133="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H133&lt;&gt;K133,"CEK JENIS ZONA",IF(A133="","Zona kosong",IF(B133="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A133="",F133=""),"",IF(F133="","Belum ditempatkan",IF(I133="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G133="","CEK ZONA NO kosong",IF(K133="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H133&lt;&gt;K133,"CEK JENIS ZONA",IF(A133="","Zona STOCK",IF(B133="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6937,7 +6937,7 @@
         <v/>
       </c>
       <c r="M134" s="12">
-        <f>IF(AND(A134="",F134=""),"",IF(F134="","Belum ditempatkan",IF(I134="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G134="","CEK ZONA NO kosong",IF(K134="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H134&lt;&gt;K134,"CEK JENIS ZONA",IF(A134="","Zona kosong",IF(B134="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A134="",F134=""),"",IF(F134="","Belum ditempatkan",IF(I134="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G134="","CEK ZONA NO kosong",IF(K134="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H134&lt;&gt;K134,"CEK JENIS ZONA",IF(A134="","Zona STOCK",IF(B134="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6967,7 +6967,7 @@
         <v/>
       </c>
       <c r="M135" s="12">
-        <f>IF(AND(A135="",F135=""),"",IF(F135="","Belum ditempatkan",IF(I135="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G135="","CEK ZONA NO kosong",IF(K135="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H135&lt;&gt;K135,"CEK JENIS ZONA",IF(A135="","Zona kosong",IF(B135="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A135="",F135=""),"",IF(F135="","Belum ditempatkan",IF(I135="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G135="","CEK ZONA NO kosong",IF(K135="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H135&lt;&gt;K135,"CEK JENIS ZONA",IF(A135="","Zona STOCK",IF(B135="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -6997,7 +6997,7 @@
         <v/>
       </c>
       <c r="M136" s="12">
-        <f>IF(AND(A136="",F136=""),"",IF(F136="","Belum ditempatkan",IF(I136="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G136="","CEK ZONA NO kosong",IF(K136="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H136&lt;&gt;K136,"CEK JENIS ZONA",IF(A136="","Zona kosong",IF(B136="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A136="",F136=""),"",IF(F136="","Belum ditempatkan",IF(I136="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G136="","CEK ZONA NO kosong",IF(K136="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H136&lt;&gt;K136,"CEK JENIS ZONA",IF(A136="","Zona STOCK",IF(B136="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7027,7 +7027,7 @@
         <v/>
       </c>
       <c r="M137" s="12">
-        <f>IF(AND(A137="",F137=""),"",IF(F137="","Belum ditempatkan",IF(I137="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G137="","CEK ZONA NO kosong",IF(K137="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H137&lt;&gt;K137,"CEK JENIS ZONA",IF(A137="","Zona kosong",IF(B137="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A137="",F137=""),"",IF(F137="","Belum ditempatkan",IF(I137="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G137="","CEK ZONA NO kosong",IF(K137="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H137&lt;&gt;K137,"CEK JENIS ZONA",IF(A137="","Zona STOCK",IF(B137="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="M138" s="12">
-        <f>IF(AND(A138="",F138=""),"",IF(F138="","Belum ditempatkan",IF(I138="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G138="","CEK ZONA NO kosong",IF(K138="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H138&lt;&gt;K138,"CEK JENIS ZONA",IF(A138="","Zona kosong",IF(B138="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A138="",F138=""),"",IF(F138="","Belum ditempatkan",IF(I138="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G138="","CEK ZONA NO kosong",IF(K138="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H138&lt;&gt;K138,"CEK JENIS ZONA",IF(A138="","Zona STOCK",IF(B138="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7087,7 +7087,7 @@
         <v/>
       </c>
       <c r="M139" s="12">
-        <f>IF(AND(A139="",F139=""),"",IF(F139="","Belum ditempatkan",IF(I139="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G139="","CEK ZONA NO kosong",IF(K139="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H139&lt;&gt;K139,"CEK JENIS ZONA",IF(A139="","Zona kosong",IF(B139="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A139="",F139=""),"",IF(F139="","Belum ditempatkan",IF(I139="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G139="","CEK ZONA NO kosong",IF(K139="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H139&lt;&gt;K139,"CEK JENIS ZONA",IF(A139="","Zona STOCK",IF(B139="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7117,7 +7117,7 @@
         <v/>
       </c>
       <c r="M140" s="12">
-        <f>IF(AND(A140="",F140=""),"",IF(F140="","Belum ditempatkan",IF(I140="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G140="","CEK ZONA NO kosong",IF(K140="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H140&lt;&gt;K140,"CEK JENIS ZONA",IF(A140="","Zona kosong",IF(B140="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A140="",F140=""),"",IF(F140="","Belum ditempatkan",IF(I140="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G140="","CEK ZONA NO kosong",IF(K140="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H140&lt;&gt;K140,"CEK JENIS ZONA",IF(A140="","Zona STOCK",IF(B140="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7147,7 +7147,7 @@
         <v/>
       </c>
       <c r="M141" s="12">
-        <f>IF(AND(A141="",F141=""),"",IF(F141="","Belum ditempatkan",IF(I141="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G141="","CEK ZONA NO kosong",IF(K141="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H141&lt;&gt;K141,"CEK JENIS ZONA",IF(A141="","Zona kosong",IF(B141="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A141="",F141=""),"",IF(F141="","Belum ditempatkan",IF(I141="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G141="","CEK ZONA NO kosong",IF(K141="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H141&lt;&gt;K141,"CEK JENIS ZONA",IF(A141="","Zona STOCK",IF(B141="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7177,7 +7177,7 @@
         <v/>
       </c>
       <c r="M142" s="12">
-        <f>IF(AND(A142="",F142=""),"",IF(F142="","Belum ditempatkan",IF(I142="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G142="","CEK ZONA NO kosong",IF(K142="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H142&lt;&gt;K142,"CEK JENIS ZONA",IF(A142="","Zona kosong",IF(B142="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A142="",F142=""),"",IF(F142="","Belum ditempatkan",IF(I142="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G142="","CEK ZONA NO kosong",IF(K142="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H142&lt;&gt;K142,"CEK JENIS ZONA",IF(A142="","Zona STOCK",IF(B142="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7207,7 +7207,7 @@
         <v/>
       </c>
       <c r="M143" s="12">
-        <f>IF(AND(A143="",F143=""),"",IF(F143="","Belum ditempatkan",IF(I143="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G143="","CEK ZONA NO kosong",IF(K143="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H143&lt;&gt;K143,"CEK JENIS ZONA",IF(A143="","Zona kosong",IF(B143="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A143="",F143=""),"",IF(F143="","Belum ditempatkan",IF(I143="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G143="","CEK ZONA NO kosong",IF(K143="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H143&lt;&gt;K143,"CEK JENIS ZONA",IF(A143="","Zona STOCK",IF(B143="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
         <v/>
       </c>
       <c r="M144" s="12">
-        <f>IF(AND(A144="",F144=""),"",IF(F144="","Belum ditempatkan",IF(I144="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G144="","CEK ZONA NO kosong",IF(K144="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H144&lt;&gt;K144,"CEK JENIS ZONA",IF(A144="","Zona kosong",IF(B144="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A144="",F144=""),"",IF(F144="","Belum ditempatkan",IF(I144="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G144="","CEK ZONA NO kosong",IF(K144="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H144&lt;&gt;K144,"CEK JENIS ZONA",IF(A144="","Zona STOCK",IF(B144="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7267,7 +7267,7 @@
         <v/>
       </c>
       <c r="M145" s="12">
-        <f>IF(AND(A145="",F145=""),"",IF(F145="","Belum ditempatkan",IF(I145="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G145="","CEK ZONA NO kosong",IF(K145="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H145&lt;&gt;K145,"CEK JENIS ZONA",IF(A145="","Zona kosong",IF(B145="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A145="",F145=""),"",IF(F145="","Belum ditempatkan",IF(I145="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G145="","CEK ZONA NO kosong",IF(K145="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H145&lt;&gt;K145,"CEK JENIS ZONA",IF(A145="","Zona STOCK",IF(B145="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
         <v/>
       </c>
       <c r="M146" s="12">
-        <f>IF(AND(A146="",F146=""),"",IF(F146="","Belum ditempatkan",IF(I146="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G146="","CEK ZONA NO kosong",IF(K146="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H146&lt;&gt;K146,"CEK JENIS ZONA",IF(A146="","Zona kosong",IF(B146="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A146="",F146=""),"",IF(F146="","Belum ditempatkan",IF(I146="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G146="","CEK ZONA NO kosong",IF(K146="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H146&lt;&gt;K146,"CEK JENIS ZONA",IF(A146="","Zona STOCK",IF(B146="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7327,7 +7327,7 @@
         <v/>
       </c>
       <c r="M147" s="12">
-        <f>IF(AND(A147="",F147=""),"",IF(F147="","Belum ditempatkan",IF(I147="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G147="","CEK ZONA NO kosong",IF(K147="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H147&lt;&gt;K147,"CEK JENIS ZONA",IF(A147="","Zona kosong",IF(B147="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A147="",F147=""),"",IF(F147="","Belum ditempatkan",IF(I147="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G147="","CEK ZONA NO kosong",IF(K147="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H147&lt;&gt;K147,"CEK JENIS ZONA",IF(A147="","Zona STOCK",IF(B147="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7357,7 +7357,7 @@
         <v/>
       </c>
       <c r="M148" s="12">
-        <f>IF(AND(A148="",F148=""),"",IF(F148="","Belum ditempatkan",IF(I148="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G148="","CEK ZONA NO kosong",IF(K148="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H148&lt;&gt;K148,"CEK JENIS ZONA",IF(A148="","Zona kosong",IF(B148="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A148="",F148=""),"",IF(F148="","Belum ditempatkan",IF(I148="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G148="","CEK ZONA NO kosong",IF(K148="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H148&lt;&gt;K148,"CEK JENIS ZONA",IF(A148="","Zona STOCK",IF(B148="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7387,7 +7387,7 @@
         <v/>
       </c>
       <c r="M149" s="12">
-        <f>IF(AND(A149="",F149=""),"",IF(F149="","Belum ditempatkan",IF(I149="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G149="","CEK ZONA NO kosong",IF(K149="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H149&lt;&gt;K149,"CEK JENIS ZONA",IF(A149="","Zona kosong",IF(B149="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A149="",F149=""),"",IF(F149="","Belum ditempatkan",IF(I149="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G149="","CEK ZONA NO kosong",IF(K149="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H149&lt;&gt;K149,"CEK JENIS ZONA",IF(A149="","Zona STOCK",IF(B149="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7417,7 +7417,7 @@
         <v/>
       </c>
       <c r="M150" s="12">
-        <f>IF(AND(A150="",F150=""),"",IF(F150="","Belum ditempatkan",IF(I150="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G150="","CEK ZONA NO kosong",IF(K150="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H150&lt;&gt;K150,"CEK JENIS ZONA",IF(A150="","Zona kosong",IF(B150="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A150="",F150=""),"",IF(F150="","Belum ditempatkan",IF(I150="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G150="","CEK ZONA NO kosong",IF(K150="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H150&lt;&gt;K150,"CEK JENIS ZONA",IF(A150="","Zona STOCK",IF(B150="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
         <v/>
       </c>
       <c r="M151" s="12">
-        <f>IF(AND(A151="",F151=""),"",IF(F151="","Belum ditempatkan",IF(I151="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G151="","CEK ZONA NO kosong",IF(K151="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H151&lt;&gt;K151,"CEK JENIS ZONA",IF(A151="","Zona kosong",IF(B151="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A151="",F151=""),"",IF(F151="","Belum ditempatkan",IF(I151="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G151="","CEK ZONA NO kosong",IF(K151="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H151&lt;&gt;K151,"CEK JENIS ZONA",IF(A151="","Zona STOCK",IF(B151="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7477,7 +7477,7 @@
         <v/>
       </c>
       <c r="M152" s="12">
-        <f>IF(AND(A152="",F152=""),"",IF(F152="","Belum ditempatkan",IF(I152="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G152="","CEK ZONA NO kosong",IF(K152="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H152&lt;&gt;K152,"CEK JENIS ZONA",IF(A152="","Zona kosong",IF(B152="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A152="",F152=""),"",IF(F152="","Belum ditempatkan",IF(I152="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G152="","CEK ZONA NO kosong",IF(K152="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H152&lt;&gt;K152,"CEK JENIS ZONA",IF(A152="","Zona STOCK",IF(B152="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7507,7 +7507,7 @@
         <v/>
       </c>
       <c r="M153" s="12">
-        <f>IF(AND(A153="",F153=""),"",IF(F153="","Belum ditempatkan",IF(I153="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G153="","CEK ZONA NO kosong",IF(K153="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H153&lt;&gt;K153,"CEK JENIS ZONA",IF(A153="","Zona kosong",IF(B153="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A153="",F153=""),"",IF(F153="","Belum ditempatkan",IF(I153="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G153="","CEK ZONA NO kosong",IF(K153="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H153&lt;&gt;K153,"CEK JENIS ZONA",IF(A153="","Zona STOCK",IF(B153="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7537,7 +7537,7 @@
         <v/>
       </c>
       <c r="M154" s="12">
-        <f>IF(AND(A154="",F154=""),"",IF(F154="","Belum ditempatkan",IF(I154="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G154="","CEK ZONA NO kosong",IF(K154="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H154&lt;&gt;K154,"CEK JENIS ZONA",IF(A154="","Zona kosong",IF(B154="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A154="",F154=""),"",IF(F154="","Belum ditempatkan",IF(I154="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G154="","CEK ZONA NO kosong",IF(K154="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H154&lt;&gt;K154,"CEK JENIS ZONA",IF(A154="","Zona STOCK",IF(B154="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7567,7 +7567,7 @@
         <v/>
       </c>
       <c r="M155" s="12">
-        <f>IF(AND(A155="",F155=""),"",IF(F155="","Belum ditempatkan",IF(I155="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G155="","CEK ZONA NO kosong",IF(K155="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H155&lt;&gt;K155,"CEK JENIS ZONA",IF(A155="","Zona kosong",IF(B155="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A155="",F155=""),"",IF(F155="","Belum ditempatkan",IF(I155="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G155="","CEK ZONA NO kosong",IF(K155="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H155&lt;&gt;K155,"CEK JENIS ZONA",IF(A155="","Zona STOCK",IF(B155="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7597,7 +7597,7 @@
         <v/>
       </c>
       <c r="M156" s="12">
-        <f>IF(AND(A156="",F156=""),"",IF(F156="","Belum ditempatkan",IF(I156="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G156="","CEK ZONA NO kosong",IF(K156="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H156&lt;&gt;K156,"CEK JENIS ZONA",IF(A156="","Zona kosong",IF(B156="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A156="",F156=""),"",IF(F156="","Belum ditempatkan",IF(I156="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G156="","CEK ZONA NO kosong",IF(K156="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H156&lt;&gt;K156,"CEK JENIS ZONA",IF(A156="","Zona STOCK",IF(B156="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
         <v/>
       </c>
       <c r="M157" s="12">
-        <f>IF(AND(A157="",F157=""),"",IF(F157="","Belum ditempatkan",IF(I157="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G157="","CEK ZONA NO kosong",IF(K157="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H157&lt;&gt;K157,"CEK JENIS ZONA",IF(A157="","Zona kosong",IF(B157="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A157="",F157=""),"",IF(F157="","Belum ditempatkan",IF(I157="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G157="","CEK ZONA NO kosong",IF(K157="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H157&lt;&gt;K157,"CEK JENIS ZONA",IF(A157="","Zona STOCK",IF(B157="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7657,7 +7657,7 @@
         <v/>
       </c>
       <c r="M158" s="12">
-        <f>IF(AND(A158="",F158=""),"",IF(F158="","Belum ditempatkan",IF(I158="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G158="","CEK ZONA NO kosong",IF(K158="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H158&lt;&gt;K158,"CEK JENIS ZONA",IF(A158="","Zona kosong",IF(B158="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A158="",F158=""),"",IF(F158="","Belum ditempatkan",IF(I158="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G158="","CEK ZONA NO kosong",IF(K158="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H158&lt;&gt;K158,"CEK JENIS ZONA",IF(A158="","Zona STOCK",IF(B158="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7687,7 +7687,7 @@
         <v/>
       </c>
       <c r="M159" s="12">
-        <f>IF(AND(A159="",F159=""),"",IF(F159="","Belum ditempatkan",IF(I159="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G159="","CEK ZONA NO kosong",IF(K159="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H159&lt;&gt;K159,"CEK JENIS ZONA",IF(A159="","Zona kosong",IF(B159="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A159="",F159=""),"",IF(F159="","Belum ditempatkan",IF(I159="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G159="","CEK ZONA NO kosong",IF(K159="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H159&lt;&gt;K159,"CEK JENIS ZONA",IF(A159="","Zona STOCK",IF(B159="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7717,7 +7717,7 @@
         <v/>
       </c>
       <c r="M160" s="12">
-        <f>IF(AND(A160="",F160=""),"",IF(F160="","Belum ditempatkan",IF(I160="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G160="","CEK ZONA NO kosong",IF(K160="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H160&lt;&gt;K160,"CEK JENIS ZONA",IF(A160="","Zona kosong",IF(B160="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A160="",F160=""),"",IF(F160="","Belum ditempatkan",IF(I160="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G160="","CEK ZONA NO kosong",IF(K160="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H160&lt;&gt;K160,"CEK JENIS ZONA",IF(A160="","Zona STOCK",IF(B160="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7747,7 +7747,7 @@
         <v/>
       </c>
       <c r="M161" s="12">
-        <f>IF(AND(A161="",F161=""),"",IF(F161="","Belum ditempatkan",IF(I161="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G161="","CEK ZONA NO kosong",IF(K161="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H161&lt;&gt;K161,"CEK JENIS ZONA",IF(A161="","Zona kosong",IF(B161="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A161="",F161=""),"",IF(F161="","Belum ditempatkan",IF(I161="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G161="","CEK ZONA NO kosong",IF(K161="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H161&lt;&gt;K161,"CEK JENIS ZONA",IF(A161="","Zona STOCK",IF(B161="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7777,7 +7777,7 @@
         <v/>
       </c>
       <c r="M162" s="12">
-        <f>IF(AND(A162="",F162=""),"",IF(F162="","Belum ditempatkan",IF(I162="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G162="","CEK ZONA NO kosong",IF(K162="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H162&lt;&gt;K162,"CEK JENIS ZONA",IF(A162="","Zona kosong",IF(B162="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A162="",F162=""),"",IF(F162="","Belum ditempatkan",IF(I162="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G162="","CEK ZONA NO kosong",IF(K162="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H162&lt;&gt;K162,"CEK JENIS ZONA",IF(A162="","Zona STOCK",IF(B162="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7807,7 +7807,7 @@
         <v/>
       </c>
       <c r="M163" s="12">
-        <f>IF(AND(A163="",F163=""),"",IF(F163="","Belum ditempatkan",IF(I163="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G163="","CEK ZONA NO kosong",IF(K163="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H163&lt;&gt;K163,"CEK JENIS ZONA",IF(A163="","Zona kosong",IF(B163="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A163="",F163=""),"",IF(F163="","Belum ditempatkan",IF(I163="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G163="","CEK ZONA NO kosong",IF(K163="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H163&lt;&gt;K163,"CEK JENIS ZONA",IF(A163="","Zona STOCK",IF(B163="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
         <v/>
       </c>
       <c r="M164" s="12">
-        <f>IF(AND(A164="",F164=""),"",IF(F164="","Belum ditempatkan",IF(I164="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G164="","CEK ZONA NO kosong",IF(K164="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H164&lt;&gt;K164,"CEK JENIS ZONA",IF(A164="","Zona kosong",IF(B164="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A164="",F164=""),"",IF(F164="","Belum ditempatkan",IF(I164="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G164="","CEK ZONA NO kosong",IF(K164="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H164&lt;&gt;K164,"CEK JENIS ZONA",IF(A164="","Zona STOCK",IF(B164="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7867,7 +7867,7 @@
         <v/>
       </c>
       <c r="M165" s="12">
-        <f>IF(AND(A165="",F165=""),"",IF(F165="","Belum ditempatkan",IF(I165="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G165="","CEK ZONA NO kosong",IF(K165="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H165&lt;&gt;K165,"CEK JENIS ZONA",IF(A165="","Zona kosong",IF(B165="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A165="",F165=""),"",IF(F165="","Belum ditempatkan",IF(I165="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G165="","CEK ZONA NO kosong",IF(K165="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H165&lt;&gt;K165,"CEK JENIS ZONA",IF(A165="","Zona STOCK",IF(B165="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7897,7 +7897,7 @@
         <v/>
       </c>
       <c r="M166" s="12">
-        <f>IF(AND(A166="",F166=""),"",IF(F166="","Belum ditempatkan",IF(I166="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G166="","CEK ZONA NO kosong",IF(K166="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H166&lt;&gt;K166,"CEK JENIS ZONA",IF(A166="","Zona kosong",IF(B166="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A166="",F166=""),"",IF(F166="","Belum ditempatkan",IF(I166="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G166="","CEK ZONA NO kosong",IF(K166="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H166&lt;&gt;K166,"CEK JENIS ZONA",IF(A166="","Zona STOCK",IF(B166="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7927,7 +7927,7 @@
         <v/>
       </c>
       <c r="M167" s="12">
-        <f>IF(AND(A167="",F167=""),"",IF(F167="","Belum ditempatkan",IF(I167="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G167="","CEK ZONA NO kosong",IF(K167="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H167&lt;&gt;K167,"CEK JENIS ZONA",IF(A167="","Zona kosong",IF(B167="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A167="",F167=""),"",IF(F167="","Belum ditempatkan",IF(I167="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G167="","CEK ZONA NO kosong",IF(K167="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H167&lt;&gt;K167,"CEK JENIS ZONA",IF(A167="","Zona STOCK",IF(B167="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7957,7 +7957,7 @@
         <v/>
       </c>
       <c r="M168" s="12">
-        <f>IF(AND(A168="",F168=""),"",IF(F168="","Belum ditempatkan",IF(I168="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G168="","CEK ZONA NO kosong",IF(K168="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H168&lt;&gt;K168,"CEK JENIS ZONA",IF(A168="","Zona kosong",IF(B168="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A168="",F168=""),"",IF(F168="","Belum ditempatkan",IF(I168="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G168="","CEK ZONA NO kosong",IF(K168="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H168&lt;&gt;K168,"CEK JENIS ZONA",IF(A168="","Zona STOCK",IF(B168="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -7987,7 +7987,7 @@
         <v/>
       </c>
       <c r="M169" s="12">
-        <f>IF(AND(A169="",F169=""),"",IF(F169="","Belum ditempatkan",IF(I169="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G169="","CEK ZONA NO kosong",IF(K169="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H169&lt;&gt;K169,"CEK JENIS ZONA",IF(A169="","Zona kosong",IF(B169="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A169="",F169=""),"",IF(F169="","Belum ditempatkan",IF(I169="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G169="","CEK ZONA NO kosong",IF(K169="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H169&lt;&gt;K169,"CEK JENIS ZONA",IF(A169="","Zona STOCK",IF(B169="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
         <v/>
       </c>
       <c r="M170" s="12">
-        <f>IF(AND(A170="",F170=""),"",IF(F170="","Belum ditempatkan",IF(I170="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G170="","CEK ZONA NO kosong",IF(K170="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H170&lt;&gt;K170,"CEK JENIS ZONA",IF(A170="","Zona kosong",IF(B170="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A170="",F170=""),"",IF(F170="","Belum ditempatkan",IF(I170="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G170="","CEK ZONA NO kosong",IF(K170="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H170&lt;&gt;K170,"CEK JENIS ZONA",IF(A170="","Zona STOCK",IF(B170="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8047,7 +8047,7 @@
         <v/>
       </c>
       <c r="M171" s="12">
-        <f>IF(AND(A171="",F171=""),"",IF(F171="","Belum ditempatkan",IF(I171="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G171="","CEK ZONA NO kosong",IF(K171="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H171&lt;&gt;K171,"CEK JENIS ZONA",IF(A171="","Zona kosong",IF(B171="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A171="",F171=""),"",IF(F171="","Belum ditempatkan",IF(I171="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G171="","CEK ZONA NO kosong",IF(K171="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H171&lt;&gt;K171,"CEK JENIS ZONA",IF(A171="","Zona STOCK",IF(B171="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8077,7 +8077,7 @@
         <v/>
       </c>
       <c r="M172" s="12">
-        <f>IF(AND(A172="",F172=""),"",IF(F172="","Belum ditempatkan",IF(I172="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G172="","CEK ZONA NO kosong",IF(K172="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H172&lt;&gt;K172,"CEK JENIS ZONA",IF(A172="","Zona kosong",IF(B172="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A172="",F172=""),"",IF(F172="","Belum ditempatkan",IF(I172="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G172="","CEK ZONA NO kosong",IF(K172="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H172&lt;&gt;K172,"CEK JENIS ZONA",IF(A172="","Zona STOCK",IF(B172="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8107,7 +8107,7 @@
         <v/>
       </c>
       <c r="M173" s="12">
-        <f>IF(AND(A173="",F173=""),"",IF(F173="","Belum ditempatkan",IF(I173="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G173="","CEK ZONA NO kosong",IF(K173="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H173&lt;&gt;K173,"CEK JENIS ZONA",IF(A173="","Zona kosong",IF(B173="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A173="",F173=""),"",IF(F173="","Belum ditempatkan",IF(I173="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G173="","CEK ZONA NO kosong",IF(K173="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H173&lt;&gt;K173,"CEK JENIS ZONA",IF(A173="","Zona STOCK",IF(B173="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8137,7 +8137,7 @@
         <v/>
       </c>
       <c r="M174" s="12">
-        <f>IF(AND(A174="",F174=""),"",IF(F174="","Belum ditempatkan",IF(I174="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G174="","CEK ZONA NO kosong",IF(K174="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H174&lt;&gt;K174,"CEK JENIS ZONA",IF(A174="","Zona kosong",IF(B174="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A174="",F174=""),"",IF(F174="","Belum ditempatkan",IF(I174="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G174="","CEK ZONA NO kosong",IF(K174="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H174&lt;&gt;K174,"CEK JENIS ZONA",IF(A174="","Zona STOCK",IF(B174="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8167,7 +8167,7 @@
         <v/>
       </c>
       <c r="M175" s="12">
-        <f>IF(AND(A175="",F175=""),"",IF(F175="","Belum ditempatkan",IF(I175="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G175="","CEK ZONA NO kosong",IF(K175="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H175&lt;&gt;K175,"CEK JENIS ZONA",IF(A175="","Zona kosong",IF(B175="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A175="",F175=""),"",IF(F175="","Belum ditempatkan",IF(I175="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G175="","CEK ZONA NO kosong",IF(K175="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H175&lt;&gt;K175,"CEK JENIS ZONA",IF(A175="","Zona STOCK",IF(B175="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8197,7 +8197,7 @@
         <v/>
       </c>
       <c r="M176" s="12">
-        <f>IF(AND(A176="",F176=""),"",IF(F176="","Belum ditempatkan",IF(I176="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G176="","CEK ZONA NO kosong",IF(K176="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H176&lt;&gt;K176,"CEK JENIS ZONA",IF(A176="","Zona kosong",IF(B176="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A176="",F176=""),"",IF(F176="","Belum ditempatkan",IF(I176="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G176="","CEK ZONA NO kosong",IF(K176="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H176&lt;&gt;K176,"CEK JENIS ZONA",IF(A176="","Zona STOCK",IF(B176="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8227,7 +8227,7 @@
         <v/>
       </c>
       <c r="M177" s="12">
-        <f>IF(AND(A177="",F177=""),"",IF(F177="","Belum ditempatkan",IF(I177="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G177="","CEK ZONA NO kosong",IF(K177="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H177&lt;&gt;K177,"CEK JENIS ZONA",IF(A177="","Zona kosong",IF(B177="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A177="",F177=""),"",IF(F177="","Belum ditempatkan",IF(I177="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G177="","CEK ZONA NO kosong",IF(K177="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H177&lt;&gt;K177,"CEK JENIS ZONA",IF(A177="","Zona STOCK",IF(B177="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8257,7 +8257,7 @@
         <v/>
       </c>
       <c r="M178" s="12">
-        <f>IF(AND(A178="",F178=""),"",IF(F178="","Belum ditempatkan",IF(I178="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G178="","CEK ZONA NO kosong",IF(K178="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H178&lt;&gt;K178,"CEK JENIS ZONA",IF(A178="","Zona kosong",IF(B178="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A178="",F178=""),"",IF(F178="","Belum ditempatkan",IF(I178="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G178="","CEK ZONA NO kosong",IF(K178="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H178&lt;&gt;K178,"CEK JENIS ZONA",IF(A178="","Zona STOCK",IF(B178="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8287,7 +8287,7 @@
         <v/>
       </c>
       <c r="M179" s="12">
-        <f>IF(AND(A179="",F179=""),"",IF(F179="","Belum ditempatkan",IF(I179="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G179="","CEK ZONA NO kosong",IF(K179="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H179&lt;&gt;K179,"CEK JENIS ZONA",IF(A179="","Zona kosong",IF(B179="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A179="",F179=""),"",IF(F179="","Belum ditempatkan",IF(I179="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G179="","CEK ZONA NO kosong",IF(K179="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H179&lt;&gt;K179,"CEK JENIS ZONA",IF(A179="","Zona STOCK",IF(B179="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8317,7 +8317,7 @@
         <v/>
       </c>
       <c r="M180" s="12">
-        <f>IF(AND(A180="",F180=""),"",IF(F180="","Belum ditempatkan",IF(I180="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G180="","CEK ZONA NO kosong",IF(K180="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H180&lt;&gt;K180,"CEK JENIS ZONA",IF(A180="","Zona kosong",IF(B180="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A180="",F180=""),"",IF(F180="","Belum ditempatkan",IF(I180="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G180="","CEK ZONA NO kosong",IF(K180="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H180&lt;&gt;K180,"CEK JENIS ZONA",IF(A180="","Zona STOCK",IF(B180="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8347,7 +8347,7 @@
         <v/>
       </c>
       <c r="M181" s="12">
-        <f>IF(AND(A181="",F181=""),"",IF(F181="","Belum ditempatkan",IF(I181="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G181="","CEK ZONA NO kosong",IF(K181="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H181&lt;&gt;K181,"CEK JENIS ZONA",IF(A181="","Zona kosong",IF(B181="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A181="",F181=""),"",IF(F181="","Belum ditempatkan",IF(I181="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G181="","CEK ZONA NO kosong",IF(K181="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H181&lt;&gt;K181,"CEK JENIS ZONA",IF(A181="","Zona STOCK",IF(B181="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8377,7 +8377,7 @@
         <v/>
       </c>
       <c r="M182" s="12">
-        <f>IF(AND(A182="",F182=""),"",IF(F182="","Belum ditempatkan",IF(I182="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G182="","CEK ZONA NO kosong",IF(K182="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H182&lt;&gt;K182,"CEK JENIS ZONA",IF(A182="","Zona kosong",IF(B182="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A182="",F182=""),"",IF(F182="","Belum ditempatkan",IF(I182="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G182="","CEK ZONA NO kosong",IF(K182="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H182&lt;&gt;K182,"CEK JENIS ZONA",IF(A182="","Zona STOCK",IF(B182="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8407,7 +8407,7 @@
         <v/>
       </c>
       <c r="M183" s="12">
-        <f>IF(AND(A183="",F183=""),"",IF(F183="","Belum ditempatkan",IF(I183="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G183="","CEK ZONA NO kosong",IF(K183="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H183&lt;&gt;K183,"CEK JENIS ZONA",IF(A183="","Zona kosong",IF(B183="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A183="",F183=""),"",IF(F183="","Belum ditempatkan",IF(I183="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G183="","CEK ZONA NO kosong",IF(K183="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H183&lt;&gt;K183,"CEK JENIS ZONA",IF(A183="","Zona STOCK",IF(B183="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8437,7 +8437,7 @@
         <v/>
       </c>
       <c r="M184" s="12">
-        <f>IF(AND(A184="",F184=""),"",IF(F184="","Belum ditempatkan",IF(I184="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G184="","CEK ZONA NO kosong",IF(K184="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H184&lt;&gt;K184,"CEK JENIS ZONA",IF(A184="","Zona kosong",IF(B184="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A184="",F184=""),"",IF(F184="","Belum ditempatkan",IF(I184="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G184="","CEK ZONA NO kosong",IF(K184="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H184&lt;&gt;K184,"CEK JENIS ZONA",IF(A184="","Zona STOCK",IF(B184="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8467,7 +8467,7 @@
         <v/>
       </c>
       <c r="M185" s="12">
-        <f>IF(AND(A185="",F185=""),"",IF(F185="","Belum ditempatkan",IF(I185="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G185="","CEK ZONA NO kosong",IF(K185="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H185&lt;&gt;K185,"CEK JENIS ZONA",IF(A185="","Zona kosong",IF(B185="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A185="",F185=""),"",IF(F185="","Belum ditempatkan",IF(I185="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G185="","CEK ZONA NO kosong",IF(K185="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H185&lt;&gt;K185,"CEK JENIS ZONA",IF(A185="","Zona STOCK",IF(B185="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8497,7 +8497,7 @@
         <v/>
       </c>
       <c r="M186" s="12">
-        <f>IF(AND(A186="",F186=""),"",IF(F186="","Belum ditempatkan",IF(I186="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G186="","CEK ZONA NO kosong",IF(K186="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H186&lt;&gt;K186,"CEK JENIS ZONA",IF(A186="","Zona kosong",IF(B186="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A186="",F186=""),"",IF(F186="","Belum ditempatkan",IF(I186="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G186="","CEK ZONA NO kosong",IF(K186="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H186&lt;&gt;K186,"CEK JENIS ZONA",IF(A186="","Zona STOCK",IF(B186="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8527,7 +8527,7 @@
         <v/>
       </c>
       <c r="M187" s="12">
-        <f>IF(AND(A187="",F187=""),"",IF(F187="","Belum ditempatkan",IF(I187="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G187="","CEK ZONA NO kosong",IF(K187="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H187&lt;&gt;K187,"CEK JENIS ZONA",IF(A187="","Zona kosong",IF(B187="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A187="",F187=""),"",IF(F187="","Belum ditempatkan",IF(I187="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G187="","CEK ZONA NO kosong",IF(K187="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H187&lt;&gt;K187,"CEK JENIS ZONA",IF(A187="","Zona STOCK",IF(B187="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8557,7 +8557,7 @@
         <v/>
       </c>
       <c r="M188" s="12">
-        <f>IF(AND(A188="",F188=""),"",IF(F188="","Belum ditempatkan",IF(I188="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G188="","CEK ZONA NO kosong",IF(K188="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H188&lt;&gt;K188,"CEK JENIS ZONA",IF(A188="","Zona kosong",IF(B188="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A188="",F188=""),"",IF(F188="","Belum ditempatkan",IF(I188="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G188="","CEK ZONA NO kosong",IF(K188="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H188&lt;&gt;K188,"CEK JENIS ZONA",IF(A188="","Zona STOCK",IF(B188="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8587,7 +8587,7 @@
         <v/>
       </c>
       <c r="M189" s="12">
-        <f>IF(AND(A189="",F189=""),"",IF(F189="","Belum ditempatkan",IF(I189="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G189="","CEK ZONA NO kosong",IF(K189="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H189&lt;&gt;K189,"CEK JENIS ZONA",IF(A189="","Zona kosong",IF(B189="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A189="",F189=""),"",IF(F189="","Belum ditempatkan",IF(I189="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G189="","CEK ZONA NO kosong",IF(K189="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H189&lt;&gt;K189,"CEK JENIS ZONA",IF(A189="","Zona STOCK",IF(B189="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8617,7 +8617,7 @@
         <v/>
       </c>
       <c r="M190" s="12">
-        <f>IF(AND(A190="",F190=""),"",IF(F190="","Belum ditempatkan",IF(I190="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G190="","CEK ZONA NO kosong",IF(K190="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H190&lt;&gt;K190,"CEK JENIS ZONA",IF(A190="","Zona kosong",IF(B190="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A190="",F190=""),"",IF(F190="","Belum ditempatkan",IF(I190="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G190="","CEK ZONA NO kosong",IF(K190="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H190&lt;&gt;K190,"CEK JENIS ZONA",IF(A190="","Zona STOCK",IF(B190="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8647,7 +8647,7 @@
         <v/>
       </c>
       <c r="M191" s="12">
-        <f>IF(AND(A191="",F191=""),"",IF(F191="","Belum ditempatkan",IF(I191="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G191="","CEK ZONA NO kosong",IF(K191="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H191&lt;&gt;K191,"CEK JENIS ZONA",IF(A191="","Zona kosong",IF(B191="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A191="",F191=""),"",IF(F191="","Belum ditempatkan",IF(I191="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G191="","CEK ZONA NO kosong",IF(K191="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H191&lt;&gt;K191,"CEK JENIS ZONA",IF(A191="","Zona STOCK",IF(B191="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8677,7 +8677,7 @@
         <v/>
       </c>
       <c r="M192" s="12">
-        <f>IF(AND(A192="",F192=""),"",IF(F192="","Belum ditempatkan",IF(I192="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G192="","CEK ZONA NO kosong",IF(K192="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H192&lt;&gt;K192,"CEK JENIS ZONA",IF(A192="","Zona kosong",IF(B192="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A192="",F192=""),"",IF(F192="","Belum ditempatkan",IF(I192="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G192="","CEK ZONA NO kosong",IF(K192="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H192&lt;&gt;K192,"CEK JENIS ZONA",IF(A192="","Zona STOCK",IF(B192="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8707,7 +8707,7 @@
         <v/>
       </c>
       <c r="M193" s="12">
-        <f>IF(AND(A193="",F193=""),"",IF(F193="","Belum ditempatkan",IF(I193="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G193="","CEK ZONA NO kosong",IF(K193="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H193&lt;&gt;K193,"CEK JENIS ZONA",IF(A193="","Zona kosong",IF(B193="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A193="",F193=""),"",IF(F193="","Belum ditempatkan",IF(I193="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G193="","CEK ZONA NO kosong",IF(K193="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H193&lt;&gt;K193,"CEK JENIS ZONA",IF(A193="","Zona STOCK",IF(B193="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
         <v/>
       </c>
       <c r="M194" s="12">
-        <f>IF(AND(A194="",F194=""),"",IF(F194="","Belum ditempatkan",IF(I194="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G194="","CEK ZONA NO kosong",IF(K194="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H194&lt;&gt;K194,"CEK JENIS ZONA",IF(A194="","Zona kosong",IF(B194="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A194="",F194=""),"",IF(F194="","Belum ditempatkan",IF(I194="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G194="","CEK ZONA NO kosong",IF(K194="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H194&lt;&gt;K194,"CEK JENIS ZONA",IF(A194="","Zona STOCK",IF(B194="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8767,7 +8767,7 @@
         <v/>
       </c>
       <c r="M195" s="12">
-        <f>IF(AND(A195="",F195=""),"",IF(F195="","Belum ditempatkan",IF(I195="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G195="","CEK ZONA NO kosong",IF(K195="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H195&lt;&gt;K195,"CEK JENIS ZONA",IF(A195="","Zona kosong",IF(B195="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A195="",F195=""),"",IF(F195="","Belum ditempatkan",IF(I195="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G195="","CEK ZONA NO kosong",IF(K195="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H195&lt;&gt;K195,"CEK JENIS ZONA",IF(A195="","Zona STOCK",IF(B195="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8797,7 +8797,7 @@
         <v/>
       </c>
       <c r="M196" s="12">
-        <f>IF(AND(A196="",F196=""),"",IF(F196="","Belum ditempatkan",IF(I196="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G196="","CEK ZONA NO kosong",IF(K196="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H196&lt;&gt;K196,"CEK JENIS ZONA",IF(A196="","Zona kosong",IF(B196="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A196="",F196=""),"",IF(F196="","Belum ditempatkan",IF(I196="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G196="","CEK ZONA NO kosong",IF(K196="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H196&lt;&gt;K196,"CEK JENIS ZONA",IF(A196="","Zona STOCK",IF(B196="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8827,7 +8827,7 @@
         <v/>
       </c>
       <c r="M197" s="12">
-        <f>IF(AND(A197="",F197=""),"",IF(F197="","Belum ditempatkan",IF(I197="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G197="","CEK ZONA NO kosong",IF(K197="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H197&lt;&gt;K197,"CEK JENIS ZONA",IF(A197="","Zona kosong",IF(B197="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A197="",F197=""),"",IF(F197="","Belum ditempatkan",IF(I197="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G197="","CEK ZONA NO kosong",IF(K197="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H197&lt;&gt;K197,"CEK JENIS ZONA",IF(A197="","Zona STOCK",IF(B197="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8857,7 +8857,7 @@
         <v/>
       </c>
       <c r="M198" s="12">
-        <f>IF(AND(A198="",F198=""),"",IF(F198="","Belum ditempatkan",IF(I198="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G198="","CEK ZONA NO kosong",IF(K198="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H198&lt;&gt;K198,"CEK JENIS ZONA",IF(A198="","Zona kosong",IF(B198="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A198="",F198=""),"",IF(F198="","Belum ditempatkan",IF(I198="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G198="","CEK ZONA NO kosong",IF(K198="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H198&lt;&gt;K198,"CEK JENIS ZONA",IF(A198="","Zona STOCK",IF(B198="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8887,7 +8887,7 @@
         <v/>
       </c>
       <c r="M199" s="12">
-        <f>IF(AND(A199="",F199=""),"",IF(F199="","Belum ditempatkan",IF(I199="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G199="","CEK ZONA NO kosong",IF(K199="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H199&lt;&gt;K199,"CEK JENIS ZONA",IF(A199="","Zona kosong",IF(B199="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A199="",F199=""),"",IF(F199="","Belum ditempatkan",IF(I199="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G199="","CEK ZONA NO kosong",IF(K199="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H199&lt;&gt;K199,"CEK JENIS ZONA",IF(A199="","Zona STOCK",IF(B199="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8917,7 +8917,7 @@
         <v/>
       </c>
       <c r="M200" s="12">
-        <f>IF(AND(A200="",F200=""),"",IF(F200="","Belum ditempatkan",IF(I200="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G200="","CEK ZONA NO kosong",IF(K200="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H200&lt;&gt;K200,"CEK JENIS ZONA",IF(A200="","Zona kosong",IF(B200="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A200="",F200=""),"",IF(F200="","Belum ditempatkan",IF(I200="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G200="","CEK ZONA NO kosong",IF(K200="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H200&lt;&gt;K200,"CEK JENIS ZONA",IF(A200="","Zona STOCK",IF(B200="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8947,7 +8947,7 @@
         <v/>
       </c>
       <c r="M201" s="12">
-        <f>IF(AND(A201="",F201=""),"",IF(F201="","Belum ditempatkan",IF(I201="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G201="","CEK ZONA NO kosong",IF(K201="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H201&lt;&gt;K201,"CEK JENIS ZONA",IF(A201="","Zona kosong",IF(B201="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A201="",F201=""),"",IF(F201="","Belum ditempatkan",IF(I201="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G201="","CEK ZONA NO kosong",IF(K201="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H201&lt;&gt;K201,"CEK JENIS ZONA",IF(A201="","Zona STOCK",IF(B201="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -8977,7 +8977,7 @@
         <v/>
       </c>
       <c r="M202" s="12">
-        <f>IF(AND(A202="",F202=""),"",IF(F202="","Belum ditempatkan",IF(I202="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G202="","CEK ZONA NO kosong",IF(K202="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H202&lt;&gt;K202,"CEK JENIS ZONA",IF(A202="","Zona kosong",IF(B202="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A202="",F202=""),"",IF(F202="","Belum ditempatkan",IF(I202="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G202="","CEK ZONA NO kosong",IF(K202="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H202&lt;&gt;K202,"CEK JENIS ZONA",IF(A202="","Zona STOCK",IF(B202="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9007,7 +9007,7 @@
         <v/>
       </c>
       <c r="M203" s="12">
-        <f>IF(AND(A203="",F203=""),"",IF(F203="","Belum ditempatkan",IF(I203="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G203="","CEK ZONA NO kosong",IF(K203="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H203&lt;&gt;K203,"CEK JENIS ZONA",IF(A203="","Zona kosong",IF(B203="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A203="",F203=""),"",IF(F203="","Belum ditempatkan",IF(I203="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G203="","CEK ZONA NO kosong",IF(K203="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H203&lt;&gt;K203,"CEK JENIS ZONA",IF(A203="","Zona STOCK",IF(B203="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9037,7 +9037,7 @@
         <v/>
       </c>
       <c r="M204" s="12">
-        <f>IF(AND(A204="",F204=""),"",IF(F204="","Belum ditempatkan",IF(I204="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G204="","CEK ZONA NO kosong",IF(K204="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H204&lt;&gt;K204,"CEK JENIS ZONA",IF(A204="","Zona kosong",IF(B204="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A204="",F204=""),"",IF(F204="","Belum ditempatkan",IF(I204="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G204="","CEK ZONA NO kosong",IF(K204="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H204&lt;&gt;K204,"CEK JENIS ZONA",IF(A204="","Zona STOCK",IF(B204="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9067,7 +9067,7 @@
         <v/>
       </c>
       <c r="M205" s="12">
-        <f>IF(AND(A205="",F205=""),"",IF(F205="","Belum ditempatkan",IF(I205="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G205="","CEK ZONA NO kosong",IF(K205="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H205&lt;&gt;K205,"CEK JENIS ZONA",IF(A205="","Zona kosong",IF(B205="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A205="",F205=""),"",IF(F205="","Belum ditempatkan",IF(I205="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G205="","CEK ZONA NO kosong",IF(K205="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H205&lt;&gt;K205,"CEK JENIS ZONA",IF(A205="","Zona STOCK",IF(B205="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9097,7 +9097,7 @@
         <v/>
       </c>
       <c r="M206" s="12">
-        <f>IF(AND(A206="",F206=""),"",IF(F206="","Belum ditempatkan",IF(I206="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G206="","CEK ZONA NO kosong",IF(K206="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H206&lt;&gt;K206,"CEK JENIS ZONA",IF(A206="","Zona kosong",IF(B206="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A206="",F206=""),"",IF(F206="","Belum ditempatkan",IF(I206="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G206="","CEK ZONA NO kosong",IF(K206="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H206&lt;&gt;K206,"CEK JENIS ZONA",IF(A206="","Zona STOCK",IF(B206="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9127,7 +9127,7 @@
         <v/>
       </c>
       <c r="M207" s="12">
-        <f>IF(AND(A207="",F207=""),"",IF(F207="","Belum ditempatkan",IF(I207="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G207="","CEK ZONA NO kosong",IF(K207="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H207&lt;&gt;K207,"CEK JENIS ZONA",IF(A207="","Zona kosong",IF(B207="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A207="",F207=""),"",IF(F207="","Belum ditempatkan",IF(I207="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G207="","CEK ZONA NO kosong",IF(K207="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H207&lt;&gt;K207,"CEK JENIS ZONA",IF(A207="","Zona STOCK",IF(B207="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9157,7 +9157,7 @@
         <v/>
       </c>
       <c r="M208" s="12">
-        <f>IF(AND(A208="",F208=""),"",IF(F208="","Belum ditempatkan",IF(I208="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G208="","CEK ZONA NO kosong",IF(K208="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H208&lt;&gt;K208,"CEK JENIS ZONA",IF(A208="","Zona kosong",IF(B208="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A208="",F208=""),"",IF(F208="","Belum ditempatkan",IF(I208="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G208="","CEK ZONA NO kosong",IF(K208="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H208&lt;&gt;K208,"CEK JENIS ZONA",IF(A208="","Zona STOCK",IF(B208="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9187,7 +9187,7 @@
         <v/>
       </c>
       <c r="M209" s="12">
-        <f>IF(AND(A209="",F209=""),"",IF(F209="","Belum ditempatkan",IF(I209="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G209="","CEK ZONA NO kosong",IF(K209="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H209&lt;&gt;K209,"CEK JENIS ZONA",IF(A209="","Zona kosong",IF(B209="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A209="",F209=""),"",IF(F209="","Belum ditempatkan",IF(I209="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G209="","CEK ZONA NO kosong",IF(K209="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H209&lt;&gt;K209,"CEK JENIS ZONA",IF(A209="","Zona STOCK",IF(B209="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9217,7 +9217,7 @@
         <v/>
       </c>
       <c r="M210" s="12">
-        <f>IF(AND(A210="",F210=""),"",IF(F210="","Belum ditempatkan",IF(I210="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G210="","CEK ZONA NO kosong",IF(K210="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H210&lt;&gt;K210,"CEK JENIS ZONA",IF(A210="","Zona kosong",IF(B210="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A210="",F210=""),"",IF(F210="","Belum ditempatkan",IF(I210="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G210="","CEK ZONA NO kosong",IF(K210="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H210&lt;&gt;K210,"CEK JENIS ZONA",IF(A210="","Zona STOCK",IF(B210="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9247,7 +9247,7 @@
         <v/>
       </c>
       <c r="M211" s="12">
-        <f>IF(AND(A211="",F211=""),"",IF(F211="","Belum ditempatkan",IF(I211="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G211="","CEK ZONA NO kosong",IF(K211="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H211&lt;&gt;K211,"CEK JENIS ZONA",IF(A211="","Zona kosong",IF(B211="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A211="",F211=""),"",IF(F211="","Belum ditempatkan",IF(I211="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G211="","CEK ZONA NO kosong",IF(K211="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H211&lt;&gt;K211,"CEK JENIS ZONA",IF(A211="","Zona STOCK",IF(B211="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9277,7 +9277,7 @@
         <v/>
       </c>
       <c r="M212" s="12">
-        <f>IF(AND(A212="",F212=""),"",IF(F212="","Belum ditempatkan",IF(I212="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G212="","CEK ZONA NO kosong",IF(K212="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H212&lt;&gt;K212,"CEK JENIS ZONA",IF(A212="","Zona kosong",IF(B212="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A212="",F212=""),"",IF(F212="","Belum ditempatkan",IF(I212="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G212="","CEK ZONA NO kosong",IF(K212="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H212&lt;&gt;K212,"CEK JENIS ZONA",IF(A212="","Zona STOCK",IF(B212="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9307,7 +9307,7 @@
         <v/>
       </c>
       <c r="M213" s="12">
-        <f>IF(AND(A213="",F213=""),"",IF(F213="","Belum ditempatkan",IF(I213="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G213="","CEK ZONA NO kosong",IF(K213="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H213&lt;&gt;K213,"CEK JENIS ZONA",IF(A213="","Zona kosong",IF(B213="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A213="",F213=""),"",IF(F213="","Belum ditempatkan",IF(I213="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G213="","CEK ZONA NO kosong",IF(K213="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H213&lt;&gt;K213,"CEK JENIS ZONA",IF(A213="","Zona STOCK",IF(B213="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9337,7 +9337,7 @@
         <v/>
       </c>
       <c r="M214" s="12">
-        <f>IF(AND(A214="",F214=""),"",IF(F214="","Belum ditempatkan",IF(I214="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G214="","CEK ZONA NO kosong",IF(K214="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H214&lt;&gt;K214,"CEK JENIS ZONA",IF(A214="","Zona kosong",IF(B214="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A214="",F214=""),"",IF(F214="","Belum ditempatkan",IF(I214="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G214="","CEK ZONA NO kosong",IF(K214="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H214&lt;&gt;K214,"CEK JENIS ZONA",IF(A214="","Zona STOCK",IF(B214="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9367,7 +9367,7 @@
         <v/>
       </c>
       <c r="M215" s="12">
-        <f>IF(AND(A215="",F215=""),"",IF(F215="","Belum ditempatkan",IF(I215="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G215="","CEK ZONA NO kosong",IF(K215="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H215&lt;&gt;K215,"CEK JENIS ZONA",IF(A215="","Zona kosong",IF(B215="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A215="",F215=""),"",IF(F215="","Belum ditempatkan",IF(I215="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G215="","CEK ZONA NO kosong",IF(K215="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H215&lt;&gt;K215,"CEK JENIS ZONA",IF(A215="","Zona STOCK",IF(B215="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9397,7 +9397,7 @@
         <v/>
       </c>
       <c r="M216" s="12">
-        <f>IF(AND(A216="",F216=""),"",IF(F216="","Belum ditempatkan",IF(I216="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G216="","CEK ZONA NO kosong",IF(K216="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H216&lt;&gt;K216,"CEK JENIS ZONA",IF(A216="","Zona kosong",IF(B216="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A216="",F216=""),"",IF(F216="","Belum ditempatkan",IF(I216="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G216="","CEK ZONA NO kosong",IF(K216="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H216&lt;&gt;K216,"CEK JENIS ZONA",IF(A216="","Zona STOCK",IF(B216="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9427,7 +9427,7 @@
         <v/>
       </c>
       <c r="M217" s="12">
-        <f>IF(AND(A217="",F217=""),"",IF(F217="","Belum ditempatkan",IF(I217="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G217="","CEK ZONA NO kosong",IF(K217="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H217&lt;&gt;K217,"CEK JENIS ZONA",IF(A217="","Zona kosong",IF(B217="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A217="",F217=""),"",IF(F217="","Belum ditempatkan",IF(I217="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G217="","CEK ZONA NO kosong",IF(K217="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H217&lt;&gt;K217,"CEK JENIS ZONA",IF(A217="","Zona STOCK",IF(B217="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9457,7 +9457,7 @@
         <v/>
       </c>
       <c r="M218" s="12">
-        <f>IF(AND(A218="",F218=""),"",IF(F218="","Belum ditempatkan",IF(I218="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G218="","CEK ZONA NO kosong",IF(K218="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H218&lt;&gt;K218,"CEK JENIS ZONA",IF(A218="","Zona kosong",IF(B218="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A218="",F218=""),"",IF(F218="","Belum ditempatkan",IF(I218="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G218="","CEK ZONA NO kosong",IF(K218="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H218&lt;&gt;K218,"CEK JENIS ZONA",IF(A218="","Zona STOCK",IF(B218="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9487,7 +9487,7 @@
         <v/>
       </c>
       <c r="M219" s="12">
-        <f>IF(AND(A219="",F219=""),"",IF(F219="","Belum ditempatkan",IF(I219="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G219="","CEK ZONA NO kosong",IF(K219="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H219&lt;&gt;K219,"CEK JENIS ZONA",IF(A219="","Zona kosong",IF(B219="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A219="",F219=""),"",IF(F219="","Belum ditempatkan",IF(I219="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G219="","CEK ZONA NO kosong",IF(K219="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H219&lt;&gt;K219,"CEK JENIS ZONA",IF(A219="","Zona STOCK",IF(B219="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9517,7 +9517,7 @@
         <v/>
       </c>
       <c r="M220" s="12">
-        <f>IF(AND(A220="",F220=""),"",IF(F220="","Belum ditempatkan",IF(I220="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G220="","CEK ZONA NO kosong",IF(K220="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H220&lt;&gt;K220,"CEK JENIS ZONA",IF(A220="","Zona kosong",IF(B220="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A220="",F220=""),"",IF(F220="","Belum ditempatkan",IF(I220="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G220="","CEK ZONA NO kosong",IF(K220="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H220&lt;&gt;K220,"CEK JENIS ZONA",IF(A220="","Zona STOCK",IF(B220="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9547,7 +9547,7 @@
         <v/>
       </c>
       <c r="M221" s="12">
-        <f>IF(AND(A221="",F221=""),"",IF(F221="","Belum ditempatkan",IF(I221="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G221="","CEK ZONA NO kosong",IF(K221="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H221&lt;&gt;K221,"CEK JENIS ZONA",IF(A221="","Zona kosong",IF(B221="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A221="",F221=""),"",IF(F221="","Belum ditempatkan",IF(I221="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G221="","CEK ZONA NO kosong",IF(K221="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H221&lt;&gt;K221,"CEK JENIS ZONA",IF(A221="","Zona STOCK",IF(B221="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9577,7 +9577,7 @@
         <v/>
       </c>
       <c r="M222" s="12">
-        <f>IF(AND(A222="",F222=""),"",IF(F222="","Belum ditempatkan",IF(I222="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G222="","CEK ZONA NO kosong",IF(K222="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H222&lt;&gt;K222,"CEK JENIS ZONA",IF(A222="","Zona kosong",IF(B222="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A222="",F222=""),"",IF(F222="","Belum ditempatkan",IF(I222="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G222="","CEK ZONA NO kosong",IF(K222="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H222&lt;&gt;K222,"CEK JENIS ZONA",IF(A222="","Zona STOCK",IF(B222="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9607,7 +9607,7 @@
         <v/>
       </c>
       <c r="M223" s="12">
-        <f>IF(AND(A223="",F223=""),"",IF(F223="","Belum ditempatkan",IF(I223="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G223="","CEK ZONA NO kosong",IF(K223="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H223&lt;&gt;K223,"CEK JENIS ZONA",IF(A223="","Zona kosong",IF(B223="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A223="",F223=""),"",IF(F223="","Belum ditempatkan",IF(I223="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G223="","CEK ZONA NO kosong",IF(K223="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H223&lt;&gt;K223,"CEK JENIS ZONA",IF(A223="","Zona STOCK",IF(B223="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9637,7 +9637,7 @@
         <v/>
       </c>
       <c r="M224" s="12">
-        <f>IF(AND(A224="",F224=""),"",IF(F224="","Belum ditempatkan",IF(I224="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G224="","CEK ZONA NO kosong",IF(K224="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H224&lt;&gt;K224,"CEK JENIS ZONA",IF(A224="","Zona kosong",IF(B224="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A224="",F224=""),"",IF(F224="","Belum ditempatkan",IF(I224="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G224="","CEK ZONA NO kosong",IF(K224="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H224&lt;&gt;K224,"CEK JENIS ZONA",IF(A224="","Zona STOCK",IF(B224="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
         <v/>
       </c>
       <c r="M225" s="12">
-        <f>IF(AND(A225="",F225=""),"",IF(F225="","Belum ditempatkan",IF(I225="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G225="","CEK ZONA NO kosong",IF(K225="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H225&lt;&gt;K225,"CEK JENIS ZONA",IF(A225="","Zona kosong",IF(B225="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A225="",F225=""),"",IF(F225="","Belum ditempatkan",IF(I225="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G225="","CEK ZONA NO kosong",IF(K225="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H225&lt;&gt;K225,"CEK JENIS ZONA",IF(A225="","Zona STOCK",IF(B225="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9697,7 +9697,7 @@
         <v/>
       </c>
       <c r="M226" s="12">
-        <f>IF(AND(A226="",F226=""),"",IF(F226="","Belum ditempatkan",IF(I226="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G226="","CEK ZONA NO kosong",IF(K226="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H226&lt;&gt;K226,"CEK JENIS ZONA",IF(A226="","Zona kosong",IF(B226="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A226="",F226=""),"",IF(F226="","Belum ditempatkan",IF(I226="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G226="","CEK ZONA NO kosong",IF(K226="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H226&lt;&gt;K226,"CEK JENIS ZONA",IF(A226="","Zona STOCK",IF(B226="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9727,7 +9727,7 @@
         <v/>
       </c>
       <c r="M227" s="12">
-        <f>IF(AND(A227="",F227=""),"",IF(F227="","Belum ditempatkan",IF(I227="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G227="","CEK ZONA NO kosong",IF(K227="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H227&lt;&gt;K227,"CEK JENIS ZONA",IF(A227="","Zona kosong",IF(B227="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A227="",F227=""),"",IF(F227="","Belum ditempatkan",IF(I227="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G227="","CEK ZONA NO kosong",IF(K227="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H227&lt;&gt;K227,"CEK JENIS ZONA",IF(A227="","Zona STOCK",IF(B227="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9757,7 +9757,7 @@
         <v/>
       </c>
       <c r="M228" s="12">
-        <f>IF(AND(A228="",F228=""),"",IF(F228="","Belum ditempatkan",IF(I228="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G228="","CEK ZONA NO kosong",IF(K228="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H228&lt;&gt;K228,"CEK JENIS ZONA",IF(A228="","Zona kosong",IF(B228="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A228="",F228=""),"",IF(F228="","Belum ditempatkan",IF(I228="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G228="","CEK ZONA NO kosong",IF(K228="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H228&lt;&gt;K228,"CEK JENIS ZONA",IF(A228="","Zona STOCK",IF(B228="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9787,7 +9787,7 @@
         <v/>
       </c>
       <c r="M229" s="12">
-        <f>IF(AND(A229="",F229=""),"",IF(F229="","Belum ditempatkan",IF(I229="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G229="","CEK ZONA NO kosong",IF(K229="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H229&lt;&gt;K229,"CEK JENIS ZONA",IF(A229="","Zona kosong",IF(B229="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A229="",F229=""),"",IF(F229="","Belum ditempatkan",IF(I229="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G229="","CEK ZONA NO kosong",IF(K229="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H229&lt;&gt;K229,"CEK JENIS ZONA",IF(A229="","Zona STOCK",IF(B229="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9817,7 +9817,7 @@
         <v/>
       </c>
       <c r="M230" s="12">
-        <f>IF(AND(A230="",F230=""),"",IF(F230="","Belum ditempatkan",IF(I230="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G230="","CEK ZONA NO kosong",IF(K230="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H230&lt;&gt;K230,"CEK JENIS ZONA",IF(A230="","Zona kosong",IF(B230="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A230="",F230=""),"",IF(F230="","Belum ditempatkan",IF(I230="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G230="","CEK ZONA NO kosong",IF(K230="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H230&lt;&gt;K230,"CEK JENIS ZONA",IF(A230="","Zona STOCK",IF(B230="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
         <v/>
       </c>
       <c r="M231" s="12">
-        <f>IF(AND(A231="",F231=""),"",IF(F231="","Belum ditempatkan",IF(I231="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G231="","CEK ZONA NO kosong",IF(K231="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H231&lt;&gt;K231,"CEK JENIS ZONA",IF(A231="","Zona kosong",IF(B231="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A231="",F231=""),"",IF(F231="","Belum ditempatkan",IF(I231="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G231="","CEK ZONA NO kosong",IF(K231="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H231&lt;&gt;K231,"CEK JENIS ZONA",IF(A231="","Zona STOCK",IF(B231="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9877,7 +9877,7 @@
         <v/>
       </c>
       <c r="M232" s="12">
-        <f>IF(AND(A232="",F232=""),"",IF(F232="","Belum ditempatkan",IF(I232="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G232="","CEK ZONA NO kosong",IF(K232="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H232&lt;&gt;K232,"CEK JENIS ZONA",IF(A232="","Zona kosong",IF(B232="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A232="",F232=""),"",IF(F232="","Belum ditempatkan",IF(I232="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G232="","CEK ZONA NO kosong",IF(K232="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H232&lt;&gt;K232,"CEK JENIS ZONA",IF(A232="","Zona STOCK",IF(B232="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9907,7 +9907,7 @@
         <v/>
       </c>
       <c r="M233" s="12">
-        <f>IF(AND(A233="",F233=""),"",IF(F233="","Belum ditempatkan",IF(I233="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G233="","CEK ZONA NO kosong",IF(K233="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H233&lt;&gt;K233,"CEK JENIS ZONA",IF(A233="","Zona kosong",IF(B233="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A233="",F233=""),"",IF(F233="","Belum ditempatkan",IF(I233="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G233="","CEK ZONA NO kosong",IF(K233="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H233&lt;&gt;K233,"CEK JENIS ZONA",IF(A233="","Zona STOCK",IF(B233="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9937,7 +9937,7 @@
         <v/>
       </c>
       <c r="M234" s="12">
-        <f>IF(AND(A234="",F234=""),"",IF(F234="","Belum ditempatkan",IF(I234="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G234="","CEK ZONA NO kosong",IF(K234="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H234&lt;&gt;K234,"CEK JENIS ZONA",IF(A234="","Zona kosong",IF(B234="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A234="",F234=""),"",IF(F234="","Belum ditempatkan",IF(I234="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G234="","CEK ZONA NO kosong",IF(K234="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H234&lt;&gt;K234,"CEK JENIS ZONA",IF(A234="","Zona STOCK",IF(B234="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9967,7 +9967,7 @@
         <v/>
       </c>
       <c r="M235" s="12">
-        <f>IF(AND(A235="",F235=""),"",IF(F235="","Belum ditempatkan",IF(I235="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G235="","CEK ZONA NO kosong",IF(K235="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H235&lt;&gt;K235,"CEK JENIS ZONA",IF(A235="","Zona kosong",IF(B235="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A235="",F235=""),"",IF(F235="","Belum ditempatkan",IF(I235="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G235="","CEK ZONA NO kosong",IF(K235="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H235&lt;&gt;K235,"CEK JENIS ZONA",IF(A235="","Zona STOCK",IF(B235="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
         <v/>
       </c>
       <c r="M236" s="12">
-        <f>IF(AND(A236="",F236=""),"",IF(F236="","Belum ditempatkan",IF(I236="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G236="","CEK ZONA NO kosong",IF(K236="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H236&lt;&gt;K236,"CEK JENIS ZONA",IF(A236="","Zona kosong",IF(B236="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A236="",F236=""),"",IF(F236="","Belum ditempatkan",IF(I236="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G236="","CEK ZONA NO kosong",IF(K236="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H236&lt;&gt;K236,"CEK JENIS ZONA",IF(A236="","Zona STOCK",IF(B236="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10027,7 +10027,7 @@
         <v/>
       </c>
       <c r="M237" s="12">
-        <f>IF(AND(A237="",F237=""),"",IF(F237="","Belum ditempatkan",IF(I237="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G237="","CEK ZONA NO kosong",IF(K237="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H237&lt;&gt;K237,"CEK JENIS ZONA",IF(A237="","Zona kosong",IF(B237="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A237="",F237=""),"",IF(F237="","Belum ditempatkan",IF(I237="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G237="","CEK ZONA NO kosong",IF(K237="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H237&lt;&gt;K237,"CEK JENIS ZONA",IF(A237="","Zona STOCK",IF(B237="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10057,7 +10057,7 @@
         <v/>
       </c>
       <c r="M238" s="12">
-        <f>IF(AND(A238="",F238=""),"",IF(F238="","Belum ditempatkan",IF(I238="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G238="","CEK ZONA NO kosong",IF(K238="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H238&lt;&gt;K238,"CEK JENIS ZONA",IF(A238="","Zona kosong",IF(B238="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A238="",F238=""),"",IF(F238="","Belum ditempatkan",IF(I238="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G238="","CEK ZONA NO kosong",IF(K238="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H238&lt;&gt;K238,"CEK JENIS ZONA",IF(A238="","Zona STOCK",IF(B238="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10087,7 +10087,7 @@
         <v/>
       </c>
       <c r="M239" s="12">
-        <f>IF(AND(A239="",F239=""),"",IF(F239="","Belum ditempatkan",IF(I239="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G239="","CEK ZONA NO kosong",IF(K239="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H239&lt;&gt;K239,"CEK JENIS ZONA",IF(A239="","Zona kosong",IF(B239="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A239="",F239=""),"",IF(F239="","Belum ditempatkan",IF(I239="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G239="","CEK ZONA NO kosong",IF(K239="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H239&lt;&gt;K239,"CEK JENIS ZONA",IF(A239="","Zona STOCK",IF(B239="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10117,7 +10117,7 @@
         <v/>
       </c>
       <c r="M240" s="12">
-        <f>IF(AND(A240="",F240=""),"",IF(F240="","Belum ditempatkan",IF(I240="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G240="","CEK ZONA NO kosong",IF(K240="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H240&lt;&gt;K240,"CEK JENIS ZONA",IF(A240="","Zona kosong",IF(B240="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A240="",F240=""),"",IF(F240="","Belum ditempatkan",IF(I240="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G240="","CEK ZONA NO kosong",IF(K240="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H240&lt;&gt;K240,"CEK JENIS ZONA",IF(A240="","Zona STOCK",IF(B240="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10147,7 +10147,7 @@
         <v/>
       </c>
       <c r="M241" s="12">
-        <f>IF(AND(A241="",F241=""),"",IF(F241="","Belum ditempatkan",IF(I241="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G241="","CEK ZONA NO kosong",IF(K241="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H241&lt;&gt;K241,"CEK JENIS ZONA",IF(A241="","Zona kosong",IF(B241="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A241="",F241=""),"",IF(F241="","Belum ditempatkan",IF(I241="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G241="","CEK ZONA NO kosong",IF(K241="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H241&lt;&gt;K241,"CEK JENIS ZONA",IF(A241="","Zona STOCK",IF(B241="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10177,7 +10177,7 @@
         <v/>
       </c>
       <c r="M242" s="12">
-        <f>IF(AND(A242="",F242=""),"",IF(F242="","Belum ditempatkan",IF(I242="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G242="","CEK ZONA NO kosong",IF(K242="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H242&lt;&gt;K242,"CEK JENIS ZONA",IF(A242="","Zona kosong",IF(B242="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A242="",F242=""),"",IF(F242="","Belum ditempatkan",IF(I242="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G242="","CEK ZONA NO kosong",IF(K242="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H242&lt;&gt;K242,"CEK JENIS ZONA",IF(A242="","Zona STOCK",IF(B242="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10207,7 +10207,7 @@
         <v/>
       </c>
       <c r="M243" s="12">
-        <f>IF(AND(A243="",F243=""),"",IF(F243="","Belum ditempatkan",IF(I243="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G243="","CEK ZONA NO kosong",IF(K243="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H243&lt;&gt;K243,"CEK JENIS ZONA",IF(A243="","Zona kosong",IF(B243="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A243="",F243=""),"",IF(F243="","Belum ditempatkan",IF(I243="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G243="","CEK ZONA NO kosong",IF(K243="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H243&lt;&gt;K243,"CEK JENIS ZONA",IF(A243="","Zona STOCK",IF(B243="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10237,7 +10237,7 @@
         <v/>
       </c>
       <c r="M244" s="12">
-        <f>IF(AND(A244="",F244=""),"",IF(F244="","Belum ditempatkan",IF(I244="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G244="","CEK ZONA NO kosong",IF(K244="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H244&lt;&gt;K244,"CEK JENIS ZONA",IF(A244="","Zona kosong",IF(B244="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A244="",F244=""),"",IF(F244="","Belum ditempatkan",IF(I244="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G244="","CEK ZONA NO kosong",IF(K244="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H244&lt;&gt;K244,"CEK JENIS ZONA",IF(A244="","Zona STOCK",IF(B244="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10267,7 +10267,7 @@
         <v/>
       </c>
       <c r="M245" s="12">
-        <f>IF(AND(A245="",F245=""),"",IF(F245="","Belum ditempatkan",IF(I245="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G245="","CEK ZONA NO kosong",IF(K245="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H245&lt;&gt;K245,"CEK JENIS ZONA",IF(A245="","Zona kosong",IF(B245="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A245="",F245=""),"",IF(F245="","Belum ditempatkan",IF(I245="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G245="","CEK ZONA NO kosong",IF(K245="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H245&lt;&gt;K245,"CEK JENIS ZONA",IF(A245="","Zona STOCK",IF(B245="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10297,7 +10297,7 @@
         <v/>
       </c>
       <c r="M246" s="12">
-        <f>IF(AND(A246="",F246=""),"",IF(F246="","Belum ditempatkan",IF(I246="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G246="","CEK ZONA NO kosong",IF(K246="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H246&lt;&gt;K246,"CEK JENIS ZONA",IF(A246="","Zona kosong",IF(B246="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A246="",F246=""),"",IF(F246="","Belum ditempatkan",IF(I246="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G246="","CEK ZONA NO kosong",IF(K246="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H246&lt;&gt;K246,"CEK JENIS ZONA",IF(A246="","Zona STOCK",IF(B246="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10327,7 +10327,7 @@
         <v/>
       </c>
       <c r="M247" s="12">
-        <f>IF(AND(A247="",F247=""),"",IF(F247="","Belum ditempatkan",IF(I247="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G247="","CEK ZONA NO kosong",IF(K247="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H247&lt;&gt;K247,"CEK JENIS ZONA",IF(A247="","Zona kosong",IF(B247="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A247="",F247=""),"",IF(F247="","Belum ditempatkan",IF(I247="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G247="","CEK ZONA NO kosong",IF(K247="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H247&lt;&gt;K247,"CEK JENIS ZONA",IF(A247="","Zona STOCK",IF(B247="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10357,7 +10357,7 @@
         <v/>
       </c>
       <c r="M248" s="12">
-        <f>IF(AND(A248="",F248=""),"",IF(F248="","Belum ditempatkan",IF(I248="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G248="","CEK ZONA NO kosong",IF(K248="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H248&lt;&gt;K248,"CEK JENIS ZONA",IF(A248="","Zona kosong",IF(B248="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A248="",F248=""),"",IF(F248="","Belum ditempatkan",IF(I248="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G248="","CEK ZONA NO kosong",IF(K248="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H248&lt;&gt;K248,"CEK JENIS ZONA",IF(A248="","Zona STOCK",IF(B248="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10387,7 +10387,7 @@
         <v/>
       </c>
       <c r="M249" s="12">
-        <f>IF(AND(A249="",F249=""),"",IF(F249="","Belum ditempatkan",IF(I249="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G249="","CEK ZONA NO kosong",IF(K249="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H249&lt;&gt;K249,"CEK JENIS ZONA",IF(A249="","Zona kosong",IF(B249="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A249="",F249=""),"",IF(F249="","Belum ditempatkan",IF(I249="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G249="","CEK ZONA NO kosong",IF(K249="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H249&lt;&gt;K249,"CEK JENIS ZONA",IF(A249="","Zona STOCK",IF(B249="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10417,7 +10417,7 @@
         <v/>
       </c>
       <c r="M250" s="12">
-        <f>IF(AND(A250="",F250=""),"",IF(F250="","Belum ditempatkan",IF(I250="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G250="","CEK ZONA NO kosong",IF(K250="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H250&lt;&gt;K250,"CEK JENIS ZONA",IF(A250="","Zona kosong",IF(B250="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A250="",F250=""),"",IF(F250="","Belum ditempatkan",IF(I250="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G250="","CEK ZONA NO kosong",IF(K250="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H250&lt;&gt;K250,"CEK JENIS ZONA",IF(A250="","Zona STOCK",IF(B250="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10447,7 +10447,7 @@
         <v/>
       </c>
       <c r="M251" s="12">
-        <f>IF(AND(A251="",F251=""),"",IF(F251="","Belum ditempatkan",IF(I251="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G251="","CEK ZONA NO kosong",IF(K251="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H251&lt;&gt;K251,"CEK JENIS ZONA",IF(A251="","Zona kosong",IF(B251="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A251="",F251=""),"",IF(F251="","Belum ditempatkan",IF(I251="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G251="","CEK ZONA NO kosong",IF(K251="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H251&lt;&gt;K251,"CEK JENIS ZONA",IF(A251="","Zona STOCK",IF(B251="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10477,7 +10477,7 @@
         <v/>
       </c>
       <c r="M252" s="12">
-        <f>IF(AND(A252="",F252=""),"",IF(F252="","Belum ditempatkan",IF(I252="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G252="","CEK ZONA NO kosong",IF(K252="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H252&lt;&gt;K252,"CEK JENIS ZONA",IF(A252="","Zona kosong",IF(B252="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A252="",F252=""),"",IF(F252="","Belum ditempatkan",IF(I252="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G252="","CEK ZONA NO kosong",IF(K252="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H252&lt;&gt;K252,"CEK JENIS ZONA",IF(A252="","Zona STOCK",IF(B252="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10507,7 +10507,7 @@
         <v/>
       </c>
       <c r="M253" s="12">
-        <f>IF(AND(A253="",F253=""),"",IF(F253="","Belum ditempatkan",IF(I253="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G253="","CEK ZONA NO kosong",IF(K253="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H253&lt;&gt;K253,"CEK JENIS ZONA",IF(A253="","Zona kosong",IF(B253="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A253="",F253=""),"",IF(F253="","Belum ditempatkan",IF(I253="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G253="","CEK ZONA NO kosong",IF(K253="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H253&lt;&gt;K253,"CEK JENIS ZONA",IF(A253="","Zona STOCK",IF(B253="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10537,7 +10537,7 @@
         <v/>
       </c>
       <c r="M254" s="12">
-        <f>IF(AND(A254="",F254=""),"",IF(F254="","Belum ditempatkan",IF(I254="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G254="","CEK ZONA NO kosong",IF(K254="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H254&lt;&gt;K254,"CEK JENIS ZONA",IF(A254="","Zona kosong",IF(B254="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A254="",F254=""),"",IF(F254="","Belum ditempatkan",IF(I254="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G254="","CEK ZONA NO kosong",IF(K254="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H254&lt;&gt;K254,"CEK JENIS ZONA",IF(A254="","Zona STOCK",IF(B254="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10567,7 +10567,7 @@
         <v/>
       </c>
       <c r="M255" s="12">
-        <f>IF(AND(A255="",F255=""),"",IF(F255="","Belum ditempatkan",IF(I255="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G255="","CEK ZONA NO kosong",IF(K255="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H255&lt;&gt;K255,"CEK JENIS ZONA",IF(A255="","Zona kosong",IF(B255="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A255="",F255=""),"",IF(F255="","Belum ditempatkan",IF(I255="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G255="","CEK ZONA NO kosong",IF(K255="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H255&lt;&gt;K255,"CEK JENIS ZONA",IF(A255="","Zona STOCK",IF(B255="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10597,7 +10597,7 @@
         <v/>
       </c>
       <c r="M256" s="12">
-        <f>IF(AND(A256="",F256=""),"",IF(F256="","Belum ditempatkan",IF(I256="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G256="","CEK ZONA NO kosong",IF(K256="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H256&lt;&gt;K256,"CEK JENIS ZONA",IF(A256="","Zona kosong",IF(B256="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A256="",F256=""),"",IF(F256="","Belum ditempatkan",IF(I256="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G256="","CEK ZONA NO kosong",IF(K256="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H256&lt;&gt;K256,"CEK JENIS ZONA",IF(A256="","Zona STOCK",IF(B256="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10627,7 +10627,7 @@
         <v/>
       </c>
       <c r="M257" s="12">
-        <f>IF(AND(A257="",F257=""),"",IF(F257="","Belum ditempatkan",IF(I257="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G257="","CEK ZONA NO kosong",IF(K257="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H257&lt;&gt;K257,"CEK JENIS ZONA",IF(A257="","Zona kosong",IF(B257="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A257="",F257=""),"",IF(F257="","Belum ditempatkan",IF(I257="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G257="","CEK ZONA NO kosong",IF(K257="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H257&lt;&gt;K257,"CEK JENIS ZONA",IF(A257="","Zona STOCK",IF(B257="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10657,7 +10657,7 @@
         <v/>
       </c>
       <c r="M258" s="12">
-        <f>IF(AND(A258="",F258=""),"",IF(F258="","Belum ditempatkan",IF(I258="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G258="","CEK ZONA NO kosong",IF(K258="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H258&lt;&gt;K258,"CEK JENIS ZONA",IF(A258="","Zona kosong",IF(B258="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A258="",F258=""),"",IF(F258="","Belum ditempatkan",IF(I258="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G258="","CEK ZONA NO kosong",IF(K258="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H258&lt;&gt;K258,"CEK JENIS ZONA",IF(A258="","Zona STOCK",IF(B258="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10687,7 +10687,7 @@
         <v/>
       </c>
       <c r="M259" s="12">
-        <f>IF(AND(A259="",F259=""),"",IF(F259="","Belum ditempatkan",IF(I259="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G259="","CEK ZONA NO kosong",IF(K259="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H259&lt;&gt;K259,"CEK JENIS ZONA",IF(A259="","Zona kosong",IF(B259="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A259="",F259=""),"",IF(F259="","Belum ditempatkan",IF(I259="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G259="","CEK ZONA NO kosong",IF(K259="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H259&lt;&gt;K259,"CEK JENIS ZONA",IF(A259="","Zona STOCK",IF(B259="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10717,7 +10717,7 @@
         <v/>
       </c>
       <c r="M260" s="12">
-        <f>IF(AND(A260="",F260=""),"",IF(F260="","Belum ditempatkan",IF(I260="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G260="","CEK ZONA NO kosong",IF(K260="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H260&lt;&gt;K260,"CEK JENIS ZONA",IF(A260="","Zona kosong",IF(B260="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A260="",F260=""),"",IF(F260="","Belum ditempatkan",IF(I260="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G260="","CEK ZONA NO kosong",IF(K260="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H260&lt;&gt;K260,"CEK JENIS ZONA",IF(A260="","Zona STOCK",IF(B260="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10747,7 +10747,7 @@
         <v/>
       </c>
       <c r="M261" s="12">
-        <f>IF(AND(A261="",F261=""),"",IF(F261="","Belum ditempatkan",IF(I261="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G261="","CEK ZONA NO kosong",IF(K261="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H261&lt;&gt;K261,"CEK JENIS ZONA",IF(A261="","Zona kosong",IF(B261="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A261="",F261=""),"",IF(F261="","Belum ditempatkan",IF(I261="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G261="","CEK ZONA NO kosong",IF(K261="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H261&lt;&gt;K261,"CEK JENIS ZONA",IF(A261="","Zona STOCK",IF(B261="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10777,7 +10777,7 @@
         <v/>
       </c>
       <c r="M262" s="12">
-        <f>IF(AND(A262="",F262=""),"",IF(F262="","Belum ditempatkan",IF(I262="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G262="","CEK ZONA NO kosong",IF(K262="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H262&lt;&gt;K262,"CEK JENIS ZONA",IF(A262="","Zona kosong",IF(B262="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A262="",F262=""),"",IF(F262="","Belum ditempatkan",IF(I262="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G262="","CEK ZONA NO kosong",IF(K262="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H262&lt;&gt;K262,"CEK JENIS ZONA",IF(A262="","Zona STOCK",IF(B262="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10807,7 +10807,7 @@
         <v/>
       </c>
       <c r="M263" s="12">
-        <f>IF(AND(A263="",F263=""),"",IF(F263="","Belum ditempatkan",IF(I263="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G263="","CEK ZONA NO kosong",IF(K263="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H263&lt;&gt;K263,"CEK JENIS ZONA",IF(A263="","Zona kosong",IF(B263="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A263="",F263=""),"",IF(F263="","Belum ditempatkan",IF(I263="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G263="","CEK ZONA NO kosong",IF(K263="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H263&lt;&gt;K263,"CEK JENIS ZONA",IF(A263="","Zona STOCK",IF(B263="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10837,7 +10837,7 @@
         <v/>
       </c>
       <c r="M264" s="12">
-        <f>IF(AND(A264="",F264=""),"",IF(F264="","Belum ditempatkan",IF(I264="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G264="","CEK ZONA NO kosong",IF(K264="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H264&lt;&gt;K264,"CEK JENIS ZONA",IF(A264="","Zona kosong",IF(B264="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A264="",F264=""),"",IF(F264="","Belum ditempatkan",IF(I264="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G264="","CEK ZONA NO kosong",IF(K264="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H264&lt;&gt;K264,"CEK JENIS ZONA",IF(A264="","Zona STOCK",IF(B264="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10867,7 +10867,7 @@
         <v/>
       </c>
       <c r="M265" s="12">
-        <f>IF(AND(A265="",F265=""),"",IF(F265="","Belum ditempatkan",IF(I265="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G265="","CEK ZONA NO kosong",IF(K265="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H265&lt;&gt;K265,"CEK JENIS ZONA",IF(A265="","Zona kosong",IF(B265="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A265="",F265=""),"",IF(F265="","Belum ditempatkan",IF(I265="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G265="","CEK ZONA NO kosong",IF(K265="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H265&lt;&gt;K265,"CEK JENIS ZONA",IF(A265="","Zona STOCK",IF(B265="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10897,7 +10897,7 @@
         <v/>
       </c>
       <c r="M266" s="12">
-        <f>IF(AND(A266="",F266=""),"",IF(F266="","Belum ditempatkan",IF(I266="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G266="","CEK ZONA NO kosong",IF(K266="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H266&lt;&gt;K266,"CEK JENIS ZONA",IF(A266="","Zona kosong",IF(B266="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A266="",F266=""),"",IF(F266="","Belum ditempatkan",IF(I266="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G266="","CEK ZONA NO kosong",IF(K266="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H266&lt;&gt;K266,"CEK JENIS ZONA",IF(A266="","Zona STOCK",IF(B266="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10927,7 +10927,7 @@
         <v/>
       </c>
       <c r="M267" s="12">
-        <f>IF(AND(A267="",F267=""),"",IF(F267="","Belum ditempatkan",IF(I267="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G267="","CEK ZONA NO kosong",IF(K267="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H267&lt;&gt;K267,"CEK JENIS ZONA",IF(A267="","Zona kosong",IF(B267="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A267="",F267=""),"",IF(F267="","Belum ditempatkan",IF(I267="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G267="","CEK ZONA NO kosong",IF(K267="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H267&lt;&gt;K267,"CEK JENIS ZONA",IF(A267="","Zona STOCK",IF(B267="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10957,7 +10957,7 @@
         <v/>
       </c>
       <c r="M268" s="12">
-        <f>IF(AND(A268="",F268=""),"",IF(F268="","Belum ditempatkan",IF(I268="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G268="","CEK ZONA NO kosong",IF(K268="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H268&lt;&gt;K268,"CEK JENIS ZONA",IF(A268="","Zona kosong",IF(B268="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A268="",F268=""),"",IF(F268="","Belum ditempatkan",IF(I268="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G268="","CEK ZONA NO kosong",IF(K268="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H268&lt;&gt;K268,"CEK JENIS ZONA",IF(A268="","Zona STOCK",IF(B268="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -10987,7 +10987,7 @@
         <v/>
       </c>
       <c r="M269" s="12">
-        <f>IF(AND(A269="",F269=""),"",IF(F269="","Belum ditempatkan",IF(I269="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G269="","CEK ZONA NO kosong",IF(K269="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H269&lt;&gt;K269,"CEK JENIS ZONA",IF(A269="","Zona kosong",IF(B269="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A269="",F269=""),"",IF(F269="","Belum ditempatkan",IF(I269="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G269="","CEK ZONA NO kosong",IF(K269="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H269&lt;&gt;K269,"CEK JENIS ZONA",IF(A269="","Zona STOCK",IF(B269="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11017,7 +11017,7 @@
         <v/>
       </c>
       <c r="M270" s="12">
-        <f>IF(AND(A270="",F270=""),"",IF(F270="","Belum ditempatkan",IF(I270="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G270="","CEK ZONA NO kosong",IF(K270="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H270&lt;&gt;K270,"CEK JENIS ZONA",IF(A270="","Zona kosong",IF(B270="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A270="",F270=""),"",IF(F270="","Belum ditempatkan",IF(I270="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G270="","CEK ZONA NO kosong",IF(K270="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H270&lt;&gt;K270,"CEK JENIS ZONA",IF(A270="","Zona STOCK",IF(B270="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="M271" s="12">
-        <f>IF(AND(A271="",F271=""),"",IF(F271="","Belum ditempatkan",IF(I271="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G271="","CEK ZONA NO kosong",IF(K271="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H271&lt;&gt;K271,"CEK JENIS ZONA",IF(A271="","Zona kosong",IF(B271="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A271="",F271=""),"",IF(F271="","Belum ditempatkan",IF(I271="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G271="","CEK ZONA NO kosong",IF(K271="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H271&lt;&gt;K271,"CEK JENIS ZONA",IF(A271="","Zona STOCK",IF(B271="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11077,7 +11077,7 @@
         <v/>
       </c>
       <c r="M272" s="12">
-        <f>IF(AND(A272="",F272=""),"",IF(F272="","Belum ditempatkan",IF(I272="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G272="","CEK ZONA NO kosong",IF(K272="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H272&lt;&gt;K272,"CEK JENIS ZONA",IF(A272="","Zona kosong",IF(B272="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A272="",F272=""),"",IF(F272="","Belum ditempatkan",IF(I272="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G272="","CEK ZONA NO kosong",IF(K272="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H272&lt;&gt;K272,"CEK JENIS ZONA",IF(A272="","Zona STOCK",IF(B272="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11107,7 +11107,7 @@
         <v/>
       </c>
       <c r="M273" s="12">
-        <f>IF(AND(A273="",F273=""),"",IF(F273="","Belum ditempatkan",IF(I273="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G273="","CEK ZONA NO kosong",IF(K273="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H273&lt;&gt;K273,"CEK JENIS ZONA",IF(A273="","Zona kosong",IF(B273="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A273="",F273=""),"",IF(F273="","Belum ditempatkan",IF(I273="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G273="","CEK ZONA NO kosong",IF(K273="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H273&lt;&gt;K273,"CEK JENIS ZONA",IF(A273="","Zona STOCK",IF(B273="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11137,7 +11137,7 @@
         <v/>
       </c>
       <c r="M274" s="12">
-        <f>IF(AND(A274="",F274=""),"",IF(F274="","Belum ditempatkan",IF(I274="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G274="","CEK ZONA NO kosong",IF(K274="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H274&lt;&gt;K274,"CEK JENIS ZONA",IF(A274="","Zona kosong",IF(B274="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A274="",F274=""),"",IF(F274="","Belum ditempatkan",IF(I274="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G274="","CEK ZONA NO kosong",IF(K274="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H274&lt;&gt;K274,"CEK JENIS ZONA",IF(A274="","Zona STOCK",IF(B274="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11167,7 +11167,7 @@
         <v/>
       </c>
       <c r="M275" s="12">
-        <f>IF(AND(A275="",F275=""),"",IF(F275="","Belum ditempatkan",IF(I275="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G275="","CEK ZONA NO kosong",IF(K275="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H275&lt;&gt;K275,"CEK JENIS ZONA",IF(A275="","Zona kosong",IF(B275="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A275="",F275=""),"",IF(F275="","Belum ditempatkan",IF(I275="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G275="","CEK ZONA NO kosong",IF(K275="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H275&lt;&gt;K275,"CEK JENIS ZONA",IF(A275="","Zona STOCK",IF(B275="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11197,7 +11197,7 @@
         <v/>
       </c>
       <c r="M276" s="12">
-        <f>IF(AND(A276="",F276=""),"",IF(F276="","Belum ditempatkan",IF(I276="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G276="","CEK ZONA NO kosong",IF(K276="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H276&lt;&gt;K276,"CEK JENIS ZONA",IF(A276="","Zona kosong",IF(B276="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A276="",F276=""),"",IF(F276="","Belum ditempatkan",IF(I276="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G276="","CEK ZONA NO kosong",IF(K276="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H276&lt;&gt;K276,"CEK JENIS ZONA",IF(A276="","Zona STOCK",IF(B276="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11227,7 +11227,7 @@
         <v/>
       </c>
       <c r="M277" s="12">
-        <f>IF(AND(A277="",F277=""),"",IF(F277="","Belum ditempatkan",IF(I277="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G277="","CEK ZONA NO kosong",IF(K277="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H277&lt;&gt;K277,"CEK JENIS ZONA",IF(A277="","Zona kosong",IF(B277="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A277="",F277=""),"",IF(F277="","Belum ditempatkan",IF(I277="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G277="","CEK ZONA NO kosong",IF(K277="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H277&lt;&gt;K277,"CEK JENIS ZONA",IF(A277="","Zona STOCK",IF(B277="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11257,7 +11257,7 @@
         <v/>
       </c>
       <c r="M278" s="12">
-        <f>IF(AND(A278="",F278=""),"",IF(F278="","Belum ditempatkan",IF(I278="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G278="","CEK ZONA NO kosong",IF(K278="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H278&lt;&gt;K278,"CEK JENIS ZONA",IF(A278="","Zona kosong",IF(B278="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A278="",F278=""),"",IF(F278="","Belum ditempatkan",IF(I278="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G278="","CEK ZONA NO kosong",IF(K278="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H278&lt;&gt;K278,"CEK JENIS ZONA",IF(A278="","Zona STOCK",IF(B278="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11287,7 +11287,7 @@
         <v/>
       </c>
       <c r="M279" s="12">
-        <f>IF(AND(A279="",F279=""),"",IF(F279="","Belum ditempatkan",IF(I279="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G279="","CEK ZONA NO kosong",IF(K279="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H279&lt;&gt;K279,"CEK JENIS ZONA",IF(A279="","Zona kosong",IF(B279="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A279="",F279=""),"",IF(F279="","Belum ditempatkan",IF(I279="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G279="","CEK ZONA NO kosong",IF(K279="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H279&lt;&gt;K279,"CEK JENIS ZONA",IF(A279="","Zona STOCK",IF(B279="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11317,7 +11317,7 @@
         <v/>
       </c>
       <c r="M280" s="12">
-        <f>IF(AND(A280="",F280=""),"",IF(F280="","Belum ditempatkan",IF(I280="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G280="","CEK ZONA NO kosong",IF(K280="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H280&lt;&gt;K280,"CEK JENIS ZONA",IF(A280="","Zona kosong",IF(B280="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A280="",F280=""),"",IF(F280="","Belum ditempatkan",IF(I280="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G280="","CEK ZONA NO kosong",IF(K280="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H280&lt;&gt;K280,"CEK JENIS ZONA",IF(A280="","Zona STOCK",IF(B280="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11347,7 +11347,7 @@
         <v/>
       </c>
       <c r="M281" s="12">
-        <f>IF(AND(A281="",F281=""),"",IF(F281="","Belum ditempatkan",IF(I281="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G281="","CEK ZONA NO kosong",IF(K281="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H281&lt;&gt;K281,"CEK JENIS ZONA",IF(A281="","Zona kosong",IF(B281="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A281="",F281=""),"",IF(F281="","Belum ditempatkan",IF(I281="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G281="","CEK ZONA NO kosong",IF(K281="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H281&lt;&gt;K281,"CEK JENIS ZONA",IF(A281="","Zona STOCK",IF(B281="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11377,7 +11377,7 @@
         <v/>
       </c>
       <c r="M282" s="12">
-        <f>IF(AND(A282="",F282=""),"",IF(F282="","Belum ditempatkan",IF(I282="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G282="","CEK ZONA NO kosong",IF(K282="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H282&lt;&gt;K282,"CEK JENIS ZONA",IF(A282="","Zona kosong",IF(B282="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A282="",F282=""),"",IF(F282="","Belum ditempatkan",IF(I282="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G282="","CEK ZONA NO kosong",IF(K282="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H282&lt;&gt;K282,"CEK JENIS ZONA",IF(A282="","Zona STOCK",IF(B282="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11407,7 +11407,7 @@
         <v/>
       </c>
       <c r="M283" s="12">
-        <f>IF(AND(A283="",F283=""),"",IF(F283="","Belum ditempatkan",IF(I283="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G283="","CEK ZONA NO kosong",IF(K283="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H283&lt;&gt;K283,"CEK JENIS ZONA",IF(A283="","Zona kosong",IF(B283="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A283="",F283=""),"",IF(F283="","Belum ditempatkan",IF(I283="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G283="","CEK ZONA NO kosong",IF(K283="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H283&lt;&gt;K283,"CEK JENIS ZONA",IF(A283="","Zona STOCK",IF(B283="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11437,7 +11437,7 @@
         <v/>
       </c>
       <c r="M284" s="12">
-        <f>IF(AND(A284="",F284=""),"",IF(F284="","Belum ditempatkan",IF(I284="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G284="","CEK ZONA NO kosong",IF(K284="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H284&lt;&gt;K284,"CEK JENIS ZONA",IF(A284="","Zona kosong",IF(B284="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A284="",F284=""),"",IF(F284="","Belum ditempatkan",IF(I284="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G284="","CEK ZONA NO kosong",IF(K284="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H284&lt;&gt;K284,"CEK JENIS ZONA",IF(A284="","Zona STOCK",IF(B284="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11467,7 +11467,7 @@
         <v/>
       </c>
       <c r="M285" s="12">
-        <f>IF(AND(A285="",F285=""),"",IF(F285="","Belum ditempatkan",IF(I285="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G285="","CEK ZONA NO kosong",IF(K285="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H285&lt;&gt;K285,"CEK JENIS ZONA",IF(A285="","Zona kosong",IF(B285="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A285="",F285=""),"",IF(F285="","Belum ditempatkan",IF(I285="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G285="","CEK ZONA NO kosong",IF(K285="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H285&lt;&gt;K285,"CEK JENIS ZONA",IF(A285="","Zona STOCK",IF(B285="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11497,7 +11497,7 @@
         <v/>
       </c>
       <c r="M286" s="12">
-        <f>IF(AND(A286="",F286=""),"",IF(F286="","Belum ditempatkan",IF(I286="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G286="","CEK ZONA NO kosong",IF(K286="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H286&lt;&gt;K286,"CEK JENIS ZONA",IF(A286="","Zona kosong",IF(B286="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A286="",F286=""),"",IF(F286="","Belum ditempatkan",IF(I286="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G286="","CEK ZONA NO kosong",IF(K286="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H286&lt;&gt;K286,"CEK JENIS ZONA",IF(A286="","Zona STOCK",IF(B286="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11527,7 +11527,7 @@
         <v/>
       </c>
       <c r="M287" s="12">
-        <f>IF(AND(A287="",F287=""),"",IF(F287="","Belum ditempatkan",IF(I287="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G287="","CEK ZONA NO kosong",IF(K287="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H287&lt;&gt;K287,"CEK JENIS ZONA",IF(A287="","Zona kosong",IF(B287="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A287="",F287=""),"",IF(F287="","Belum ditempatkan",IF(I287="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G287="","CEK ZONA NO kosong",IF(K287="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H287&lt;&gt;K287,"CEK JENIS ZONA",IF(A287="","Zona STOCK",IF(B287="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11557,7 +11557,7 @@
         <v/>
       </c>
       <c r="M288" s="12">
-        <f>IF(AND(A288="",F288=""),"",IF(F288="","Belum ditempatkan",IF(I288="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G288="","CEK ZONA NO kosong",IF(K288="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H288&lt;&gt;K288,"CEK JENIS ZONA",IF(A288="","Zona kosong",IF(B288="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A288="",F288=""),"",IF(F288="","Belum ditempatkan",IF(I288="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G288="","CEK ZONA NO kosong",IF(K288="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H288&lt;&gt;K288,"CEK JENIS ZONA",IF(A288="","Zona STOCK",IF(B288="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11587,7 +11587,7 @@
         <v/>
       </c>
       <c r="M289" s="12">
-        <f>IF(AND(A289="",F289=""),"",IF(F289="","Belum ditempatkan",IF(I289="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G289="","CEK ZONA NO kosong",IF(K289="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H289&lt;&gt;K289,"CEK JENIS ZONA",IF(A289="","Zona kosong",IF(B289="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A289="",F289=""),"",IF(F289="","Belum ditempatkan",IF(I289="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G289="","CEK ZONA NO kosong",IF(K289="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H289&lt;&gt;K289,"CEK JENIS ZONA",IF(A289="","Zona STOCK",IF(B289="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11617,7 +11617,7 @@
         <v/>
       </c>
       <c r="M290" s="12">
-        <f>IF(AND(A290="",F290=""),"",IF(F290="","Belum ditempatkan",IF(I290="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G290="","CEK ZONA NO kosong",IF(K290="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H290&lt;&gt;K290,"CEK JENIS ZONA",IF(A290="","Zona kosong",IF(B290="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A290="",F290=""),"",IF(F290="","Belum ditempatkan",IF(I290="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G290="","CEK ZONA NO kosong",IF(K290="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H290&lt;&gt;K290,"CEK JENIS ZONA",IF(A290="","Zona STOCK",IF(B290="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11647,7 +11647,7 @@
         <v/>
       </c>
       <c r="M291" s="12">
-        <f>IF(AND(A291="",F291=""),"",IF(F291="","Belum ditempatkan",IF(I291="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G291="","CEK ZONA NO kosong",IF(K291="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H291&lt;&gt;K291,"CEK JENIS ZONA",IF(A291="","Zona kosong",IF(B291="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A291="",F291=""),"",IF(F291="","Belum ditempatkan",IF(I291="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G291="","CEK ZONA NO kosong",IF(K291="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H291&lt;&gt;K291,"CEK JENIS ZONA",IF(A291="","Zona STOCK",IF(B291="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11677,7 +11677,7 @@
         <v/>
       </c>
       <c r="M292" s="12">
-        <f>IF(AND(A292="",F292=""),"",IF(F292="","Belum ditempatkan",IF(I292="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G292="","CEK ZONA NO kosong",IF(K292="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H292&lt;&gt;K292,"CEK JENIS ZONA",IF(A292="","Zona kosong",IF(B292="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A292="",F292=""),"",IF(F292="","Belum ditempatkan",IF(I292="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G292="","CEK ZONA NO kosong",IF(K292="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H292&lt;&gt;K292,"CEK JENIS ZONA",IF(A292="","Zona STOCK",IF(B292="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11707,7 +11707,7 @@
         <v/>
       </c>
       <c r="M293" s="12">
-        <f>IF(AND(A293="",F293=""),"",IF(F293="","Belum ditempatkan",IF(I293="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G293="","CEK ZONA NO kosong",IF(K293="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H293&lt;&gt;K293,"CEK JENIS ZONA",IF(A293="","Zona kosong",IF(B293="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A293="",F293=""),"",IF(F293="","Belum ditempatkan",IF(I293="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G293="","CEK ZONA NO kosong",IF(K293="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H293&lt;&gt;K293,"CEK JENIS ZONA",IF(A293="","Zona STOCK",IF(B293="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11737,7 +11737,7 @@
         <v/>
       </c>
       <c r="M294" s="12">
-        <f>IF(AND(A294="",F294=""),"",IF(F294="","Belum ditempatkan",IF(I294="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G294="","CEK ZONA NO kosong",IF(K294="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H294&lt;&gt;K294,"CEK JENIS ZONA",IF(A294="","Zona kosong",IF(B294="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A294="",F294=""),"",IF(F294="","Belum ditempatkan",IF(I294="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G294="","CEK ZONA NO kosong",IF(K294="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H294&lt;&gt;K294,"CEK JENIS ZONA",IF(A294="","Zona STOCK",IF(B294="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11767,7 +11767,7 @@
         <v/>
       </c>
       <c r="M295" s="12">
-        <f>IF(AND(A295="",F295=""),"",IF(F295="","Belum ditempatkan",IF(I295="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G295="","CEK ZONA NO kosong",IF(K295="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H295&lt;&gt;K295,"CEK JENIS ZONA",IF(A295="","Zona kosong",IF(B295="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A295="",F295=""),"",IF(F295="","Belum ditempatkan",IF(I295="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G295="","CEK ZONA NO kosong",IF(K295="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H295&lt;&gt;K295,"CEK JENIS ZONA",IF(A295="","Zona STOCK",IF(B295="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11797,7 +11797,7 @@
         <v/>
       </c>
       <c r="M296" s="12">
-        <f>IF(AND(A296="",F296=""),"",IF(F296="","Belum ditempatkan",IF(I296="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G296="","CEK ZONA NO kosong",IF(K296="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H296&lt;&gt;K296,"CEK JENIS ZONA",IF(A296="","Zona kosong",IF(B296="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A296="",F296=""),"",IF(F296="","Belum ditempatkan",IF(I296="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G296="","CEK ZONA NO kosong",IF(K296="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H296&lt;&gt;K296,"CEK JENIS ZONA",IF(A296="","Zona STOCK",IF(B296="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11827,7 +11827,7 @@
         <v/>
       </c>
       <c r="M297" s="12">
-        <f>IF(AND(A297="",F297=""),"",IF(F297="","Belum ditempatkan",IF(I297="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G297="","CEK ZONA NO kosong",IF(K297="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H297&lt;&gt;K297,"CEK JENIS ZONA",IF(A297="","Zona kosong",IF(B297="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A297="",F297=""),"",IF(F297="","Belum ditempatkan",IF(I297="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G297="","CEK ZONA NO kosong",IF(K297="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H297&lt;&gt;K297,"CEK JENIS ZONA",IF(A297="","Zona STOCK",IF(B297="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11857,7 +11857,7 @@
         <v/>
       </c>
       <c r="M298" s="12">
-        <f>IF(AND(A298="",F298=""),"",IF(F298="","Belum ditempatkan",IF(I298="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G298="","CEK ZONA NO kosong",IF(K298="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H298&lt;&gt;K298,"CEK JENIS ZONA",IF(A298="","Zona kosong",IF(B298="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A298="",F298=""),"",IF(F298="","Belum ditempatkan",IF(I298="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G298="","CEK ZONA NO kosong",IF(K298="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H298&lt;&gt;K298,"CEK JENIS ZONA",IF(A298="","Zona STOCK",IF(B298="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11887,7 +11887,7 @@
         <v/>
       </c>
       <c r="M299" s="12">
-        <f>IF(AND(A299="",F299=""),"",IF(F299="","Belum ditempatkan",IF(I299="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G299="","CEK ZONA NO kosong",IF(K299="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H299&lt;&gt;K299,"CEK JENIS ZONA",IF(A299="","Zona kosong",IF(B299="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A299="",F299=""),"",IF(F299="","Belum ditempatkan",IF(I299="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G299="","CEK ZONA NO kosong",IF(K299="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H299&lt;&gt;K299,"CEK JENIS ZONA",IF(A299="","Zona STOCK",IF(B299="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11917,7 +11917,7 @@
         <v/>
       </c>
       <c r="M300" s="12">
-        <f>IF(AND(A300="",F300=""),"",IF(F300="","Belum ditempatkan",IF(I300="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G300="","CEK ZONA NO kosong",IF(K300="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H300&lt;&gt;K300,"CEK JENIS ZONA",IF(A300="","Zona kosong",IF(B300="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A300="",F300=""),"",IF(F300="","Belum ditempatkan",IF(I300="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G300="","CEK ZONA NO kosong",IF(K300="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H300&lt;&gt;K300,"CEK JENIS ZONA",IF(A300="","Zona STOCK",IF(B300="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11947,7 +11947,7 @@
         <v/>
       </c>
       <c r="M301" s="12">
-        <f>IF(AND(A301="",F301=""),"",IF(F301="","Belum ditempatkan",IF(I301="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G301="","CEK ZONA NO kosong",IF(K301="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H301&lt;&gt;K301,"CEK JENIS ZONA",IF(A301="","Zona kosong",IF(B301="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A301="",F301=""),"",IF(F301="","Belum ditempatkan",IF(I301="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G301="","CEK ZONA NO kosong",IF(K301="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H301&lt;&gt;K301,"CEK JENIS ZONA",IF(A301="","Zona STOCK",IF(B301="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -11977,7 +11977,7 @@
         <v/>
       </c>
       <c r="M302" s="12">
-        <f>IF(AND(A302="",F302=""),"",IF(F302="","Belum ditempatkan",IF(I302="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G302="","CEK ZONA NO kosong",IF(K302="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H302&lt;&gt;K302,"CEK JENIS ZONA",IF(A302="","Zona kosong",IF(B302="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A302="",F302=""),"",IF(F302="","Belum ditempatkan",IF(I302="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G302="","CEK ZONA NO kosong",IF(K302="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H302&lt;&gt;K302,"CEK JENIS ZONA",IF(A302="","Zona STOCK",IF(B302="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12007,7 +12007,7 @@
         <v/>
       </c>
       <c r="M303" s="12">
-        <f>IF(AND(A303="",F303=""),"",IF(F303="","Belum ditempatkan",IF(I303="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G303="","CEK ZONA NO kosong",IF(K303="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H303&lt;&gt;K303,"CEK JENIS ZONA",IF(A303="","Zona kosong",IF(B303="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A303="",F303=""),"",IF(F303="","Belum ditempatkan",IF(I303="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G303="","CEK ZONA NO kosong",IF(K303="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H303&lt;&gt;K303,"CEK JENIS ZONA",IF(A303="","Zona STOCK",IF(B303="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12037,7 +12037,7 @@
         <v/>
       </c>
       <c r="M304" s="12">
-        <f>IF(AND(A304="",F304=""),"",IF(F304="","Belum ditempatkan",IF(I304="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G304="","CEK ZONA NO kosong",IF(K304="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H304&lt;&gt;K304,"CEK JENIS ZONA",IF(A304="","Zona kosong",IF(B304="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A304="",F304=""),"",IF(F304="","Belum ditempatkan",IF(I304="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G304="","CEK ZONA NO kosong",IF(K304="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H304&lt;&gt;K304,"CEK JENIS ZONA",IF(A304="","Zona STOCK",IF(B304="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12067,7 +12067,7 @@
         <v/>
       </c>
       <c r="M305" s="12">
-        <f>IF(AND(A305="",F305=""),"",IF(F305="","Belum ditempatkan",IF(I305="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G305="","CEK ZONA NO kosong",IF(K305="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H305&lt;&gt;K305,"CEK JENIS ZONA",IF(A305="","Zona kosong",IF(B305="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A305="",F305=""),"",IF(F305="","Belum ditempatkan",IF(I305="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G305="","CEK ZONA NO kosong",IF(K305="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H305&lt;&gt;K305,"CEK JENIS ZONA",IF(A305="","Zona STOCK",IF(B305="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12097,7 +12097,7 @@
         <v/>
       </c>
       <c r="M306" s="12">
-        <f>IF(AND(A306="",F306=""),"",IF(F306="","Belum ditempatkan",IF(I306="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G306="","CEK ZONA NO kosong",IF(K306="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H306&lt;&gt;K306,"CEK JENIS ZONA",IF(A306="","Zona kosong",IF(B306="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A306="",F306=""),"",IF(F306="","Belum ditempatkan",IF(I306="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G306="","CEK ZONA NO kosong",IF(K306="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H306&lt;&gt;K306,"CEK JENIS ZONA",IF(A306="","Zona STOCK",IF(B306="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12127,7 +12127,7 @@
         <v/>
       </c>
       <c r="M307" s="12">
-        <f>IF(AND(A307="",F307=""),"",IF(F307="","Belum ditempatkan",IF(I307="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G307="","CEK ZONA NO kosong",IF(K307="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H307&lt;&gt;K307,"CEK JENIS ZONA",IF(A307="","Zona kosong",IF(B307="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A307="",F307=""),"",IF(F307="","Belum ditempatkan",IF(I307="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G307="","CEK ZONA NO kosong",IF(K307="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H307&lt;&gt;K307,"CEK JENIS ZONA",IF(A307="","Zona STOCK",IF(B307="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12157,7 +12157,7 @@
         <v/>
       </c>
       <c r="M308" s="12">
-        <f>IF(AND(A308="",F308=""),"",IF(F308="","Belum ditempatkan",IF(I308="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G308="","CEK ZONA NO kosong",IF(K308="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H308&lt;&gt;K308,"CEK JENIS ZONA",IF(A308="","Zona kosong",IF(B308="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A308="",F308=""),"",IF(F308="","Belum ditempatkan",IF(I308="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G308="","CEK ZONA NO kosong",IF(K308="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H308&lt;&gt;K308,"CEK JENIS ZONA",IF(A308="","Zona STOCK",IF(B308="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12187,7 +12187,7 @@
         <v/>
       </c>
       <c r="M309" s="12">
-        <f>IF(AND(A309="",F309=""),"",IF(F309="","Belum ditempatkan",IF(I309="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G309="","CEK ZONA NO kosong",IF(K309="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H309&lt;&gt;K309,"CEK JENIS ZONA",IF(A309="","Zona kosong",IF(B309="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A309="",F309=""),"",IF(F309="","Belum ditempatkan",IF(I309="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G309="","CEK ZONA NO kosong",IF(K309="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H309&lt;&gt;K309,"CEK JENIS ZONA",IF(A309="","Zona STOCK",IF(B309="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12217,7 +12217,7 @@
         <v/>
       </c>
       <c r="M310" s="12">
-        <f>IF(AND(A310="",F310=""),"",IF(F310="","Belum ditempatkan",IF(I310="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G310="","CEK ZONA NO kosong",IF(K310="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H310&lt;&gt;K310,"CEK JENIS ZONA",IF(A310="","Zona kosong",IF(B310="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A310="",F310=""),"",IF(F310="","Belum ditempatkan",IF(I310="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G310="","CEK ZONA NO kosong",IF(K310="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H310&lt;&gt;K310,"CEK JENIS ZONA",IF(A310="","Zona STOCK",IF(B310="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12247,7 +12247,7 @@
         <v/>
       </c>
       <c r="M311" s="12">
-        <f>IF(AND(A311="",F311=""),"",IF(F311="","Belum ditempatkan",IF(I311="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G311="","CEK ZONA NO kosong",IF(K311="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H311&lt;&gt;K311,"CEK JENIS ZONA",IF(A311="","Zona kosong",IF(B311="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A311="",F311=""),"",IF(F311="","Belum ditempatkan",IF(I311="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G311="","CEK ZONA NO kosong",IF(K311="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H311&lt;&gt;K311,"CEK JENIS ZONA",IF(A311="","Zona STOCK",IF(B311="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12277,7 +12277,7 @@
         <v/>
       </c>
       <c r="M312" s="12">
-        <f>IF(AND(A312="",F312=""),"",IF(F312="","Belum ditempatkan",IF(I312="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G312="","CEK ZONA NO kosong",IF(K312="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H312&lt;&gt;K312,"CEK JENIS ZONA",IF(A312="","Zona kosong",IF(B312="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A312="",F312=""),"",IF(F312="","Belum ditempatkan",IF(I312="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G312="","CEK ZONA NO kosong",IF(K312="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H312&lt;&gt;K312,"CEK JENIS ZONA",IF(A312="","Zona STOCK",IF(B312="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12307,7 +12307,7 @@
         <v/>
       </c>
       <c r="M313" s="12">
-        <f>IF(AND(A313="",F313=""),"",IF(F313="","Belum ditempatkan",IF(I313="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G313="","CEK ZONA NO kosong",IF(K313="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H313&lt;&gt;K313,"CEK JENIS ZONA",IF(A313="","Zona kosong",IF(B313="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A313="",F313=""),"",IF(F313="","Belum ditempatkan",IF(I313="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G313="","CEK ZONA NO kosong",IF(K313="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H313&lt;&gt;K313,"CEK JENIS ZONA",IF(A313="","Zona STOCK",IF(B313="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12337,7 +12337,7 @@
         <v/>
       </c>
       <c r="M314" s="12">
-        <f>IF(AND(A314="",F314=""),"",IF(F314="","Belum ditempatkan",IF(I314="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G314="","CEK ZONA NO kosong",IF(K314="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H314&lt;&gt;K314,"CEK JENIS ZONA",IF(A314="","Zona kosong",IF(B314="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A314="",F314=""),"",IF(F314="","Belum ditempatkan",IF(I314="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G314="","CEK ZONA NO kosong",IF(K314="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H314&lt;&gt;K314,"CEK JENIS ZONA",IF(A314="","Zona STOCK",IF(B314="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12367,7 +12367,7 @@
         <v/>
       </c>
       <c r="M315" s="12">
-        <f>IF(AND(A315="",F315=""),"",IF(F315="","Belum ditempatkan",IF(I315="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G315="","CEK ZONA NO kosong",IF(K315="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H315&lt;&gt;K315,"CEK JENIS ZONA",IF(A315="","Zona kosong",IF(B315="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A315="",F315=""),"",IF(F315="","Belum ditempatkan",IF(I315="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G315="","CEK ZONA NO kosong",IF(K315="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H315&lt;&gt;K315,"CEK JENIS ZONA",IF(A315="","Zona STOCK",IF(B315="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12397,7 +12397,7 @@
         <v/>
       </c>
       <c r="M316" s="12">
-        <f>IF(AND(A316="",F316=""),"",IF(F316="","Belum ditempatkan",IF(I316="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G316="","CEK ZONA NO kosong",IF(K316="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H316&lt;&gt;K316,"CEK JENIS ZONA",IF(A316="","Zona kosong",IF(B316="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A316="",F316=""),"",IF(F316="","Belum ditempatkan",IF(I316="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G316="","CEK ZONA NO kosong",IF(K316="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H316&lt;&gt;K316,"CEK JENIS ZONA",IF(A316="","Zona STOCK",IF(B316="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12427,7 +12427,7 @@
         <v/>
       </c>
       <c r="M317" s="12">
-        <f>IF(AND(A317="",F317=""),"",IF(F317="","Belum ditempatkan",IF(I317="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G317="","CEK ZONA NO kosong",IF(K317="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H317&lt;&gt;K317,"CEK JENIS ZONA",IF(A317="","Zona kosong",IF(B317="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A317="",F317=""),"",IF(F317="","Belum ditempatkan",IF(I317="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G317="","CEK ZONA NO kosong",IF(K317="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H317&lt;&gt;K317,"CEK JENIS ZONA",IF(A317="","Zona STOCK",IF(B317="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12457,7 +12457,7 @@
         <v/>
       </c>
       <c r="M318" s="12">
-        <f>IF(AND(A318="",F318=""),"",IF(F318="","Belum ditempatkan",IF(I318="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G318="","CEK ZONA NO kosong",IF(K318="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H318&lt;&gt;K318,"CEK JENIS ZONA",IF(A318="","Zona kosong",IF(B318="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A318="",F318=""),"",IF(F318="","Belum ditempatkan",IF(I318="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G318="","CEK ZONA NO kosong",IF(K318="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H318&lt;&gt;K318,"CEK JENIS ZONA",IF(A318="","Zona STOCK",IF(B318="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12487,7 +12487,7 @@
         <v/>
       </c>
       <c r="M319" s="12">
-        <f>IF(AND(A319="",F319=""),"",IF(F319="","Belum ditempatkan",IF(I319="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G319="","CEK ZONA NO kosong",IF(K319="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H319&lt;&gt;K319,"CEK JENIS ZONA",IF(A319="","Zona kosong",IF(B319="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A319="",F319=""),"",IF(F319="","Belum ditempatkan",IF(I319="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G319="","CEK ZONA NO kosong",IF(K319="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H319&lt;&gt;K319,"CEK JENIS ZONA",IF(A319="","Zona STOCK",IF(B319="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12517,7 +12517,7 @@
         <v/>
       </c>
       <c r="M320" s="12">
-        <f>IF(AND(A320="",F320=""),"",IF(F320="","Belum ditempatkan",IF(I320="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G320="","CEK ZONA NO kosong",IF(K320="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H320&lt;&gt;K320,"CEK JENIS ZONA",IF(A320="","Zona kosong",IF(B320="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A320="",F320=""),"",IF(F320="","Belum ditempatkan",IF(I320="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G320="","CEK ZONA NO kosong",IF(K320="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H320&lt;&gt;K320,"CEK JENIS ZONA",IF(A320="","Zona STOCK",IF(B320="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12547,7 +12547,7 @@
         <v/>
       </c>
       <c r="M321" s="12">
-        <f>IF(AND(A321="",F321=""),"",IF(F321="","Belum ditempatkan",IF(I321="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G321="","CEK ZONA NO kosong",IF(K321="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H321&lt;&gt;K321,"CEK JENIS ZONA",IF(A321="","Zona kosong",IF(B321="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A321="",F321=""),"",IF(F321="","Belum ditempatkan",IF(I321="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G321="","CEK ZONA NO kosong",IF(K321="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H321&lt;&gt;K321,"CEK JENIS ZONA",IF(A321="","Zona STOCK",IF(B321="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12577,7 +12577,7 @@
         <v/>
       </c>
       <c r="M322" s="12">
-        <f>IF(AND(A322="",F322=""),"",IF(F322="","Belum ditempatkan",IF(I322="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G322="","CEK ZONA NO kosong",IF(K322="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H322&lt;&gt;K322,"CEK JENIS ZONA",IF(A322="","Zona kosong",IF(B322="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A322="",F322=""),"",IF(F322="","Belum ditempatkan",IF(I322="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G322="","CEK ZONA NO kosong",IF(K322="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H322&lt;&gt;K322,"CEK JENIS ZONA",IF(A322="","Zona STOCK",IF(B322="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12607,7 +12607,7 @@
         <v/>
       </c>
       <c r="M323" s="12">
-        <f>IF(AND(A323="",F323=""),"",IF(F323="","Belum ditempatkan",IF(I323="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G323="","CEK ZONA NO kosong",IF(K323="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H323&lt;&gt;K323,"CEK JENIS ZONA",IF(A323="","Zona kosong",IF(B323="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A323="",F323=""),"",IF(F323="","Belum ditempatkan",IF(I323="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G323="","CEK ZONA NO kosong",IF(K323="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H323&lt;&gt;K323,"CEK JENIS ZONA",IF(A323="","Zona STOCK",IF(B323="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12637,7 +12637,7 @@
         <v/>
       </c>
       <c r="M324" s="12">
-        <f>IF(AND(A324="",F324=""),"",IF(F324="","Belum ditempatkan",IF(I324="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G324="","CEK ZONA NO kosong",IF(K324="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H324&lt;&gt;K324,"CEK JENIS ZONA",IF(A324="","Zona kosong",IF(B324="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A324="",F324=""),"",IF(F324="","Belum ditempatkan",IF(I324="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G324="","CEK ZONA NO kosong",IF(K324="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H324&lt;&gt;K324,"CEK JENIS ZONA",IF(A324="","Zona STOCK",IF(B324="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12667,7 +12667,7 @@
         <v/>
       </c>
       <c r="M325" s="12">
-        <f>IF(AND(A325="",F325=""),"",IF(F325="","Belum ditempatkan",IF(I325="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G325="","CEK ZONA NO kosong",IF(K325="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H325&lt;&gt;K325,"CEK JENIS ZONA",IF(A325="","Zona kosong",IF(B325="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A325="",F325=""),"",IF(F325="","Belum ditempatkan",IF(I325="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G325="","CEK ZONA NO kosong",IF(K325="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H325&lt;&gt;K325,"CEK JENIS ZONA",IF(A325="","Zona STOCK",IF(B325="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12697,7 +12697,7 @@
         <v/>
       </c>
       <c r="M326" s="12">
-        <f>IF(AND(A326="",F326=""),"",IF(F326="","Belum ditempatkan",IF(I326="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G326="","CEK ZONA NO kosong",IF(K326="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H326&lt;&gt;K326,"CEK JENIS ZONA",IF(A326="","Zona kosong",IF(B326="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A326="",F326=""),"",IF(F326="","Belum ditempatkan",IF(I326="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G326="","CEK ZONA NO kosong",IF(K326="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H326&lt;&gt;K326,"CEK JENIS ZONA",IF(A326="","Zona STOCK",IF(B326="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12727,7 +12727,7 @@
         <v/>
       </c>
       <c r="M327" s="12">
-        <f>IF(AND(A327="",F327=""),"",IF(F327="","Belum ditempatkan",IF(I327="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G327="","CEK ZONA NO kosong",IF(K327="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H327&lt;&gt;K327,"CEK JENIS ZONA",IF(A327="","Zona kosong",IF(B327="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A327="",F327=""),"",IF(F327="","Belum ditempatkan",IF(I327="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G327="","CEK ZONA NO kosong",IF(K327="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H327&lt;&gt;K327,"CEK JENIS ZONA",IF(A327="","Zona STOCK",IF(B327="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12757,7 +12757,7 @@
         <v/>
       </c>
       <c r="M328" s="12">
-        <f>IF(AND(A328="",F328=""),"",IF(F328="","Belum ditempatkan",IF(I328="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G328="","CEK ZONA NO kosong",IF(K328="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H328&lt;&gt;K328,"CEK JENIS ZONA",IF(A328="","Zona kosong",IF(B328="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A328="",F328=""),"",IF(F328="","Belum ditempatkan",IF(I328="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G328="","CEK ZONA NO kosong",IF(K328="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H328&lt;&gt;K328,"CEK JENIS ZONA",IF(A328="","Zona STOCK",IF(B328="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12787,7 +12787,7 @@
         <v/>
       </c>
       <c r="M329" s="12">
-        <f>IF(AND(A329="",F329=""),"",IF(F329="","Belum ditempatkan",IF(I329="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G329="","CEK ZONA NO kosong",IF(K329="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H329&lt;&gt;K329,"CEK JENIS ZONA",IF(A329="","Zona kosong",IF(B329="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A329="",F329=""),"",IF(F329="","Belum ditempatkan",IF(I329="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G329="","CEK ZONA NO kosong",IF(K329="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H329&lt;&gt;K329,"CEK JENIS ZONA",IF(A329="","Zona STOCK",IF(B329="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12817,7 +12817,7 @@
         <v/>
       </c>
       <c r="M330" s="12">
-        <f>IF(AND(A330="",F330=""),"",IF(F330="","Belum ditempatkan",IF(I330="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G330="","CEK ZONA NO kosong",IF(K330="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H330&lt;&gt;K330,"CEK JENIS ZONA",IF(A330="","Zona kosong",IF(B330="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A330="",F330=""),"",IF(F330="","Belum ditempatkan",IF(I330="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G330="","CEK ZONA NO kosong",IF(K330="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H330&lt;&gt;K330,"CEK JENIS ZONA",IF(A330="","Zona STOCK",IF(B330="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12847,7 +12847,7 @@
         <v/>
       </c>
       <c r="M331" s="12">
-        <f>IF(AND(A331="",F331=""),"",IF(F331="","Belum ditempatkan",IF(I331="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G331="","CEK ZONA NO kosong",IF(K331="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H331&lt;&gt;K331,"CEK JENIS ZONA",IF(A331="","Zona kosong",IF(B331="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A331="",F331=""),"",IF(F331="","Belum ditempatkan",IF(I331="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G331="","CEK ZONA NO kosong",IF(K331="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H331&lt;&gt;K331,"CEK JENIS ZONA",IF(A331="","Zona STOCK",IF(B331="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12877,7 +12877,7 @@
         <v/>
       </c>
       <c r="M332" s="12">
-        <f>IF(AND(A332="",F332=""),"",IF(F332="","Belum ditempatkan",IF(I332="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G332="","CEK ZONA NO kosong",IF(K332="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H332&lt;&gt;K332,"CEK JENIS ZONA",IF(A332="","Zona kosong",IF(B332="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A332="",F332=""),"",IF(F332="","Belum ditempatkan",IF(I332="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G332="","CEK ZONA NO kosong",IF(K332="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H332&lt;&gt;K332,"CEK JENIS ZONA",IF(A332="","Zona STOCK",IF(B332="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12907,7 +12907,7 @@
         <v/>
       </c>
       <c r="M333" s="12">
-        <f>IF(AND(A333="",F333=""),"",IF(F333="","Belum ditempatkan",IF(I333="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G333="","CEK ZONA NO kosong",IF(K333="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H333&lt;&gt;K333,"CEK JENIS ZONA",IF(A333="","Zona kosong",IF(B333="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A333="",F333=""),"",IF(F333="","Belum ditempatkan",IF(I333="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G333="","CEK ZONA NO kosong",IF(K333="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H333&lt;&gt;K333,"CEK JENIS ZONA",IF(A333="","Zona STOCK",IF(B333="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12937,7 +12937,7 @@
         <v/>
       </c>
       <c r="M334" s="12">
-        <f>IF(AND(A334="",F334=""),"",IF(F334="","Belum ditempatkan",IF(I334="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G334="","CEK ZONA NO kosong",IF(K334="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H334&lt;&gt;K334,"CEK JENIS ZONA",IF(A334="","Zona kosong",IF(B334="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A334="",F334=""),"",IF(F334="","Belum ditempatkan",IF(I334="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G334="","CEK ZONA NO kosong",IF(K334="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H334&lt;&gt;K334,"CEK JENIS ZONA",IF(A334="","Zona STOCK",IF(B334="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12967,7 +12967,7 @@
         <v/>
       </c>
       <c r="M335" s="12">
-        <f>IF(AND(A335="",F335=""),"",IF(F335="","Belum ditempatkan",IF(I335="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G335="","CEK ZONA NO kosong",IF(K335="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H335&lt;&gt;K335,"CEK JENIS ZONA",IF(A335="","Zona kosong",IF(B335="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A335="",F335=""),"",IF(F335="","Belum ditempatkan",IF(I335="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G335="","CEK ZONA NO kosong",IF(K335="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H335&lt;&gt;K335,"CEK JENIS ZONA",IF(A335="","Zona STOCK",IF(B335="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -12997,7 +12997,7 @@
         <v/>
       </c>
       <c r="M336" s="12">
-        <f>IF(AND(A336="",F336=""),"",IF(F336="","Belum ditempatkan",IF(I336="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G336="","CEK ZONA NO kosong",IF(K336="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H336&lt;&gt;K336,"CEK JENIS ZONA",IF(A336="","Zona kosong",IF(B336="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A336="",F336=""),"",IF(F336="","Belum ditempatkan",IF(I336="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G336="","CEK ZONA NO kosong",IF(K336="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H336&lt;&gt;K336,"CEK JENIS ZONA",IF(A336="","Zona STOCK",IF(B336="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13027,7 +13027,7 @@
         <v/>
       </c>
       <c r="M337" s="12">
-        <f>IF(AND(A337="",F337=""),"",IF(F337="","Belum ditempatkan",IF(I337="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G337="","CEK ZONA NO kosong",IF(K337="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H337&lt;&gt;K337,"CEK JENIS ZONA",IF(A337="","Zona kosong",IF(B337="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A337="",F337=""),"",IF(F337="","Belum ditempatkan",IF(I337="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G337="","CEK ZONA NO kosong",IF(K337="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H337&lt;&gt;K337,"CEK JENIS ZONA",IF(A337="","Zona STOCK",IF(B337="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13057,7 +13057,7 @@
         <v/>
       </c>
       <c r="M338" s="12">
-        <f>IF(AND(A338="",F338=""),"",IF(F338="","Belum ditempatkan",IF(I338="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G338="","CEK ZONA NO kosong",IF(K338="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H338&lt;&gt;K338,"CEK JENIS ZONA",IF(A338="","Zona kosong",IF(B338="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A338="",F338=""),"",IF(F338="","Belum ditempatkan",IF(I338="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G338="","CEK ZONA NO kosong",IF(K338="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H338&lt;&gt;K338,"CEK JENIS ZONA",IF(A338="","Zona STOCK",IF(B338="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13087,7 +13087,7 @@
         <v/>
       </c>
       <c r="M339" s="12">
-        <f>IF(AND(A339="",F339=""),"",IF(F339="","Belum ditempatkan",IF(I339="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G339="","CEK ZONA NO kosong",IF(K339="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H339&lt;&gt;K339,"CEK JENIS ZONA",IF(A339="","Zona kosong",IF(B339="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A339="",F339=""),"",IF(F339="","Belum ditempatkan",IF(I339="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G339="","CEK ZONA NO kosong",IF(K339="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H339&lt;&gt;K339,"CEK JENIS ZONA",IF(A339="","Zona STOCK",IF(B339="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13117,7 +13117,7 @@
         <v/>
       </c>
       <c r="M340" s="12">
-        <f>IF(AND(A340="",F340=""),"",IF(F340="","Belum ditempatkan",IF(I340="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G340="","CEK ZONA NO kosong",IF(K340="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H340&lt;&gt;K340,"CEK JENIS ZONA",IF(A340="","Zona kosong",IF(B340="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A340="",F340=""),"",IF(F340="","Belum ditempatkan",IF(I340="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G340="","CEK ZONA NO kosong",IF(K340="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H340&lt;&gt;K340,"CEK JENIS ZONA",IF(A340="","Zona STOCK",IF(B340="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13147,7 +13147,7 @@
         <v/>
       </c>
       <c r="M341" s="12">
-        <f>IF(AND(A341="",F341=""),"",IF(F341="","Belum ditempatkan",IF(I341="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G341="","CEK ZONA NO kosong",IF(K341="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H341&lt;&gt;K341,"CEK JENIS ZONA",IF(A341="","Zona kosong",IF(B341="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A341="",F341=""),"",IF(F341="","Belum ditempatkan",IF(I341="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G341="","CEK ZONA NO kosong",IF(K341="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H341&lt;&gt;K341,"CEK JENIS ZONA",IF(A341="","Zona STOCK",IF(B341="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13177,7 +13177,7 @@
         <v/>
       </c>
       <c r="M342" s="12">
-        <f>IF(AND(A342="",F342=""),"",IF(F342="","Belum ditempatkan",IF(I342="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G342="","CEK ZONA NO kosong",IF(K342="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H342&lt;&gt;K342,"CEK JENIS ZONA",IF(A342="","Zona kosong",IF(B342="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A342="",F342=""),"",IF(F342="","Belum ditempatkan",IF(I342="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G342="","CEK ZONA NO kosong",IF(K342="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H342&lt;&gt;K342,"CEK JENIS ZONA",IF(A342="","Zona STOCK",IF(B342="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13207,7 +13207,7 @@
         <v/>
       </c>
       <c r="M343" s="12">
-        <f>IF(AND(A343="",F343=""),"",IF(F343="","Belum ditempatkan",IF(I343="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G343="","CEK ZONA NO kosong",IF(K343="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H343&lt;&gt;K343,"CEK JENIS ZONA",IF(A343="","Zona kosong",IF(B343="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A343="",F343=""),"",IF(F343="","Belum ditempatkan",IF(I343="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G343="","CEK ZONA NO kosong",IF(K343="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H343&lt;&gt;K343,"CEK JENIS ZONA",IF(A343="","Zona STOCK",IF(B343="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13237,7 +13237,7 @@
         <v/>
       </c>
       <c r="M344" s="12">
-        <f>IF(AND(A344="",F344=""),"",IF(F344="","Belum ditempatkan",IF(I344="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G344="","CEK ZONA NO kosong",IF(K344="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H344&lt;&gt;K344,"CEK JENIS ZONA",IF(A344="","Zona kosong",IF(B344="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A344="",F344=""),"",IF(F344="","Belum ditempatkan",IF(I344="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G344="","CEK ZONA NO kosong",IF(K344="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H344&lt;&gt;K344,"CEK JENIS ZONA",IF(A344="","Zona STOCK",IF(B344="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13267,7 +13267,7 @@
         <v/>
       </c>
       <c r="M345" s="12">
-        <f>IF(AND(A345="",F345=""),"",IF(F345="","Belum ditempatkan",IF(I345="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G345="","CEK ZONA NO kosong",IF(K345="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H345&lt;&gt;K345,"CEK JENIS ZONA",IF(A345="","Zona kosong",IF(B345="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A345="",F345=""),"",IF(F345="","Belum ditempatkan",IF(I345="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G345="","CEK ZONA NO kosong",IF(K345="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H345&lt;&gt;K345,"CEK JENIS ZONA",IF(A345="","Zona STOCK",IF(B345="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13297,7 +13297,7 @@
         <v/>
       </c>
       <c r="M346" s="12">
-        <f>IF(AND(A346="",F346=""),"",IF(F346="","Belum ditempatkan",IF(I346="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G346="","CEK ZONA NO kosong",IF(K346="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H346&lt;&gt;K346,"CEK JENIS ZONA",IF(A346="","Zona kosong",IF(B346="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A346="",F346=""),"",IF(F346="","Belum ditempatkan",IF(I346="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G346="","CEK ZONA NO kosong",IF(K346="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H346&lt;&gt;K346,"CEK JENIS ZONA",IF(A346="","Zona STOCK",IF(B346="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13327,7 +13327,7 @@
         <v/>
       </c>
       <c r="M347" s="12">
-        <f>IF(AND(A347="",F347=""),"",IF(F347="","Belum ditempatkan",IF(I347="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G347="","CEK ZONA NO kosong",IF(K347="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H347&lt;&gt;K347,"CEK JENIS ZONA",IF(A347="","Zona kosong",IF(B347="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A347="",F347=""),"",IF(F347="","Belum ditempatkan",IF(I347="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G347="","CEK ZONA NO kosong",IF(K347="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H347&lt;&gt;K347,"CEK JENIS ZONA",IF(A347="","Zona STOCK",IF(B347="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13357,7 +13357,7 @@
         <v/>
       </c>
       <c r="M348" s="12">
-        <f>IF(AND(A348="",F348=""),"",IF(F348="","Belum ditempatkan",IF(I348="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G348="","CEK ZONA NO kosong",IF(K348="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H348&lt;&gt;K348,"CEK JENIS ZONA",IF(A348="","Zona kosong",IF(B348="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A348="",F348=""),"",IF(F348="","Belum ditempatkan",IF(I348="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G348="","CEK ZONA NO kosong",IF(K348="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H348&lt;&gt;K348,"CEK JENIS ZONA",IF(A348="","Zona STOCK",IF(B348="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13387,7 +13387,7 @@
         <v/>
       </c>
       <c r="M349" s="12">
-        <f>IF(AND(A349="",F349=""),"",IF(F349="","Belum ditempatkan",IF(I349="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G349="","CEK ZONA NO kosong",IF(K349="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H349&lt;&gt;K349,"CEK JENIS ZONA",IF(A349="","Zona kosong",IF(B349="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A349="",F349=""),"",IF(F349="","Belum ditempatkan",IF(I349="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G349="","CEK ZONA NO kosong",IF(K349="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H349&lt;&gt;K349,"CEK JENIS ZONA",IF(A349="","Zona STOCK",IF(B349="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13417,7 +13417,7 @@
         <v/>
       </c>
       <c r="M350" s="12">
-        <f>IF(AND(A350="",F350=""),"",IF(F350="","Belum ditempatkan",IF(I350="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G350="","CEK ZONA NO kosong",IF(K350="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H350&lt;&gt;K350,"CEK JENIS ZONA",IF(A350="","Zona kosong",IF(B350="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A350="",F350=""),"",IF(F350="","Belum ditempatkan",IF(I350="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G350="","CEK ZONA NO kosong",IF(K350="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H350&lt;&gt;K350,"CEK JENIS ZONA",IF(A350="","Zona STOCK",IF(B350="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13447,7 +13447,7 @@
         <v/>
       </c>
       <c r="M351" s="12">
-        <f>IF(AND(A351="",F351=""),"",IF(F351="","Belum ditempatkan",IF(I351="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G351="","CEK ZONA NO kosong",IF(K351="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H351&lt;&gt;K351,"CEK JENIS ZONA",IF(A351="","Zona kosong",IF(B351="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A351="",F351=""),"",IF(F351="","Belum ditempatkan",IF(I351="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G351="","CEK ZONA NO kosong",IF(K351="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H351&lt;&gt;K351,"CEK JENIS ZONA",IF(A351="","Zona STOCK",IF(B351="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13477,7 +13477,7 @@
         <v/>
       </c>
       <c r="M352" s="12">
-        <f>IF(AND(A352="",F352=""),"",IF(F352="","Belum ditempatkan",IF(I352="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G352="","CEK ZONA NO kosong",IF(K352="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H352&lt;&gt;K352,"CEK JENIS ZONA",IF(A352="","Zona kosong",IF(B352="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A352="",F352=""),"",IF(F352="","Belum ditempatkan",IF(I352="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G352="","CEK ZONA NO kosong",IF(K352="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H352&lt;&gt;K352,"CEK JENIS ZONA",IF(A352="","Zona STOCK",IF(B352="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13507,7 +13507,7 @@
         <v/>
       </c>
       <c r="M353" s="12">
-        <f>IF(AND(A353="",F353=""),"",IF(F353="","Belum ditempatkan",IF(I353="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G353="","CEK ZONA NO kosong",IF(K353="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H353&lt;&gt;K353,"CEK JENIS ZONA",IF(A353="","Zona kosong",IF(B353="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A353="",F353=""),"",IF(F353="","Belum ditempatkan",IF(I353="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G353="","CEK ZONA NO kosong",IF(K353="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H353&lt;&gt;K353,"CEK JENIS ZONA",IF(A353="","Zona STOCK",IF(B353="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13537,7 +13537,7 @@
         <v/>
       </c>
       <c r="M354" s="12">
-        <f>IF(AND(A354="",F354=""),"",IF(F354="","Belum ditempatkan",IF(I354="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G354="","CEK ZONA NO kosong",IF(K354="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H354&lt;&gt;K354,"CEK JENIS ZONA",IF(A354="","Zona kosong",IF(B354="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A354="",F354=""),"",IF(F354="","Belum ditempatkan",IF(I354="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G354="","CEK ZONA NO kosong",IF(K354="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H354&lt;&gt;K354,"CEK JENIS ZONA",IF(A354="","Zona STOCK",IF(B354="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13567,7 +13567,7 @@
         <v/>
       </c>
       <c r="M355" s="12">
-        <f>IF(AND(A355="",F355=""),"",IF(F355="","Belum ditempatkan",IF(I355="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G355="","CEK ZONA NO kosong",IF(K355="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H355&lt;&gt;K355,"CEK JENIS ZONA",IF(A355="","Zona kosong",IF(B355="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A355="",F355=""),"",IF(F355="","Belum ditempatkan",IF(I355="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G355="","CEK ZONA NO kosong",IF(K355="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H355&lt;&gt;K355,"CEK JENIS ZONA",IF(A355="","Zona STOCK",IF(B355="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13597,7 +13597,7 @@
         <v/>
       </c>
       <c r="M356" s="12">
-        <f>IF(AND(A356="",F356=""),"",IF(F356="","Belum ditempatkan",IF(I356="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G356="","CEK ZONA NO kosong",IF(K356="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H356&lt;&gt;K356,"CEK JENIS ZONA",IF(A356="","Zona kosong",IF(B356="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A356="",F356=""),"",IF(F356="","Belum ditempatkan",IF(I356="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G356="","CEK ZONA NO kosong",IF(K356="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H356&lt;&gt;K356,"CEK JENIS ZONA",IF(A356="","Zona STOCK",IF(B356="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13627,7 +13627,7 @@
         <v/>
       </c>
       <c r="M357" s="12">
-        <f>IF(AND(A357="",F357=""),"",IF(F357="","Belum ditempatkan",IF(I357="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G357="","CEK ZONA NO kosong",IF(K357="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H357&lt;&gt;K357,"CEK JENIS ZONA",IF(A357="","Zona kosong",IF(B357="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A357="",F357=""),"",IF(F357="","Belum ditempatkan",IF(I357="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G357="","CEK ZONA NO kosong",IF(K357="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H357&lt;&gt;K357,"CEK JENIS ZONA",IF(A357="","Zona STOCK",IF(B357="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13657,7 +13657,7 @@
         <v/>
       </c>
       <c r="M358" s="12">
-        <f>IF(AND(A358="",F358=""),"",IF(F358="","Belum ditempatkan",IF(I358="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G358="","CEK ZONA NO kosong",IF(K358="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H358&lt;&gt;K358,"CEK JENIS ZONA",IF(A358="","Zona kosong",IF(B358="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A358="",F358=""),"",IF(F358="","Belum ditempatkan",IF(I358="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G358="","CEK ZONA NO kosong",IF(K358="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H358&lt;&gt;K358,"CEK JENIS ZONA",IF(A358="","Zona STOCK",IF(B358="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13687,7 +13687,7 @@
         <v/>
       </c>
       <c r="M359" s="12">
-        <f>IF(AND(A359="",F359=""),"",IF(F359="","Belum ditempatkan",IF(I359="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G359="","CEK ZONA NO kosong",IF(K359="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H359&lt;&gt;K359,"CEK JENIS ZONA",IF(A359="","Zona kosong",IF(B359="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A359="",F359=""),"",IF(F359="","Belum ditempatkan",IF(I359="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G359="","CEK ZONA NO kosong",IF(K359="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H359&lt;&gt;K359,"CEK JENIS ZONA",IF(A359="","Zona STOCK",IF(B359="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13717,7 +13717,7 @@
         <v/>
       </c>
       <c r="M360" s="12">
-        <f>IF(AND(A360="",F360=""),"",IF(F360="","Belum ditempatkan",IF(I360="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G360="","CEK ZONA NO kosong",IF(K360="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H360&lt;&gt;K360,"CEK JENIS ZONA",IF(A360="","Zona kosong",IF(B360="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A360="",F360=""),"",IF(F360="","Belum ditempatkan",IF(I360="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G360="","CEK ZONA NO kosong",IF(K360="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H360&lt;&gt;K360,"CEK JENIS ZONA",IF(A360="","Zona STOCK",IF(B360="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13747,7 +13747,7 @@
         <v/>
       </c>
       <c r="M361" s="12">
-        <f>IF(AND(A361="",F361=""),"",IF(F361="","Belum ditempatkan",IF(I361="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G361="","CEK ZONA NO kosong",IF(K361="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H361&lt;&gt;K361,"CEK JENIS ZONA",IF(A361="","Zona kosong",IF(B361="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A361="",F361=""),"",IF(F361="","Belum ditempatkan",IF(I361="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G361="","CEK ZONA NO kosong",IF(K361="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H361&lt;&gt;K361,"CEK JENIS ZONA",IF(A361="","Zona STOCK",IF(B361="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13777,7 +13777,7 @@
         <v/>
       </c>
       <c r="M362" s="12">
-        <f>IF(AND(A362="",F362=""),"",IF(F362="","Belum ditempatkan",IF(I362="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G362="","CEK ZONA NO kosong",IF(K362="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H362&lt;&gt;K362,"CEK JENIS ZONA",IF(A362="","Zona kosong",IF(B362="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A362="",F362=""),"",IF(F362="","Belum ditempatkan",IF(I362="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G362="","CEK ZONA NO kosong",IF(K362="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H362&lt;&gt;K362,"CEK JENIS ZONA",IF(A362="","Zona STOCK",IF(B362="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13807,7 +13807,7 @@
         <v/>
       </c>
       <c r="M363" s="12">
-        <f>IF(AND(A363="",F363=""),"",IF(F363="","Belum ditempatkan",IF(I363="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G363="","CEK ZONA NO kosong",IF(K363="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H363&lt;&gt;K363,"CEK JENIS ZONA",IF(A363="","Zona kosong",IF(B363="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A363="",F363=""),"",IF(F363="","Belum ditempatkan",IF(I363="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G363="","CEK ZONA NO kosong",IF(K363="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H363&lt;&gt;K363,"CEK JENIS ZONA",IF(A363="","Zona STOCK",IF(B363="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13837,7 +13837,7 @@
         <v/>
       </c>
       <c r="M364" s="12">
-        <f>IF(AND(A364="",F364=""),"",IF(F364="","Belum ditempatkan",IF(I364="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G364="","CEK ZONA NO kosong",IF(K364="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H364&lt;&gt;K364,"CEK JENIS ZONA",IF(A364="","Zona kosong",IF(B364="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A364="",F364=""),"",IF(F364="","Belum ditempatkan",IF(I364="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G364="","CEK ZONA NO kosong",IF(K364="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H364&lt;&gt;K364,"CEK JENIS ZONA",IF(A364="","Zona STOCK",IF(B364="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13867,7 +13867,7 @@
         <v/>
       </c>
       <c r="M365" s="12">
-        <f>IF(AND(A365="",F365=""),"",IF(F365="","Belum ditempatkan",IF(I365="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G365="","CEK ZONA NO kosong",IF(K365="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H365&lt;&gt;K365,"CEK JENIS ZONA",IF(A365="","Zona kosong",IF(B365="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A365="",F365=""),"",IF(F365="","Belum ditempatkan",IF(I365="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G365="","CEK ZONA NO kosong",IF(K365="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H365&lt;&gt;K365,"CEK JENIS ZONA",IF(A365="","Zona STOCK",IF(B365="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13897,7 +13897,7 @@
         <v/>
       </c>
       <c r="M366" s="12">
-        <f>IF(AND(A366="",F366=""),"",IF(F366="","Belum ditempatkan",IF(I366="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G366="","CEK ZONA NO kosong",IF(K366="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H366&lt;&gt;K366,"CEK JENIS ZONA",IF(A366="","Zona kosong",IF(B366="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A366="",F366=""),"",IF(F366="","Belum ditempatkan",IF(I366="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G366="","CEK ZONA NO kosong",IF(K366="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H366&lt;&gt;K366,"CEK JENIS ZONA",IF(A366="","Zona STOCK",IF(B366="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13927,7 +13927,7 @@
         <v/>
       </c>
       <c r="M367" s="12">
-        <f>IF(AND(A367="",F367=""),"",IF(F367="","Belum ditempatkan",IF(I367="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G367="","CEK ZONA NO kosong",IF(K367="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H367&lt;&gt;K367,"CEK JENIS ZONA",IF(A367="","Zona kosong",IF(B367="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A367="",F367=""),"",IF(F367="","Belum ditempatkan",IF(I367="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G367="","CEK ZONA NO kosong",IF(K367="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H367&lt;&gt;K367,"CEK JENIS ZONA",IF(A367="","Zona STOCK",IF(B367="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13957,7 +13957,7 @@
         <v/>
       </c>
       <c r="M368" s="12">
-        <f>IF(AND(A368="",F368=""),"",IF(F368="","Belum ditempatkan",IF(I368="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G368="","CEK ZONA NO kosong",IF(K368="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H368&lt;&gt;K368,"CEK JENIS ZONA",IF(A368="","Zona kosong",IF(B368="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A368="",F368=""),"",IF(F368="","Belum ditempatkan",IF(I368="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G368="","CEK ZONA NO kosong",IF(K368="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H368&lt;&gt;K368,"CEK JENIS ZONA",IF(A368="","Zona STOCK",IF(B368="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -13987,7 +13987,7 @@
         <v/>
       </c>
       <c r="M369" s="12">
-        <f>IF(AND(A369="",F369=""),"",IF(F369="","Belum ditempatkan",IF(I369="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G369="","CEK ZONA NO kosong",IF(K369="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H369&lt;&gt;K369,"CEK JENIS ZONA",IF(A369="","Zona kosong",IF(B369="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A369="",F369=""),"",IF(F369="","Belum ditempatkan",IF(I369="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G369="","CEK ZONA NO kosong",IF(K369="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H369&lt;&gt;K369,"CEK JENIS ZONA",IF(A369="","Zona STOCK",IF(B369="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14017,7 +14017,7 @@
         <v/>
       </c>
       <c r="M370" s="12">
-        <f>IF(AND(A370="",F370=""),"",IF(F370="","Belum ditempatkan",IF(I370="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G370="","CEK ZONA NO kosong",IF(K370="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H370&lt;&gt;K370,"CEK JENIS ZONA",IF(A370="","Zona kosong",IF(B370="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A370="",F370=""),"",IF(F370="","Belum ditempatkan",IF(I370="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G370="","CEK ZONA NO kosong",IF(K370="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H370&lt;&gt;K370,"CEK JENIS ZONA",IF(A370="","Zona STOCK",IF(B370="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14047,7 +14047,7 @@
         <v/>
       </c>
       <c r="M371" s="12">
-        <f>IF(AND(A371="",F371=""),"",IF(F371="","Belum ditempatkan",IF(I371="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G371="","CEK ZONA NO kosong",IF(K371="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H371&lt;&gt;K371,"CEK JENIS ZONA",IF(A371="","Zona kosong",IF(B371="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A371="",F371=""),"",IF(F371="","Belum ditempatkan",IF(I371="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G371="","CEK ZONA NO kosong",IF(K371="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H371&lt;&gt;K371,"CEK JENIS ZONA",IF(A371="","Zona STOCK",IF(B371="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14077,7 +14077,7 @@
         <v/>
       </c>
       <c r="M372" s="12">
-        <f>IF(AND(A372="",F372=""),"",IF(F372="","Belum ditempatkan",IF(I372="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G372="","CEK ZONA NO kosong",IF(K372="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H372&lt;&gt;K372,"CEK JENIS ZONA",IF(A372="","Zona kosong",IF(B372="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A372="",F372=""),"",IF(F372="","Belum ditempatkan",IF(I372="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G372="","CEK ZONA NO kosong",IF(K372="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H372&lt;&gt;K372,"CEK JENIS ZONA",IF(A372="","Zona STOCK",IF(B372="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14107,7 +14107,7 @@
         <v/>
       </c>
       <c r="M373" s="12">
-        <f>IF(AND(A373="",F373=""),"",IF(F373="","Belum ditempatkan",IF(I373="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G373="","CEK ZONA NO kosong",IF(K373="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H373&lt;&gt;K373,"CEK JENIS ZONA",IF(A373="","Zona kosong",IF(B373="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A373="",F373=""),"",IF(F373="","Belum ditempatkan",IF(I373="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G373="","CEK ZONA NO kosong",IF(K373="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H373&lt;&gt;K373,"CEK JENIS ZONA",IF(A373="","Zona STOCK",IF(B373="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14137,7 +14137,7 @@
         <v/>
       </c>
       <c r="M374" s="12">
-        <f>IF(AND(A374="",F374=""),"",IF(F374="","Belum ditempatkan",IF(I374="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G374="","CEK ZONA NO kosong",IF(K374="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H374&lt;&gt;K374,"CEK JENIS ZONA",IF(A374="","Zona kosong",IF(B374="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A374="",F374=""),"",IF(F374="","Belum ditempatkan",IF(I374="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G374="","CEK ZONA NO kosong",IF(K374="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H374&lt;&gt;K374,"CEK JENIS ZONA",IF(A374="","Zona STOCK",IF(B374="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14167,7 +14167,7 @@
         <v/>
       </c>
       <c r="M375" s="12">
-        <f>IF(AND(A375="",F375=""),"",IF(F375="","Belum ditempatkan",IF(I375="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G375="","CEK ZONA NO kosong",IF(K375="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H375&lt;&gt;K375,"CEK JENIS ZONA",IF(A375="","Zona kosong",IF(B375="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A375="",F375=""),"",IF(F375="","Belum ditempatkan",IF(I375="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G375="","CEK ZONA NO kosong",IF(K375="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H375&lt;&gt;K375,"CEK JENIS ZONA",IF(A375="","Zona STOCK",IF(B375="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14197,7 +14197,7 @@
         <v/>
       </c>
       <c r="M376" s="12">
-        <f>IF(AND(A376="",F376=""),"",IF(F376="","Belum ditempatkan",IF(I376="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G376="","CEK ZONA NO kosong",IF(K376="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H376&lt;&gt;K376,"CEK JENIS ZONA",IF(A376="","Zona kosong",IF(B376="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A376="",F376=""),"",IF(F376="","Belum ditempatkan",IF(I376="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G376="","CEK ZONA NO kosong",IF(K376="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H376&lt;&gt;K376,"CEK JENIS ZONA",IF(A376="","Zona STOCK",IF(B376="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14227,7 +14227,7 @@
         <v/>
       </c>
       <c r="M377" s="12">
-        <f>IF(AND(A377="",F377=""),"",IF(F377="","Belum ditempatkan",IF(I377="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G377="","CEK ZONA NO kosong",IF(K377="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H377&lt;&gt;K377,"CEK JENIS ZONA",IF(A377="","Zona kosong",IF(B377="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A377="",F377=""),"",IF(F377="","Belum ditempatkan",IF(I377="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G377="","CEK ZONA NO kosong",IF(K377="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H377&lt;&gt;K377,"CEK JENIS ZONA",IF(A377="","Zona STOCK",IF(B377="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14257,7 +14257,7 @@
         <v/>
       </c>
       <c r="M378" s="12">
-        <f>IF(AND(A378="",F378=""),"",IF(F378="","Belum ditempatkan",IF(I378="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G378="","CEK ZONA NO kosong",IF(K378="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H378&lt;&gt;K378,"CEK JENIS ZONA",IF(A378="","Zona kosong",IF(B378="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A378="",F378=""),"",IF(F378="","Belum ditempatkan",IF(I378="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G378="","CEK ZONA NO kosong",IF(K378="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H378&lt;&gt;K378,"CEK JENIS ZONA",IF(A378="","Zona STOCK",IF(B378="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="M379" s="12">
-        <f>IF(AND(A379="",F379=""),"",IF(F379="","Belum ditempatkan",IF(I379="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G379="","CEK ZONA NO kosong",IF(K379="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H379&lt;&gt;K379,"CEK JENIS ZONA",IF(A379="","Zona kosong",IF(B379="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A379="",F379=""),"",IF(F379="","Belum ditempatkan",IF(I379="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G379="","CEK ZONA NO kosong",IF(K379="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H379&lt;&gt;K379,"CEK JENIS ZONA",IF(A379="","Zona STOCK",IF(B379="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14317,7 +14317,7 @@
         <v/>
       </c>
       <c r="M380" s="12">
-        <f>IF(AND(A380="",F380=""),"",IF(F380="","Belum ditempatkan",IF(I380="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G380="","CEK ZONA NO kosong",IF(K380="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H380&lt;&gt;K380,"CEK JENIS ZONA",IF(A380="","Zona kosong",IF(B380="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A380="",F380=""),"",IF(F380="","Belum ditempatkan",IF(I380="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G380="","CEK ZONA NO kosong",IF(K380="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H380&lt;&gt;K380,"CEK JENIS ZONA",IF(A380="","Zona STOCK",IF(B380="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14347,7 +14347,7 @@
         <v/>
       </c>
       <c r="M381" s="12">
-        <f>IF(AND(A381="",F381=""),"",IF(F381="","Belum ditempatkan",IF(I381="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G381="","CEK ZONA NO kosong",IF(K381="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H381&lt;&gt;K381,"CEK JENIS ZONA",IF(A381="","Zona kosong",IF(B381="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A381="",F381=""),"",IF(F381="","Belum ditempatkan",IF(I381="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G381="","CEK ZONA NO kosong",IF(K381="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H381&lt;&gt;K381,"CEK JENIS ZONA",IF(A381="","Zona STOCK",IF(B381="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14377,7 +14377,7 @@
         <v/>
       </c>
       <c r="M382" s="12">
-        <f>IF(AND(A382="",F382=""),"",IF(F382="","Belum ditempatkan",IF(I382="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G382="","CEK ZONA NO kosong",IF(K382="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H382&lt;&gt;K382,"CEK JENIS ZONA",IF(A382="","Zona kosong",IF(B382="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A382="",F382=""),"",IF(F382="","Belum ditempatkan",IF(I382="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G382="","CEK ZONA NO kosong",IF(K382="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H382&lt;&gt;K382,"CEK JENIS ZONA",IF(A382="","Zona STOCK",IF(B382="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14407,7 +14407,7 @@
         <v/>
       </c>
       <c r="M383" s="12">
-        <f>IF(AND(A383="",F383=""),"",IF(F383="","Belum ditempatkan",IF(I383="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G383="","CEK ZONA NO kosong",IF(K383="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H383&lt;&gt;K383,"CEK JENIS ZONA",IF(A383="","Zona kosong",IF(B383="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A383="",F383=""),"",IF(F383="","Belum ditempatkan",IF(I383="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G383="","CEK ZONA NO kosong",IF(K383="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H383&lt;&gt;K383,"CEK JENIS ZONA",IF(A383="","Zona STOCK",IF(B383="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14437,7 +14437,7 @@
         <v/>
       </c>
       <c r="M384" s="12">
-        <f>IF(AND(A384="",F384=""),"",IF(F384="","Belum ditempatkan",IF(I384="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G384="","CEK ZONA NO kosong",IF(K384="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H384&lt;&gt;K384,"CEK JENIS ZONA",IF(A384="","Zona kosong",IF(B384="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A384="",F384=""),"",IF(F384="","Belum ditempatkan",IF(I384="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G384="","CEK ZONA NO kosong",IF(K384="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H384&lt;&gt;K384,"CEK JENIS ZONA",IF(A384="","Zona STOCK",IF(B384="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14467,7 +14467,7 @@
         <v/>
       </c>
       <c r="M385" s="12">
-        <f>IF(AND(A385="",F385=""),"",IF(F385="","Belum ditempatkan",IF(I385="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G385="","CEK ZONA NO kosong",IF(K385="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H385&lt;&gt;K385,"CEK JENIS ZONA",IF(A385="","Zona kosong",IF(B385="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A385="",F385=""),"",IF(F385="","Belum ditempatkan",IF(I385="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G385="","CEK ZONA NO kosong",IF(K385="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H385&lt;&gt;K385,"CEK JENIS ZONA",IF(A385="","Zona STOCK",IF(B385="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14497,7 +14497,7 @@
         <v/>
       </c>
       <c r="M386" s="12">
-        <f>IF(AND(A386="",F386=""),"",IF(F386="","Belum ditempatkan",IF(I386="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G386="","CEK ZONA NO kosong",IF(K386="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H386&lt;&gt;K386,"CEK JENIS ZONA",IF(A386="","Zona kosong",IF(B386="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A386="",F386=""),"",IF(F386="","Belum ditempatkan",IF(I386="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G386="","CEK ZONA NO kosong",IF(K386="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H386&lt;&gt;K386,"CEK JENIS ZONA",IF(A386="","Zona STOCK",IF(B386="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14527,7 +14527,7 @@
         <v/>
       </c>
       <c r="M387" s="12">
-        <f>IF(AND(A387="",F387=""),"",IF(F387="","Belum ditempatkan",IF(I387="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G387="","CEK ZONA NO kosong",IF(K387="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H387&lt;&gt;K387,"CEK JENIS ZONA",IF(A387="","Zona kosong",IF(B387="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A387="",F387=""),"",IF(F387="","Belum ditempatkan",IF(I387="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G387="","CEK ZONA NO kosong",IF(K387="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H387&lt;&gt;K387,"CEK JENIS ZONA",IF(A387="","Zona STOCK",IF(B387="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14557,7 +14557,7 @@
         <v/>
       </c>
       <c r="M388" s="12">
-        <f>IF(AND(A388="",F388=""),"",IF(F388="","Belum ditempatkan",IF(I388="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G388="","CEK ZONA NO kosong",IF(K388="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H388&lt;&gt;K388,"CEK JENIS ZONA",IF(A388="","Zona kosong",IF(B388="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A388="",F388=""),"",IF(F388="","Belum ditempatkan",IF(I388="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G388="","CEK ZONA NO kosong",IF(K388="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H388&lt;&gt;K388,"CEK JENIS ZONA",IF(A388="","Zona STOCK",IF(B388="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14587,7 +14587,7 @@
         <v/>
       </c>
       <c r="M389" s="12">
-        <f>IF(AND(A389="",F389=""),"",IF(F389="","Belum ditempatkan",IF(I389="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G389="","CEK ZONA NO kosong",IF(K389="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H389&lt;&gt;K389,"CEK JENIS ZONA",IF(A389="","Zona kosong",IF(B389="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A389="",F389=""),"",IF(F389="","Belum ditempatkan",IF(I389="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G389="","CEK ZONA NO kosong",IF(K389="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H389&lt;&gt;K389,"CEK JENIS ZONA",IF(A389="","Zona STOCK",IF(B389="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14617,7 +14617,7 @@
         <v/>
       </c>
       <c r="M390" s="12">
-        <f>IF(AND(A390="",F390=""),"",IF(F390="","Belum ditempatkan",IF(I390="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G390="","CEK ZONA NO kosong",IF(K390="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H390&lt;&gt;K390,"CEK JENIS ZONA",IF(A390="","Zona kosong",IF(B390="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A390="",F390=""),"",IF(F390="","Belum ditempatkan",IF(I390="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G390="","CEK ZONA NO kosong",IF(K390="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H390&lt;&gt;K390,"CEK JENIS ZONA",IF(A390="","Zona STOCK",IF(B390="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14647,7 +14647,7 @@
         <v/>
       </c>
       <c r="M391" s="12">
-        <f>IF(AND(A391="",F391=""),"",IF(F391="","Belum ditempatkan",IF(I391="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G391="","CEK ZONA NO kosong",IF(K391="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H391&lt;&gt;K391,"CEK JENIS ZONA",IF(A391="","Zona kosong",IF(B391="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A391="",F391=""),"",IF(F391="","Belum ditempatkan",IF(I391="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G391="","CEK ZONA NO kosong",IF(K391="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H391&lt;&gt;K391,"CEK JENIS ZONA",IF(A391="","Zona STOCK",IF(B391="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14677,7 +14677,7 @@
         <v/>
       </c>
       <c r="M392" s="12">
-        <f>IF(AND(A392="",F392=""),"",IF(F392="","Belum ditempatkan",IF(I392="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G392="","CEK ZONA NO kosong",IF(K392="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H392&lt;&gt;K392,"CEK JENIS ZONA",IF(A392="","Zona kosong",IF(B392="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A392="",F392=""),"",IF(F392="","Belum ditempatkan",IF(I392="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G392="","CEK ZONA NO kosong",IF(K392="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H392&lt;&gt;K392,"CEK JENIS ZONA",IF(A392="","Zona STOCK",IF(B392="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14707,7 +14707,7 @@
         <v/>
       </c>
       <c r="M393" s="12">
-        <f>IF(AND(A393="",F393=""),"",IF(F393="","Belum ditempatkan",IF(I393="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G393="","CEK ZONA NO kosong",IF(K393="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H393&lt;&gt;K393,"CEK JENIS ZONA",IF(A393="","Zona kosong",IF(B393="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A393="",F393=""),"",IF(F393="","Belum ditempatkan",IF(I393="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G393="","CEK ZONA NO kosong",IF(K393="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H393&lt;&gt;K393,"CEK JENIS ZONA",IF(A393="","Zona STOCK",IF(B393="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14737,7 +14737,7 @@
         <v/>
       </c>
       <c r="M394" s="12">
-        <f>IF(AND(A394="",F394=""),"",IF(F394="","Belum ditempatkan",IF(I394="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G394="","CEK ZONA NO kosong",IF(K394="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H394&lt;&gt;K394,"CEK JENIS ZONA",IF(A394="","Zona kosong",IF(B394="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A394="",F394=""),"",IF(F394="","Belum ditempatkan",IF(I394="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G394="","CEK ZONA NO kosong",IF(K394="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H394&lt;&gt;K394,"CEK JENIS ZONA",IF(A394="","Zona STOCK",IF(B394="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14767,7 +14767,7 @@
         <v/>
       </c>
       <c r="M395" s="12">
-        <f>IF(AND(A395="",F395=""),"",IF(F395="","Belum ditempatkan",IF(I395="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G395="","CEK ZONA NO kosong",IF(K395="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H395&lt;&gt;K395,"CEK JENIS ZONA",IF(A395="","Zona kosong",IF(B395="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A395="",F395=""),"",IF(F395="","Belum ditempatkan",IF(I395="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G395="","CEK ZONA NO kosong",IF(K395="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H395&lt;&gt;K395,"CEK JENIS ZONA",IF(A395="","Zona STOCK",IF(B395="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14797,7 +14797,7 @@
         <v/>
       </c>
       <c r="M396" s="12">
-        <f>IF(AND(A396="",F396=""),"",IF(F396="","Belum ditempatkan",IF(I396="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G396="","CEK ZONA NO kosong",IF(K396="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H396&lt;&gt;K396,"CEK JENIS ZONA",IF(A396="","Zona kosong",IF(B396="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A396="",F396=""),"",IF(F396="","Belum ditempatkan",IF(I396="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G396="","CEK ZONA NO kosong",IF(K396="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H396&lt;&gt;K396,"CEK JENIS ZONA",IF(A396="","Zona STOCK",IF(B396="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14827,7 +14827,7 @@
         <v/>
       </c>
       <c r="M397" s="12">
-        <f>IF(AND(A397="",F397=""),"",IF(F397="","Belum ditempatkan",IF(I397="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G397="","CEK ZONA NO kosong",IF(K397="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H397&lt;&gt;K397,"CEK JENIS ZONA",IF(A397="","Zona kosong",IF(B397="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A397="",F397=""),"",IF(F397="","Belum ditempatkan",IF(I397="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G397="","CEK ZONA NO kosong",IF(K397="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H397&lt;&gt;K397,"CEK JENIS ZONA",IF(A397="","Zona STOCK",IF(B397="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14857,7 +14857,7 @@
         <v/>
       </c>
       <c r="M398" s="12">
-        <f>IF(AND(A398="",F398=""),"",IF(F398="","Belum ditempatkan",IF(I398="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G398="","CEK ZONA NO kosong",IF(K398="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H398&lt;&gt;K398,"CEK JENIS ZONA",IF(A398="","Zona kosong",IF(B398="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A398="",F398=""),"",IF(F398="","Belum ditempatkan",IF(I398="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G398="","CEK ZONA NO kosong",IF(K398="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H398&lt;&gt;K398,"CEK JENIS ZONA",IF(A398="","Zona STOCK",IF(B398="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14887,7 +14887,7 @@
         <v/>
       </c>
       <c r="M399" s="12">
-        <f>IF(AND(A399="",F399=""),"",IF(F399="","Belum ditempatkan",IF(I399="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G399="","CEK ZONA NO kosong",IF(K399="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H399&lt;&gt;K399,"CEK JENIS ZONA",IF(A399="","Zona kosong",IF(B399="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A399="",F399=""),"",IF(F399="","Belum ditempatkan",IF(I399="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G399="","CEK ZONA NO kosong",IF(K399="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H399&lt;&gt;K399,"CEK JENIS ZONA",IF(A399="","Zona STOCK",IF(B399="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14917,7 +14917,7 @@
         <v/>
       </c>
       <c r="M400" s="12">
-        <f>IF(AND(A400="",F400=""),"",IF(F400="","Belum ditempatkan",IF(I400="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G400="","CEK ZONA NO kosong",IF(K400="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H400&lt;&gt;K400,"CEK JENIS ZONA",IF(A400="","Zona kosong",IF(B400="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A400="",F400=""),"",IF(F400="","Belum ditempatkan",IF(I400="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G400="","CEK ZONA NO kosong",IF(K400="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H400&lt;&gt;K400,"CEK JENIS ZONA",IF(A400="","Zona STOCK",IF(B400="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14947,7 +14947,7 @@
         <v/>
       </c>
       <c r="M401" s="12">
-        <f>IF(AND(A401="",F401=""),"",IF(F401="","Belum ditempatkan",IF(I401="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G401="","CEK ZONA NO kosong",IF(K401="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H401&lt;&gt;K401,"CEK JENIS ZONA",IF(A401="","Zona kosong",IF(B401="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A401="",F401=""),"",IF(F401="","Belum ditempatkan",IF(I401="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G401="","CEK ZONA NO kosong",IF(K401="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H401&lt;&gt;K401,"CEK JENIS ZONA",IF(A401="","Zona STOCK",IF(B401="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -14977,7 +14977,7 @@
         <v/>
       </c>
       <c r="M402" s="12">
-        <f>IF(AND(A402="",F402=""),"",IF(F402="","Belum ditempatkan",IF(I402="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G402="","CEK ZONA NO kosong",IF(K402="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H402&lt;&gt;K402,"CEK JENIS ZONA",IF(A402="","Zona kosong",IF(B402="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A402="",F402=""),"",IF(F402="","Belum ditempatkan",IF(I402="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G402="","CEK ZONA NO kosong",IF(K402="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H402&lt;&gt;K402,"CEK JENIS ZONA",IF(A402="","Zona STOCK",IF(B402="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15007,7 +15007,7 @@
         <v/>
       </c>
       <c r="M403" s="12">
-        <f>IF(AND(A403="",F403=""),"",IF(F403="","Belum ditempatkan",IF(I403="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G403="","CEK ZONA NO kosong",IF(K403="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H403&lt;&gt;K403,"CEK JENIS ZONA",IF(A403="","Zona kosong",IF(B403="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A403="",F403=""),"",IF(F403="","Belum ditempatkan",IF(I403="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G403="","CEK ZONA NO kosong",IF(K403="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H403&lt;&gt;K403,"CEK JENIS ZONA",IF(A403="","Zona STOCK",IF(B403="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="M404" s="12">
-        <f>IF(AND(A404="",F404=""),"",IF(F404="","Belum ditempatkan",IF(I404="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G404="","CEK ZONA NO kosong",IF(K404="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H404&lt;&gt;K404,"CEK JENIS ZONA",IF(A404="","Zona kosong",IF(B404="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A404="",F404=""),"",IF(F404="","Belum ditempatkan",IF(I404="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G404="","CEK ZONA NO kosong",IF(K404="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H404&lt;&gt;K404,"CEK JENIS ZONA",IF(A404="","Zona STOCK",IF(B404="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15067,7 +15067,7 @@
         <v/>
       </c>
       <c r="M405" s="12">
-        <f>IF(AND(A405="",F405=""),"",IF(F405="","Belum ditempatkan",IF(I405="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G405="","CEK ZONA NO kosong",IF(K405="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H405&lt;&gt;K405,"CEK JENIS ZONA",IF(A405="","Zona kosong",IF(B405="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A405="",F405=""),"",IF(F405="","Belum ditempatkan",IF(I405="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G405="","CEK ZONA NO kosong",IF(K405="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H405&lt;&gt;K405,"CEK JENIS ZONA",IF(A405="","Zona STOCK",IF(B405="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15097,7 +15097,7 @@
         <v/>
       </c>
       <c r="M406" s="12">
-        <f>IF(AND(A406="",F406=""),"",IF(F406="","Belum ditempatkan",IF(I406="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G406="","CEK ZONA NO kosong",IF(K406="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H406&lt;&gt;K406,"CEK JENIS ZONA",IF(A406="","Zona kosong",IF(B406="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A406="",F406=""),"",IF(F406="","Belum ditempatkan",IF(I406="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G406="","CEK ZONA NO kosong",IF(K406="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H406&lt;&gt;K406,"CEK JENIS ZONA",IF(A406="","Zona STOCK",IF(B406="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15127,7 +15127,7 @@
         <v/>
       </c>
       <c r="M407" s="12">
-        <f>IF(AND(A407="",F407=""),"",IF(F407="","Belum ditempatkan",IF(I407="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G407="","CEK ZONA NO kosong",IF(K407="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H407&lt;&gt;K407,"CEK JENIS ZONA",IF(A407="","Zona kosong",IF(B407="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A407="",F407=""),"",IF(F407="","Belum ditempatkan",IF(I407="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G407="","CEK ZONA NO kosong",IF(K407="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H407&lt;&gt;K407,"CEK JENIS ZONA",IF(A407="","Zona STOCK",IF(B407="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15157,7 +15157,7 @@
         <v/>
       </c>
       <c r="M408" s="12">
-        <f>IF(AND(A408="",F408=""),"",IF(F408="","Belum ditempatkan",IF(I408="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G408="","CEK ZONA NO kosong",IF(K408="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H408&lt;&gt;K408,"CEK JENIS ZONA",IF(A408="","Zona kosong",IF(B408="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A408="",F408=""),"",IF(F408="","Belum ditempatkan",IF(I408="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G408="","CEK ZONA NO kosong",IF(K408="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H408&lt;&gt;K408,"CEK JENIS ZONA",IF(A408="","Zona STOCK",IF(B408="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15187,7 +15187,7 @@
         <v/>
       </c>
       <c r="M409" s="12">
-        <f>IF(AND(A409="",F409=""),"",IF(F409="","Belum ditempatkan",IF(I409="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G409="","CEK ZONA NO kosong",IF(K409="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H409&lt;&gt;K409,"CEK JENIS ZONA",IF(A409="","Zona kosong",IF(B409="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A409="",F409=""),"",IF(F409="","Belum ditempatkan",IF(I409="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G409="","CEK ZONA NO kosong",IF(K409="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H409&lt;&gt;K409,"CEK JENIS ZONA",IF(A409="","Zona STOCK",IF(B409="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15217,7 +15217,7 @@
         <v/>
       </c>
       <c r="M410" s="12">
-        <f>IF(AND(A410="",F410=""),"",IF(F410="","Belum ditempatkan",IF(I410="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G410="","CEK ZONA NO kosong",IF(K410="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H410&lt;&gt;K410,"CEK JENIS ZONA",IF(A410="","Zona kosong",IF(B410="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A410="",F410=""),"",IF(F410="","Belum ditempatkan",IF(I410="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G410="","CEK ZONA NO kosong",IF(K410="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H410&lt;&gt;K410,"CEK JENIS ZONA",IF(A410="","Zona STOCK",IF(B410="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15247,7 +15247,7 @@
         <v/>
       </c>
       <c r="M411" s="12">
-        <f>IF(AND(A411="",F411=""),"",IF(F411="","Belum ditempatkan",IF(I411="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G411="","CEK ZONA NO kosong",IF(K411="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H411&lt;&gt;K411,"CEK JENIS ZONA",IF(A411="","Zona kosong",IF(B411="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A411="",F411=""),"",IF(F411="","Belum ditempatkan",IF(I411="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G411="","CEK ZONA NO kosong",IF(K411="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H411&lt;&gt;K411,"CEK JENIS ZONA",IF(A411="","Zona STOCK",IF(B411="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15277,7 +15277,7 @@
         <v/>
       </c>
       <c r="M412" s="12">
-        <f>IF(AND(A412="",F412=""),"",IF(F412="","Belum ditempatkan",IF(I412="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G412="","CEK ZONA NO kosong",IF(K412="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H412&lt;&gt;K412,"CEK JENIS ZONA",IF(A412="","Zona kosong",IF(B412="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A412="",F412=""),"",IF(F412="","Belum ditempatkan",IF(I412="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G412="","CEK ZONA NO kosong",IF(K412="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H412&lt;&gt;K412,"CEK JENIS ZONA",IF(A412="","Zona STOCK",IF(B412="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15307,7 +15307,7 @@
         <v/>
       </c>
       <c r="M413" s="12">
-        <f>IF(AND(A413="",F413=""),"",IF(F413="","Belum ditempatkan",IF(I413="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G413="","CEK ZONA NO kosong",IF(K413="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H413&lt;&gt;K413,"CEK JENIS ZONA",IF(A413="","Zona kosong",IF(B413="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A413="",F413=""),"",IF(F413="","Belum ditempatkan",IF(I413="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G413="","CEK ZONA NO kosong",IF(K413="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H413&lt;&gt;K413,"CEK JENIS ZONA",IF(A413="","Zona STOCK",IF(B413="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15337,7 +15337,7 @@
         <v/>
       </c>
       <c r="M414" s="12">
-        <f>IF(AND(A414="",F414=""),"",IF(F414="","Belum ditempatkan",IF(I414="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G414="","CEK ZONA NO kosong",IF(K414="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H414&lt;&gt;K414,"CEK JENIS ZONA",IF(A414="","Zona kosong",IF(B414="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A414="",F414=""),"",IF(F414="","Belum ditempatkan",IF(I414="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G414="","CEK ZONA NO kosong",IF(K414="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H414&lt;&gt;K414,"CEK JENIS ZONA",IF(A414="","Zona STOCK",IF(B414="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15367,7 +15367,7 @@
         <v/>
       </c>
       <c r="M415" s="12">
-        <f>IF(AND(A415="",F415=""),"",IF(F415="","Belum ditempatkan",IF(I415="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G415="","CEK ZONA NO kosong",IF(K415="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H415&lt;&gt;K415,"CEK JENIS ZONA",IF(A415="","Zona kosong",IF(B415="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A415="",F415=""),"",IF(F415="","Belum ditempatkan",IF(I415="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G415="","CEK ZONA NO kosong",IF(K415="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H415&lt;&gt;K415,"CEK JENIS ZONA",IF(A415="","Zona STOCK",IF(B415="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15397,7 +15397,7 @@
         <v/>
       </c>
       <c r="M416" s="12">
-        <f>IF(AND(A416="",F416=""),"",IF(F416="","Belum ditempatkan",IF(I416="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G416="","CEK ZONA NO kosong",IF(K416="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H416&lt;&gt;K416,"CEK JENIS ZONA",IF(A416="","Zona kosong",IF(B416="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A416="",F416=""),"",IF(F416="","Belum ditempatkan",IF(I416="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G416="","CEK ZONA NO kosong",IF(K416="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H416&lt;&gt;K416,"CEK JENIS ZONA",IF(A416="","Zona STOCK",IF(B416="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15427,7 +15427,7 @@
         <v/>
       </c>
       <c r="M417" s="12">
-        <f>IF(AND(A417="",F417=""),"",IF(F417="","Belum ditempatkan",IF(I417="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G417="","CEK ZONA NO kosong",IF(K417="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H417&lt;&gt;K417,"CEK JENIS ZONA",IF(A417="","Zona kosong",IF(B417="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A417="",F417=""),"",IF(F417="","Belum ditempatkan",IF(I417="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G417="","CEK ZONA NO kosong",IF(K417="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H417&lt;&gt;K417,"CEK JENIS ZONA",IF(A417="","Zona STOCK",IF(B417="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15457,7 +15457,7 @@
         <v/>
       </c>
       <c r="M418" s="12">
-        <f>IF(AND(A418="",F418=""),"",IF(F418="","Belum ditempatkan",IF(I418="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G418="","CEK ZONA NO kosong",IF(K418="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H418&lt;&gt;K418,"CEK JENIS ZONA",IF(A418="","Zona kosong",IF(B418="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A418="",F418=""),"",IF(F418="","Belum ditempatkan",IF(I418="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G418="","CEK ZONA NO kosong",IF(K418="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H418&lt;&gt;K418,"CEK JENIS ZONA",IF(A418="","Zona STOCK",IF(B418="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15487,7 +15487,7 @@
         <v/>
       </c>
       <c r="M419" s="12">
-        <f>IF(AND(A419="",F419=""),"",IF(F419="","Belum ditempatkan",IF(I419="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G419="","CEK ZONA NO kosong",IF(K419="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H419&lt;&gt;K419,"CEK JENIS ZONA",IF(A419="","Zona kosong",IF(B419="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A419="",F419=""),"",IF(F419="","Belum ditempatkan",IF(I419="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G419="","CEK ZONA NO kosong",IF(K419="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H419&lt;&gt;K419,"CEK JENIS ZONA",IF(A419="","Zona STOCK",IF(B419="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15517,7 +15517,7 @@
         <v/>
       </c>
       <c r="M420" s="12">
-        <f>IF(AND(A420="",F420=""),"",IF(F420="","Belum ditempatkan",IF(I420="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G420="","CEK ZONA NO kosong",IF(K420="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H420&lt;&gt;K420,"CEK JENIS ZONA",IF(A420="","Zona kosong",IF(B420="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A420="",F420=""),"",IF(F420="","Belum ditempatkan",IF(I420="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G420="","CEK ZONA NO kosong",IF(K420="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H420&lt;&gt;K420,"CEK JENIS ZONA",IF(A420="","Zona STOCK",IF(B420="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15547,7 +15547,7 @@
         <v/>
       </c>
       <c r="M421" s="12">
-        <f>IF(AND(A421="",F421=""),"",IF(F421="","Belum ditempatkan",IF(I421="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G421="","CEK ZONA NO kosong",IF(K421="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H421&lt;&gt;K421,"CEK JENIS ZONA",IF(A421="","Zona kosong",IF(B421="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A421="",F421=""),"",IF(F421="","Belum ditempatkan",IF(I421="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G421="","CEK ZONA NO kosong",IF(K421="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H421&lt;&gt;K421,"CEK JENIS ZONA",IF(A421="","Zona STOCK",IF(B421="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15577,7 +15577,7 @@
         <v/>
       </c>
       <c r="M422" s="12">
-        <f>IF(AND(A422="",F422=""),"",IF(F422="","Belum ditempatkan",IF(I422="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G422="","CEK ZONA NO kosong",IF(K422="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H422&lt;&gt;K422,"CEK JENIS ZONA",IF(A422="","Zona kosong",IF(B422="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A422="",F422=""),"",IF(F422="","Belum ditempatkan",IF(I422="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G422="","CEK ZONA NO kosong",IF(K422="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H422&lt;&gt;K422,"CEK JENIS ZONA",IF(A422="","Zona STOCK",IF(B422="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15607,7 +15607,7 @@
         <v/>
       </c>
       <c r="M423" s="12">
-        <f>IF(AND(A423="",F423=""),"",IF(F423="","Belum ditempatkan",IF(I423="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G423="","CEK ZONA NO kosong",IF(K423="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H423&lt;&gt;K423,"CEK JENIS ZONA",IF(A423="","Zona kosong",IF(B423="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A423="",F423=""),"",IF(F423="","Belum ditempatkan",IF(I423="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G423="","CEK ZONA NO kosong",IF(K423="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H423&lt;&gt;K423,"CEK JENIS ZONA",IF(A423="","Zona STOCK",IF(B423="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15637,7 +15637,7 @@
         <v/>
       </c>
       <c r="M424" s="12">
-        <f>IF(AND(A424="",F424=""),"",IF(F424="","Belum ditempatkan",IF(I424="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G424="","CEK ZONA NO kosong",IF(K424="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H424&lt;&gt;K424,"CEK JENIS ZONA",IF(A424="","Zona kosong",IF(B424="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A424="",F424=""),"",IF(F424="","Belum ditempatkan",IF(I424="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G424="","CEK ZONA NO kosong",IF(K424="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H424&lt;&gt;K424,"CEK JENIS ZONA",IF(A424="","Zona STOCK",IF(B424="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15667,7 +15667,7 @@
         <v/>
       </c>
       <c r="M425" s="12">
-        <f>IF(AND(A425="",F425=""),"",IF(F425="","Belum ditempatkan",IF(I425="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G425="","CEK ZONA NO kosong",IF(K425="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H425&lt;&gt;K425,"CEK JENIS ZONA",IF(A425="","Zona kosong",IF(B425="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A425="",F425=""),"",IF(F425="","Belum ditempatkan",IF(I425="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G425="","CEK ZONA NO kosong",IF(K425="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H425&lt;&gt;K425,"CEK JENIS ZONA",IF(A425="","Zona STOCK",IF(B425="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15697,7 +15697,7 @@
         <v/>
       </c>
       <c r="M426" s="12">
-        <f>IF(AND(A426="",F426=""),"",IF(F426="","Belum ditempatkan",IF(I426="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G426="","CEK ZONA NO kosong",IF(K426="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H426&lt;&gt;K426,"CEK JENIS ZONA",IF(A426="","Zona kosong",IF(B426="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A426="",F426=""),"",IF(F426="","Belum ditempatkan",IF(I426="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G426="","CEK ZONA NO kosong",IF(K426="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H426&lt;&gt;K426,"CEK JENIS ZONA",IF(A426="","Zona STOCK",IF(B426="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15727,7 +15727,7 @@
         <v/>
       </c>
       <c r="M427" s="12">
-        <f>IF(AND(A427="",F427=""),"",IF(F427="","Belum ditempatkan",IF(I427="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G427="","CEK ZONA NO kosong",IF(K427="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H427&lt;&gt;K427,"CEK JENIS ZONA",IF(A427="","Zona kosong",IF(B427="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A427="",F427=""),"",IF(F427="","Belum ditempatkan",IF(I427="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G427="","CEK ZONA NO kosong",IF(K427="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H427&lt;&gt;K427,"CEK JENIS ZONA",IF(A427="","Zona STOCK",IF(B427="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15757,7 +15757,7 @@
         <v/>
       </c>
       <c r="M428" s="12">
-        <f>IF(AND(A428="",F428=""),"",IF(F428="","Belum ditempatkan",IF(I428="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G428="","CEK ZONA NO kosong",IF(K428="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H428&lt;&gt;K428,"CEK JENIS ZONA",IF(A428="","Zona kosong",IF(B428="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A428="",F428=""),"",IF(F428="","Belum ditempatkan",IF(I428="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G428="","CEK ZONA NO kosong",IF(K428="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H428&lt;&gt;K428,"CEK JENIS ZONA",IF(A428="","Zona STOCK",IF(B428="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15787,7 +15787,7 @@
         <v/>
       </c>
       <c r="M429" s="12">
-        <f>IF(AND(A429="",F429=""),"",IF(F429="","Belum ditempatkan",IF(I429="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G429="","CEK ZONA NO kosong",IF(K429="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H429&lt;&gt;K429,"CEK JENIS ZONA",IF(A429="","Zona kosong",IF(B429="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A429="",F429=""),"",IF(F429="","Belum ditempatkan",IF(I429="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G429="","CEK ZONA NO kosong",IF(K429="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H429&lt;&gt;K429,"CEK JENIS ZONA",IF(A429="","Zona STOCK",IF(B429="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15817,7 +15817,7 @@
         <v/>
       </c>
       <c r="M430" s="12">
-        <f>IF(AND(A430="",F430=""),"",IF(F430="","Belum ditempatkan",IF(I430="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G430="","CEK ZONA NO kosong",IF(K430="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H430&lt;&gt;K430,"CEK JENIS ZONA",IF(A430="","Zona kosong",IF(B430="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A430="",F430=""),"",IF(F430="","Belum ditempatkan",IF(I430="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G430="","CEK ZONA NO kosong",IF(K430="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H430&lt;&gt;K430,"CEK JENIS ZONA",IF(A430="","Zona STOCK",IF(B430="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15847,7 +15847,7 @@
         <v/>
       </c>
       <c r="M431" s="12">
-        <f>IF(AND(A431="",F431=""),"",IF(F431="","Belum ditempatkan",IF(I431="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G431="","CEK ZONA NO kosong",IF(K431="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H431&lt;&gt;K431,"CEK JENIS ZONA",IF(A431="","Zona kosong",IF(B431="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A431="",F431=""),"",IF(F431="","Belum ditempatkan",IF(I431="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G431="","CEK ZONA NO kosong",IF(K431="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H431&lt;&gt;K431,"CEK JENIS ZONA",IF(A431="","Zona STOCK",IF(B431="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15877,7 +15877,7 @@
         <v/>
       </c>
       <c r="M432" s="12">
-        <f>IF(AND(A432="",F432=""),"",IF(F432="","Belum ditempatkan",IF(I432="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G432="","CEK ZONA NO kosong",IF(K432="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H432&lt;&gt;K432,"CEK JENIS ZONA",IF(A432="","Zona kosong",IF(B432="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A432="",F432=""),"",IF(F432="","Belum ditempatkan",IF(I432="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G432="","CEK ZONA NO kosong",IF(K432="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H432&lt;&gt;K432,"CEK JENIS ZONA",IF(A432="","Zona STOCK",IF(B432="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15907,7 +15907,7 @@
         <v/>
       </c>
       <c r="M433" s="12">
-        <f>IF(AND(A433="",F433=""),"",IF(F433="","Belum ditempatkan",IF(I433="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G433="","CEK ZONA NO kosong",IF(K433="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H433&lt;&gt;K433,"CEK JENIS ZONA",IF(A433="","Zona kosong",IF(B433="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A433="",F433=""),"",IF(F433="","Belum ditempatkan",IF(I433="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G433="","CEK ZONA NO kosong",IF(K433="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H433&lt;&gt;K433,"CEK JENIS ZONA",IF(A433="","Zona STOCK",IF(B433="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15937,7 +15937,7 @@
         <v/>
       </c>
       <c r="M434" s="12">
-        <f>IF(AND(A434="",F434=""),"",IF(F434="","Belum ditempatkan",IF(I434="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G434="","CEK ZONA NO kosong",IF(K434="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H434&lt;&gt;K434,"CEK JENIS ZONA",IF(A434="","Zona kosong",IF(B434="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A434="",F434=""),"",IF(F434="","Belum ditempatkan",IF(I434="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G434="","CEK ZONA NO kosong",IF(K434="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H434&lt;&gt;K434,"CEK JENIS ZONA",IF(A434="","Zona STOCK",IF(B434="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15967,7 +15967,7 @@
         <v/>
       </c>
       <c r="M435" s="12">
-        <f>IF(AND(A435="",F435=""),"",IF(F435="","Belum ditempatkan",IF(I435="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G435="","CEK ZONA NO kosong",IF(K435="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H435&lt;&gt;K435,"CEK JENIS ZONA",IF(A435="","Zona kosong",IF(B435="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A435="",F435=""),"",IF(F435="","Belum ditempatkan",IF(I435="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G435="","CEK ZONA NO kosong",IF(K435="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H435&lt;&gt;K435,"CEK JENIS ZONA",IF(A435="","Zona STOCK",IF(B435="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -15997,7 +15997,7 @@
         <v/>
       </c>
       <c r="M436" s="12">
-        <f>IF(AND(A436="",F436=""),"",IF(F436="","Belum ditempatkan",IF(I436="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G436="","CEK ZONA NO kosong",IF(K436="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H436&lt;&gt;K436,"CEK JENIS ZONA",IF(A436="","Zona kosong",IF(B436="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A436="",F436=""),"",IF(F436="","Belum ditempatkan",IF(I436="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G436="","CEK ZONA NO kosong",IF(K436="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H436&lt;&gt;K436,"CEK JENIS ZONA",IF(A436="","Zona STOCK",IF(B436="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16027,7 +16027,7 @@
         <v/>
       </c>
       <c r="M437" s="12">
-        <f>IF(AND(A437="",F437=""),"",IF(F437="","Belum ditempatkan",IF(I437="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G437="","CEK ZONA NO kosong",IF(K437="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H437&lt;&gt;K437,"CEK JENIS ZONA",IF(A437="","Zona kosong",IF(B437="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A437="",F437=""),"",IF(F437="","Belum ditempatkan",IF(I437="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G437="","CEK ZONA NO kosong",IF(K437="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H437&lt;&gt;K437,"CEK JENIS ZONA",IF(A437="","Zona STOCK",IF(B437="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16057,7 +16057,7 @@
         <v/>
       </c>
       <c r="M438" s="12">
-        <f>IF(AND(A438="",F438=""),"",IF(F438="","Belum ditempatkan",IF(I438="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G438="","CEK ZONA NO kosong",IF(K438="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H438&lt;&gt;K438,"CEK JENIS ZONA",IF(A438="","Zona kosong",IF(B438="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A438="",F438=""),"",IF(F438="","Belum ditempatkan",IF(I438="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G438="","CEK ZONA NO kosong",IF(K438="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H438&lt;&gt;K438,"CEK JENIS ZONA",IF(A438="","Zona STOCK",IF(B438="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16087,7 +16087,7 @@
         <v/>
       </c>
       <c r="M439" s="12">
-        <f>IF(AND(A439="",F439=""),"",IF(F439="","Belum ditempatkan",IF(I439="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G439="","CEK ZONA NO kosong",IF(K439="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H439&lt;&gt;K439,"CEK JENIS ZONA",IF(A439="","Zona kosong",IF(B439="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A439="",F439=""),"",IF(F439="","Belum ditempatkan",IF(I439="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G439="","CEK ZONA NO kosong",IF(K439="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H439&lt;&gt;K439,"CEK JENIS ZONA",IF(A439="","Zona STOCK",IF(B439="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
         <v/>
       </c>
       <c r="M440" s="12">
-        <f>IF(AND(A440="",F440=""),"",IF(F440="","Belum ditempatkan",IF(I440="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G440="","CEK ZONA NO kosong",IF(K440="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H440&lt;&gt;K440,"CEK JENIS ZONA",IF(A440="","Zona kosong",IF(B440="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A440="",F440=""),"",IF(F440="","Belum ditempatkan",IF(I440="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G440="","CEK ZONA NO kosong",IF(K440="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H440&lt;&gt;K440,"CEK JENIS ZONA",IF(A440="","Zona STOCK",IF(B440="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16147,7 +16147,7 @@
         <v/>
       </c>
       <c r="M441" s="12">
-        <f>IF(AND(A441="",F441=""),"",IF(F441="","Belum ditempatkan",IF(I441="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G441="","CEK ZONA NO kosong",IF(K441="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H441&lt;&gt;K441,"CEK JENIS ZONA",IF(A441="","Zona kosong",IF(B441="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A441="",F441=""),"",IF(F441="","Belum ditempatkan",IF(I441="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G441="","CEK ZONA NO kosong",IF(K441="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H441&lt;&gt;K441,"CEK JENIS ZONA",IF(A441="","Zona STOCK",IF(B441="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16177,7 +16177,7 @@
         <v/>
       </c>
       <c r="M442" s="12">
-        <f>IF(AND(A442="",F442=""),"",IF(F442="","Belum ditempatkan",IF(I442="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G442="","CEK ZONA NO kosong",IF(K442="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H442&lt;&gt;K442,"CEK JENIS ZONA",IF(A442="","Zona kosong",IF(B442="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A442="",F442=""),"",IF(F442="","Belum ditempatkan",IF(I442="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G442="","CEK ZONA NO kosong",IF(K442="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H442&lt;&gt;K442,"CEK JENIS ZONA",IF(A442="","Zona STOCK",IF(B442="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16207,7 +16207,7 @@
         <v/>
       </c>
       <c r="M443" s="12">
-        <f>IF(AND(A443="",F443=""),"",IF(F443="","Belum ditempatkan",IF(I443="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G443="","CEK ZONA NO kosong",IF(K443="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H443&lt;&gt;K443,"CEK JENIS ZONA",IF(A443="","Zona kosong",IF(B443="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A443="",F443=""),"",IF(F443="","Belum ditempatkan",IF(I443="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G443="","CEK ZONA NO kosong",IF(K443="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H443&lt;&gt;K443,"CEK JENIS ZONA",IF(A443="","Zona STOCK",IF(B443="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16237,7 +16237,7 @@
         <v/>
       </c>
       <c r="M444" s="12">
-        <f>IF(AND(A444="",F444=""),"",IF(F444="","Belum ditempatkan",IF(I444="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G444="","CEK ZONA NO kosong",IF(K444="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H444&lt;&gt;K444,"CEK JENIS ZONA",IF(A444="","Zona kosong",IF(B444="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A444="",F444=""),"",IF(F444="","Belum ditempatkan",IF(I444="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G444="","CEK ZONA NO kosong",IF(K444="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H444&lt;&gt;K444,"CEK JENIS ZONA",IF(A444="","Zona STOCK",IF(B444="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16267,7 +16267,7 @@
         <v/>
       </c>
       <c r="M445" s="12">
-        <f>IF(AND(A445="",F445=""),"",IF(F445="","Belum ditempatkan",IF(I445="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G445="","CEK ZONA NO kosong",IF(K445="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H445&lt;&gt;K445,"CEK JENIS ZONA",IF(A445="","Zona kosong",IF(B445="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A445="",F445=""),"",IF(F445="","Belum ditempatkan",IF(I445="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G445="","CEK ZONA NO kosong",IF(K445="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H445&lt;&gt;K445,"CEK JENIS ZONA",IF(A445="","Zona STOCK",IF(B445="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16297,7 +16297,7 @@
         <v/>
       </c>
       <c r="M446" s="12">
-        <f>IF(AND(A446="",F446=""),"",IF(F446="","Belum ditempatkan",IF(I446="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G446="","CEK ZONA NO kosong",IF(K446="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H446&lt;&gt;K446,"CEK JENIS ZONA",IF(A446="","Zona kosong",IF(B446="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A446="",F446=""),"",IF(F446="","Belum ditempatkan",IF(I446="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G446="","CEK ZONA NO kosong",IF(K446="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H446&lt;&gt;K446,"CEK JENIS ZONA",IF(A446="","Zona STOCK",IF(B446="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
         <v/>
       </c>
       <c r="M447" s="12">
-        <f>IF(AND(A447="",F447=""),"",IF(F447="","Belum ditempatkan",IF(I447="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G447="","CEK ZONA NO kosong",IF(K447="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H447&lt;&gt;K447,"CEK JENIS ZONA",IF(A447="","Zona kosong",IF(B447="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A447="",F447=""),"",IF(F447="","Belum ditempatkan",IF(I447="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G447="","CEK ZONA NO kosong",IF(K447="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H447&lt;&gt;K447,"CEK JENIS ZONA",IF(A447="","Zona STOCK",IF(B447="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16357,7 +16357,7 @@
         <v/>
       </c>
       <c r="M448" s="12">
-        <f>IF(AND(A448="",F448=""),"",IF(F448="","Belum ditempatkan",IF(I448="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G448="","CEK ZONA NO kosong",IF(K448="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H448&lt;&gt;K448,"CEK JENIS ZONA",IF(A448="","Zona kosong",IF(B448="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A448="",F448=""),"",IF(F448="","Belum ditempatkan",IF(I448="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G448="","CEK ZONA NO kosong",IF(K448="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H448&lt;&gt;K448,"CEK JENIS ZONA",IF(A448="","Zona STOCK",IF(B448="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16387,7 +16387,7 @@
         <v/>
       </c>
       <c r="M449" s="12">
-        <f>IF(AND(A449="",F449=""),"",IF(F449="","Belum ditempatkan",IF(I449="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G449="","CEK ZONA NO kosong",IF(K449="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H449&lt;&gt;K449,"CEK JENIS ZONA",IF(A449="","Zona kosong",IF(B449="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A449="",F449=""),"",IF(F449="","Belum ditempatkan",IF(I449="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G449="","CEK ZONA NO kosong",IF(K449="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H449&lt;&gt;K449,"CEK JENIS ZONA",IF(A449="","Zona STOCK",IF(B449="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16417,7 +16417,7 @@
         <v/>
       </c>
       <c r="M450" s="12">
-        <f>IF(AND(A450="",F450=""),"",IF(F450="","Belum ditempatkan",IF(I450="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G450="","CEK ZONA NO kosong",IF(K450="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H450&lt;&gt;K450,"CEK JENIS ZONA",IF(A450="","Zona kosong",IF(B450="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A450="",F450=""),"",IF(F450="","Belum ditempatkan",IF(I450="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G450="","CEK ZONA NO kosong",IF(K450="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H450&lt;&gt;K450,"CEK JENIS ZONA",IF(A450="","Zona STOCK",IF(B450="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16447,7 +16447,7 @@
         <v/>
       </c>
       <c r="M451" s="12">
-        <f>IF(AND(A451="",F451=""),"",IF(F451="","Belum ditempatkan",IF(I451="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G451="","CEK ZONA NO kosong",IF(K451="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H451&lt;&gt;K451,"CEK JENIS ZONA",IF(A451="","Zona kosong",IF(B451="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A451="",F451=""),"",IF(F451="","Belum ditempatkan",IF(I451="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G451="","CEK ZONA NO kosong",IF(K451="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H451&lt;&gt;K451,"CEK JENIS ZONA",IF(A451="","Zona STOCK",IF(B451="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16477,7 +16477,7 @@
         <v/>
       </c>
       <c r="M452" s="12">
-        <f>IF(AND(A452="",F452=""),"",IF(F452="","Belum ditempatkan",IF(I452="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G452="","CEK ZONA NO kosong",IF(K452="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H452&lt;&gt;K452,"CEK JENIS ZONA",IF(A452="","Zona kosong",IF(B452="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A452="",F452=""),"",IF(F452="","Belum ditempatkan",IF(I452="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G452="","CEK ZONA NO kosong",IF(K452="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H452&lt;&gt;K452,"CEK JENIS ZONA",IF(A452="","Zona STOCK",IF(B452="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16507,7 +16507,7 @@
         <v/>
       </c>
       <c r="M453" s="12">
-        <f>IF(AND(A453="",F453=""),"",IF(F453="","Belum ditempatkan",IF(I453="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G453="","CEK ZONA NO kosong",IF(K453="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H453&lt;&gt;K453,"CEK JENIS ZONA",IF(A453="","Zona kosong",IF(B453="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A453="",F453=""),"",IF(F453="","Belum ditempatkan",IF(I453="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G453="","CEK ZONA NO kosong",IF(K453="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H453&lt;&gt;K453,"CEK JENIS ZONA",IF(A453="","Zona STOCK",IF(B453="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16537,7 +16537,7 @@
         <v/>
       </c>
       <c r="M454" s="12">
-        <f>IF(AND(A454="",F454=""),"",IF(F454="","Belum ditempatkan",IF(I454="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G454="","CEK ZONA NO kosong",IF(K454="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H454&lt;&gt;K454,"CEK JENIS ZONA",IF(A454="","Zona kosong",IF(B454="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A454="",F454=""),"",IF(F454="","Belum ditempatkan",IF(I454="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G454="","CEK ZONA NO kosong",IF(K454="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H454&lt;&gt;K454,"CEK JENIS ZONA",IF(A454="","Zona STOCK",IF(B454="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16567,7 +16567,7 @@
         <v/>
       </c>
       <c r="M455" s="12">
-        <f>IF(AND(A455="",F455=""),"",IF(F455="","Belum ditempatkan",IF(I455="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G455="","CEK ZONA NO kosong",IF(K455="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H455&lt;&gt;K455,"CEK JENIS ZONA",IF(A455="","Zona kosong",IF(B455="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A455="",F455=""),"",IF(F455="","Belum ditempatkan",IF(I455="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G455="","CEK ZONA NO kosong",IF(K455="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H455&lt;&gt;K455,"CEK JENIS ZONA",IF(A455="","Zona STOCK",IF(B455="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16597,7 +16597,7 @@
         <v/>
       </c>
       <c r="M456" s="12">
-        <f>IF(AND(A456="",F456=""),"",IF(F456="","Belum ditempatkan",IF(I456="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G456="","CEK ZONA NO kosong",IF(K456="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H456&lt;&gt;K456,"CEK JENIS ZONA",IF(A456="","Zona kosong",IF(B456="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A456="",F456=""),"",IF(F456="","Belum ditempatkan",IF(I456="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G456="","CEK ZONA NO kosong",IF(K456="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H456&lt;&gt;K456,"CEK JENIS ZONA",IF(A456="","Zona STOCK",IF(B456="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16627,7 +16627,7 @@
         <v/>
       </c>
       <c r="M457" s="12">
-        <f>IF(AND(A457="",F457=""),"",IF(F457="","Belum ditempatkan",IF(I457="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G457="","CEK ZONA NO kosong",IF(K457="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H457&lt;&gt;K457,"CEK JENIS ZONA",IF(A457="","Zona kosong",IF(B457="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A457="",F457=""),"",IF(F457="","Belum ditempatkan",IF(I457="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G457="","CEK ZONA NO kosong",IF(K457="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H457&lt;&gt;K457,"CEK JENIS ZONA",IF(A457="","Zona STOCK",IF(B457="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16657,7 +16657,7 @@
         <v/>
       </c>
       <c r="M458" s="12">
-        <f>IF(AND(A458="",F458=""),"",IF(F458="","Belum ditempatkan",IF(I458="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G458="","CEK ZONA NO kosong",IF(K458="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H458&lt;&gt;K458,"CEK JENIS ZONA",IF(A458="","Zona kosong",IF(B458="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A458="",F458=""),"",IF(F458="","Belum ditempatkan",IF(I458="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G458="","CEK ZONA NO kosong",IF(K458="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H458&lt;&gt;K458,"CEK JENIS ZONA",IF(A458="","Zona STOCK",IF(B458="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16687,7 +16687,7 @@
         <v/>
       </c>
       <c r="M459" s="12">
-        <f>IF(AND(A459="",F459=""),"",IF(F459="","Belum ditempatkan",IF(I459="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G459="","CEK ZONA NO kosong",IF(K459="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H459&lt;&gt;K459,"CEK JENIS ZONA",IF(A459="","Zona kosong",IF(B459="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A459="",F459=""),"",IF(F459="","Belum ditempatkan",IF(I459="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G459="","CEK ZONA NO kosong",IF(K459="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H459&lt;&gt;K459,"CEK JENIS ZONA",IF(A459="","Zona STOCK",IF(B459="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16717,7 +16717,7 @@
         <v/>
       </c>
       <c r="M460" s="12">
-        <f>IF(AND(A460="",F460=""),"",IF(F460="","Belum ditempatkan",IF(I460="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G460="","CEK ZONA NO kosong",IF(K460="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H460&lt;&gt;K460,"CEK JENIS ZONA",IF(A460="","Zona kosong",IF(B460="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A460="",F460=""),"",IF(F460="","Belum ditempatkan",IF(I460="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G460="","CEK ZONA NO kosong",IF(K460="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H460&lt;&gt;K460,"CEK JENIS ZONA",IF(A460="","Zona STOCK",IF(B460="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16747,7 +16747,7 @@
         <v/>
       </c>
       <c r="M461" s="12">
-        <f>IF(AND(A461="",F461=""),"",IF(F461="","Belum ditempatkan",IF(I461="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G461="","CEK ZONA NO kosong",IF(K461="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H461&lt;&gt;K461,"CEK JENIS ZONA",IF(A461="","Zona kosong",IF(B461="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A461="",F461=""),"",IF(F461="","Belum ditempatkan",IF(I461="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G461="","CEK ZONA NO kosong",IF(K461="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H461&lt;&gt;K461,"CEK JENIS ZONA",IF(A461="","Zona STOCK",IF(B461="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16777,7 +16777,7 @@
         <v/>
       </c>
       <c r="M462" s="12">
-        <f>IF(AND(A462="",F462=""),"",IF(F462="","Belum ditempatkan",IF(I462="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G462="","CEK ZONA NO kosong",IF(K462="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H462&lt;&gt;K462,"CEK JENIS ZONA",IF(A462="","Zona kosong",IF(B462="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A462="",F462=""),"",IF(F462="","Belum ditempatkan",IF(I462="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G462="","CEK ZONA NO kosong",IF(K462="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H462&lt;&gt;K462,"CEK JENIS ZONA",IF(A462="","Zona STOCK",IF(B462="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
         <v/>
       </c>
       <c r="M463" s="12">
-        <f>IF(AND(A463="",F463=""),"",IF(F463="","Belum ditempatkan",IF(I463="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G463="","CEK ZONA NO kosong",IF(K463="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H463&lt;&gt;K463,"CEK JENIS ZONA",IF(A463="","Zona kosong",IF(B463="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A463="",F463=""),"",IF(F463="","Belum ditempatkan",IF(I463="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G463="","CEK ZONA NO kosong",IF(K463="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H463&lt;&gt;K463,"CEK JENIS ZONA",IF(A463="","Zona STOCK",IF(B463="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16837,7 +16837,7 @@
         <v/>
       </c>
       <c r="M464" s="12">
-        <f>IF(AND(A464="",F464=""),"",IF(F464="","Belum ditempatkan",IF(I464="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G464="","CEK ZONA NO kosong",IF(K464="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H464&lt;&gt;K464,"CEK JENIS ZONA",IF(A464="","Zona kosong",IF(B464="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A464="",F464=""),"",IF(F464="","Belum ditempatkan",IF(I464="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G464="","CEK ZONA NO kosong",IF(K464="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H464&lt;&gt;K464,"CEK JENIS ZONA",IF(A464="","Zona STOCK",IF(B464="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16867,7 +16867,7 @@
         <v/>
       </c>
       <c r="M465" s="12">
-        <f>IF(AND(A465="",F465=""),"",IF(F465="","Belum ditempatkan",IF(I465="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G465="","CEK ZONA NO kosong",IF(K465="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H465&lt;&gt;K465,"CEK JENIS ZONA",IF(A465="","Zona kosong",IF(B465="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A465="",F465=""),"",IF(F465="","Belum ditempatkan",IF(I465="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G465="","CEK ZONA NO kosong",IF(K465="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H465&lt;&gt;K465,"CEK JENIS ZONA",IF(A465="","Zona STOCK",IF(B465="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16897,7 +16897,7 @@
         <v/>
       </c>
       <c r="M466" s="12">
-        <f>IF(AND(A466="",F466=""),"",IF(F466="","Belum ditempatkan",IF(I466="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G466="","CEK ZONA NO kosong",IF(K466="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H466&lt;&gt;K466,"CEK JENIS ZONA",IF(A466="","Zona kosong",IF(B466="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A466="",F466=""),"",IF(F466="","Belum ditempatkan",IF(I466="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G466="","CEK ZONA NO kosong",IF(K466="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H466&lt;&gt;K466,"CEK JENIS ZONA",IF(A466="","Zona STOCK",IF(B466="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16927,7 +16927,7 @@
         <v/>
       </c>
       <c r="M467" s="12">
-        <f>IF(AND(A467="",F467=""),"",IF(F467="","Belum ditempatkan",IF(I467="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G467="","CEK ZONA NO kosong",IF(K467="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H467&lt;&gt;K467,"CEK JENIS ZONA",IF(A467="","Zona kosong",IF(B467="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A467="",F467=""),"",IF(F467="","Belum ditempatkan",IF(I467="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G467="","CEK ZONA NO kosong",IF(K467="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H467&lt;&gt;K467,"CEK JENIS ZONA",IF(A467="","Zona STOCK",IF(B467="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16957,7 +16957,7 @@
         <v/>
       </c>
       <c r="M468" s="12">
-        <f>IF(AND(A468="",F468=""),"",IF(F468="","Belum ditempatkan",IF(I468="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G468="","CEK ZONA NO kosong",IF(K468="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H468&lt;&gt;K468,"CEK JENIS ZONA",IF(A468="","Zona kosong",IF(B468="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A468="",F468=""),"",IF(F468="","Belum ditempatkan",IF(I468="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G468="","CEK ZONA NO kosong",IF(K468="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H468&lt;&gt;K468,"CEK JENIS ZONA",IF(A468="","Zona STOCK",IF(B468="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -16987,7 +16987,7 @@
         <v/>
       </c>
       <c r="M469" s="12">
-        <f>IF(AND(A469="",F469=""),"",IF(F469="","Belum ditempatkan",IF(I469="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G469="","CEK ZONA NO kosong",IF(K469="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H469&lt;&gt;K469,"CEK JENIS ZONA",IF(A469="","Zona kosong",IF(B469="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A469="",F469=""),"",IF(F469="","Belum ditempatkan",IF(I469="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G469="","CEK ZONA NO kosong",IF(K469="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H469&lt;&gt;K469,"CEK JENIS ZONA",IF(A469="","Zona STOCK",IF(B469="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17017,7 +17017,7 @@
         <v/>
       </c>
       <c r="M470" s="12">
-        <f>IF(AND(A470="",F470=""),"",IF(F470="","Belum ditempatkan",IF(I470="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G470="","CEK ZONA NO kosong",IF(K470="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H470&lt;&gt;K470,"CEK JENIS ZONA",IF(A470="","Zona kosong",IF(B470="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A470="",F470=""),"",IF(F470="","Belum ditempatkan",IF(I470="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G470="","CEK ZONA NO kosong",IF(K470="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H470&lt;&gt;K470,"CEK JENIS ZONA",IF(A470="","Zona STOCK",IF(B470="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17047,7 +17047,7 @@
         <v/>
       </c>
       <c r="M471" s="12">
-        <f>IF(AND(A471="",F471=""),"",IF(F471="","Belum ditempatkan",IF(I471="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G471="","CEK ZONA NO kosong",IF(K471="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H471&lt;&gt;K471,"CEK JENIS ZONA",IF(A471="","Zona kosong",IF(B471="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A471="",F471=""),"",IF(F471="","Belum ditempatkan",IF(I471="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G471="","CEK ZONA NO kosong",IF(K471="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H471&lt;&gt;K471,"CEK JENIS ZONA",IF(A471="","Zona STOCK",IF(B471="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17077,7 +17077,7 @@
         <v/>
       </c>
       <c r="M472" s="12">
-        <f>IF(AND(A472="",F472=""),"",IF(F472="","Belum ditempatkan",IF(I472="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G472="","CEK ZONA NO kosong",IF(K472="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H472&lt;&gt;K472,"CEK JENIS ZONA",IF(A472="","Zona kosong",IF(B472="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A472="",F472=""),"",IF(F472="","Belum ditempatkan",IF(I472="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G472="","CEK ZONA NO kosong",IF(K472="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H472&lt;&gt;K472,"CEK JENIS ZONA",IF(A472="","Zona STOCK",IF(B472="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17107,7 +17107,7 @@
         <v/>
       </c>
       <c r="M473" s="12">
-        <f>IF(AND(A473="",F473=""),"",IF(F473="","Belum ditempatkan",IF(I473="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G473="","CEK ZONA NO kosong",IF(K473="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H473&lt;&gt;K473,"CEK JENIS ZONA",IF(A473="","Zona kosong",IF(B473="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A473="",F473=""),"",IF(F473="","Belum ditempatkan",IF(I473="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G473="","CEK ZONA NO kosong",IF(K473="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H473&lt;&gt;K473,"CEK JENIS ZONA",IF(A473="","Zona STOCK",IF(B473="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17137,7 +17137,7 @@
         <v/>
       </c>
       <c r="M474" s="12">
-        <f>IF(AND(A474="",F474=""),"",IF(F474="","Belum ditempatkan",IF(I474="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G474="","CEK ZONA NO kosong",IF(K474="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H474&lt;&gt;K474,"CEK JENIS ZONA",IF(A474="","Zona kosong",IF(B474="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A474="",F474=""),"",IF(F474="","Belum ditempatkan",IF(I474="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G474="","CEK ZONA NO kosong",IF(K474="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H474&lt;&gt;K474,"CEK JENIS ZONA",IF(A474="","Zona STOCK",IF(B474="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17167,7 +17167,7 @@
         <v/>
       </c>
       <c r="M475" s="12">
-        <f>IF(AND(A475="",F475=""),"",IF(F475="","Belum ditempatkan",IF(I475="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G475="","CEK ZONA NO kosong",IF(K475="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H475&lt;&gt;K475,"CEK JENIS ZONA",IF(A475="","Zona kosong",IF(B475="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A475="",F475=""),"",IF(F475="","Belum ditempatkan",IF(I475="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G475="","CEK ZONA NO kosong",IF(K475="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H475&lt;&gt;K475,"CEK JENIS ZONA",IF(A475="","Zona STOCK",IF(B475="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17197,7 +17197,7 @@
         <v/>
       </c>
       <c r="M476" s="12">
-        <f>IF(AND(A476="",F476=""),"",IF(F476="","Belum ditempatkan",IF(I476="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G476="","CEK ZONA NO kosong",IF(K476="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H476&lt;&gt;K476,"CEK JENIS ZONA",IF(A476="","Zona kosong",IF(B476="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A476="",F476=""),"",IF(F476="","Belum ditempatkan",IF(I476="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G476="","CEK ZONA NO kosong",IF(K476="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H476&lt;&gt;K476,"CEK JENIS ZONA",IF(A476="","Zona STOCK",IF(B476="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17227,7 +17227,7 @@
         <v/>
       </c>
       <c r="M477" s="12">
-        <f>IF(AND(A477="",F477=""),"",IF(F477="","Belum ditempatkan",IF(I477="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G477="","CEK ZONA NO kosong",IF(K477="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H477&lt;&gt;K477,"CEK JENIS ZONA",IF(A477="","Zona kosong",IF(B477="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A477="",F477=""),"",IF(F477="","Belum ditempatkan",IF(I477="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G477="","CEK ZONA NO kosong",IF(K477="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H477&lt;&gt;K477,"CEK JENIS ZONA",IF(A477="","Zona STOCK",IF(B477="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17257,7 +17257,7 @@
         <v/>
       </c>
       <c r="M478" s="12">
-        <f>IF(AND(A478="",F478=""),"",IF(F478="","Belum ditempatkan",IF(I478="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G478="","CEK ZONA NO kosong",IF(K478="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H478&lt;&gt;K478,"CEK JENIS ZONA",IF(A478="","Zona kosong",IF(B478="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A478="",F478=""),"",IF(F478="","Belum ditempatkan",IF(I478="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G478="","CEK ZONA NO kosong",IF(K478="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H478&lt;&gt;K478,"CEK JENIS ZONA",IF(A478="","Zona STOCK",IF(B478="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17287,7 +17287,7 @@
         <v/>
       </c>
       <c r="M479" s="12">
-        <f>IF(AND(A479="",F479=""),"",IF(F479="","Belum ditempatkan",IF(I479="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G479="","CEK ZONA NO kosong",IF(K479="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H479&lt;&gt;K479,"CEK JENIS ZONA",IF(A479="","Zona kosong",IF(B479="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A479="",F479=""),"",IF(F479="","Belum ditempatkan",IF(I479="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G479="","CEK ZONA NO kosong",IF(K479="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H479&lt;&gt;K479,"CEK JENIS ZONA",IF(A479="","Zona STOCK",IF(B479="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17317,7 +17317,7 @@
         <v/>
       </c>
       <c r="M480" s="12">
-        <f>IF(AND(A480="",F480=""),"",IF(F480="","Belum ditempatkan",IF(I480="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G480="","CEK ZONA NO kosong",IF(K480="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H480&lt;&gt;K480,"CEK JENIS ZONA",IF(A480="","Zona kosong",IF(B480="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A480="",F480=""),"",IF(F480="","Belum ditempatkan",IF(I480="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G480="","CEK ZONA NO kosong",IF(K480="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H480&lt;&gt;K480,"CEK JENIS ZONA",IF(A480="","Zona STOCK",IF(B480="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17347,7 +17347,7 @@
         <v/>
       </c>
       <c r="M481" s="12">
-        <f>IF(AND(A481="",F481=""),"",IF(F481="","Belum ditempatkan",IF(I481="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G481="","CEK ZONA NO kosong",IF(K481="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H481&lt;&gt;K481,"CEK JENIS ZONA",IF(A481="","Zona kosong",IF(B481="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A481="",F481=""),"",IF(F481="","Belum ditempatkan",IF(I481="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G481="","CEK ZONA NO kosong",IF(K481="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H481&lt;&gt;K481,"CEK JENIS ZONA",IF(A481="","Zona STOCK",IF(B481="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17377,7 +17377,7 @@
         <v/>
       </c>
       <c r="M482" s="12">
-        <f>IF(AND(A482="",F482=""),"",IF(F482="","Belum ditempatkan",IF(I482="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G482="","CEK ZONA NO kosong",IF(K482="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H482&lt;&gt;K482,"CEK JENIS ZONA",IF(A482="","Zona kosong",IF(B482="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A482="",F482=""),"",IF(F482="","Belum ditempatkan",IF(I482="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G482="","CEK ZONA NO kosong",IF(K482="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H482&lt;&gt;K482,"CEK JENIS ZONA",IF(A482="","Zona STOCK",IF(B482="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17407,7 +17407,7 @@
         <v/>
       </c>
       <c r="M483" s="12">
-        <f>IF(AND(A483="",F483=""),"",IF(F483="","Belum ditempatkan",IF(I483="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G483="","CEK ZONA NO kosong",IF(K483="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H483&lt;&gt;K483,"CEK JENIS ZONA",IF(A483="","Zona kosong",IF(B483="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A483="",F483=""),"",IF(F483="","Belum ditempatkan",IF(I483="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G483="","CEK ZONA NO kosong",IF(K483="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H483&lt;&gt;K483,"CEK JENIS ZONA",IF(A483="","Zona STOCK",IF(B483="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17437,7 +17437,7 @@
         <v/>
       </c>
       <c r="M484" s="12">
-        <f>IF(AND(A484="",F484=""),"",IF(F484="","Belum ditempatkan",IF(I484="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G484="","CEK ZONA NO kosong",IF(K484="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H484&lt;&gt;K484,"CEK JENIS ZONA",IF(A484="","Zona kosong",IF(B484="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A484="",F484=""),"",IF(F484="","Belum ditempatkan",IF(I484="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G484="","CEK ZONA NO kosong",IF(K484="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H484&lt;&gt;K484,"CEK JENIS ZONA",IF(A484="","Zona STOCK",IF(B484="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17467,7 +17467,7 @@
         <v/>
       </c>
       <c r="M485" s="12">
-        <f>IF(AND(A485="",F485=""),"",IF(F485="","Belum ditempatkan",IF(I485="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G485="","CEK ZONA NO kosong",IF(K485="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H485&lt;&gt;K485,"CEK JENIS ZONA",IF(A485="","Zona kosong",IF(B485="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A485="",F485=""),"",IF(F485="","Belum ditempatkan",IF(I485="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G485="","CEK ZONA NO kosong",IF(K485="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H485&lt;&gt;K485,"CEK JENIS ZONA",IF(A485="","Zona STOCK",IF(B485="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17497,7 +17497,7 @@
         <v/>
       </c>
       <c r="M486" s="12">
-        <f>IF(AND(A486="",F486=""),"",IF(F486="","Belum ditempatkan",IF(I486="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G486="","CEK ZONA NO kosong",IF(K486="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H486&lt;&gt;K486,"CEK JENIS ZONA",IF(A486="","Zona kosong",IF(B486="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A486="",F486=""),"",IF(F486="","Belum ditempatkan",IF(I486="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G486="","CEK ZONA NO kosong",IF(K486="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H486&lt;&gt;K486,"CEK JENIS ZONA",IF(A486="","Zona STOCK",IF(B486="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17527,7 +17527,7 @@
         <v/>
       </c>
       <c r="M487" s="12">
-        <f>IF(AND(A487="",F487=""),"",IF(F487="","Belum ditempatkan",IF(I487="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G487="","CEK ZONA NO kosong",IF(K487="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H487&lt;&gt;K487,"CEK JENIS ZONA",IF(A487="","Zona kosong",IF(B487="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A487="",F487=""),"",IF(F487="","Belum ditempatkan",IF(I487="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G487="","CEK ZONA NO kosong",IF(K487="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H487&lt;&gt;K487,"CEK JENIS ZONA",IF(A487="","Zona STOCK",IF(B487="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17557,7 +17557,7 @@
         <v/>
       </c>
       <c r="M488" s="12">
-        <f>IF(AND(A488="",F488=""),"",IF(F488="","Belum ditempatkan",IF(I488="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G488="","CEK ZONA NO kosong",IF(K488="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H488&lt;&gt;K488,"CEK JENIS ZONA",IF(A488="","Zona kosong",IF(B488="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A488="",F488=""),"",IF(F488="","Belum ditempatkan",IF(I488="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G488="","CEK ZONA NO kosong",IF(K488="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H488&lt;&gt;K488,"CEK JENIS ZONA",IF(A488="","Zona STOCK",IF(B488="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17587,7 +17587,7 @@
         <v/>
       </c>
       <c r="M489" s="12">
-        <f>IF(AND(A489="",F489=""),"",IF(F489="","Belum ditempatkan",IF(I489="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G489="","CEK ZONA NO kosong",IF(K489="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H489&lt;&gt;K489,"CEK JENIS ZONA",IF(A489="","Zona kosong",IF(B489="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A489="",F489=""),"",IF(F489="","Belum ditempatkan",IF(I489="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G489="","CEK ZONA NO kosong",IF(K489="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H489&lt;&gt;K489,"CEK JENIS ZONA",IF(A489="","Zona STOCK",IF(B489="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17617,7 +17617,7 @@
         <v/>
       </c>
       <c r="M490" s="12">
-        <f>IF(AND(A490="",F490=""),"",IF(F490="","Belum ditempatkan",IF(I490="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G490="","CEK ZONA NO kosong",IF(K490="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H490&lt;&gt;K490,"CEK JENIS ZONA",IF(A490="","Zona kosong",IF(B490="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A490="",F490=""),"",IF(F490="","Belum ditempatkan",IF(I490="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G490="","CEK ZONA NO kosong",IF(K490="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H490&lt;&gt;K490,"CEK JENIS ZONA",IF(A490="","Zona STOCK",IF(B490="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17647,7 +17647,7 @@
         <v/>
       </c>
       <c r="M491" s="12">
-        <f>IF(AND(A491="",F491=""),"",IF(F491="","Belum ditempatkan",IF(I491="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G491="","CEK ZONA NO kosong",IF(K491="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H491&lt;&gt;K491,"CEK JENIS ZONA",IF(A491="","Zona kosong",IF(B491="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A491="",F491=""),"",IF(F491="","Belum ditempatkan",IF(I491="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G491="","CEK ZONA NO kosong",IF(K491="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H491&lt;&gt;K491,"CEK JENIS ZONA",IF(A491="","Zona STOCK",IF(B491="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17677,7 +17677,7 @@
         <v/>
       </c>
       <c r="M492" s="12">
-        <f>IF(AND(A492="",F492=""),"",IF(F492="","Belum ditempatkan",IF(I492="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G492="","CEK ZONA NO kosong",IF(K492="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H492&lt;&gt;K492,"CEK JENIS ZONA",IF(A492="","Zona kosong",IF(B492="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A492="",F492=""),"",IF(F492="","Belum ditempatkan",IF(I492="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G492="","CEK ZONA NO kosong",IF(K492="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H492&lt;&gt;K492,"CEK JENIS ZONA",IF(A492="","Zona STOCK",IF(B492="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17707,7 +17707,7 @@
         <v/>
       </c>
       <c r="M493" s="12">
-        <f>IF(AND(A493="",F493=""),"",IF(F493="","Belum ditempatkan",IF(I493="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G493="","CEK ZONA NO kosong",IF(K493="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H493&lt;&gt;K493,"CEK JENIS ZONA",IF(A493="","Zona kosong",IF(B493="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A493="",F493=""),"",IF(F493="","Belum ditempatkan",IF(I493="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G493="","CEK ZONA NO kosong",IF(K493="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H493&lt;&gt;K493,"CEK JENIS ZONA",IF(A493="","Zona STOCK",IF(B493="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17737,7 +17737,7 @@
         <v/>
       </c>
       <c r="M494" s="12">
-        <f>IF(AND(A494="",F494=""),"",IF(F494="","Belum ditempatkan",IF(I494="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G494="","CEK ZONA NO kosong",IF(K494="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H494&lt;&gt;K494,"CEK JENIS ZONA",IF(A494="","Zona kosong",IF(B494="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A494="",F494=""),"",IF(F494="","Belum ditempatkan",IF(I494="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G494="","CEK ZONA NO kosong",IF(K494="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H494&lt;&gt;K494,"CEK JENIS ZONA",IF(A494="","Zona STOCK",IF(B494="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17767,7 +17767,7 @@
         <v/>
       </c>
       <c r="M495" s="12">
-        <f>IF(AND(A495="",F495=""),"",IF(F495="","Belum ditempatkan",IF(I495="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G495="","CEK ZONA NO kosong",IF(K495="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H495&lt;&gt;K495,"CEK JENIS ZONA",IF(A495="","Zona kosong",IF(B495="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A495="",F495=""),"",IF(F495="","Belum ditempatkan",IF(I495="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G495="","CEK ZONA NO kosong",IF(K495="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H495&lt;&gt;K495,"CEK JENIS ZONA",IF(A495="","Zona STOCK",IF(B495="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17797,7 +17797,7 @@
         <v/>
       </c>
       <c r="M496" s="12">
-        <f>IF(AND(A496="",F496=""),"",IF(F496="","Belum ditempatkan",IF(I496="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G496="","CEK ZONA NO kosong",IF(K496="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H496&lt;&gt;K496,"CEK JENIS ZONA",IF(A496="","Zona kosong",IF(B496="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A496="",F496=""),"",IF(F496="","Belum ditempatkan",IF(I496="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G496="","CEK ZONA NO kosong",IF(K496="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H496&lt;&gt;K496,"CEK JENIS ZONA",IF(A496="","Zona STOCK",IF(B496="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17827,7 +17827,7 @@
         <v/>
       </c>
       <c r="M497" s="12">
-        <f>IF(AND(A497="",F497=""),"",IF(F497="","Belum ditempatkan",IF(I497="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G497="","CEK ZONA NO kosong",IF(K497="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H497&lt;&gt;K497,"CEK JENIS ZONA",IF(A497="","Zona kosong",IF(B497="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A497="",F497=""),"",IF(F497="","Belum ditempatkan",IF(I497="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G497="","CEK ZONA NO kosong",IF(K497="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H497&lt;&gt;K497,"CEK JENIS ZONA",IF(A497="","Zona STOCK",IF(B497="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17857,7 +17857,7 @@
         <v/>
       </c>
       <c r="M498" s="12">
-        <f>IF(AND(A498="",F498=""),"",IF(F498="","Belum ditempatkan",IF(I498="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G498="","CEK ZONA NO kosong",IF(K498="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H498&lt;&gt;K498,"CEK JENIS ZONA",IF(A498="","Zona kosong",IF(B498="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A498="",F498=""),"",IF(F498="","Belum ditempatkan",IF(I498="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G498="","CEK ZONA NO kosong",IF(K498="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H498&lt;&gt;K498,"CEK JENIS ZONA",IF(A498="","Zona STOCK",IF(B498="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17887,7 +17887,7 @@
         <v/>
       </c>
       <c r="M499" s="12">
-        <f>IF(AND(A499="",F499=""),"",IF(F499="","Belum ditempatkan",IF(I499="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G499="","CEK ZONA NO kosong",IF(K499="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H499&lt;&gt;K499,"CEK JENIS ZONA",IF(A499="","Zona kosong",IF(B499="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A499="",F499=""),"",IF(F499="","Belum ditempatkan",IF(I499="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G499="","CEK ZONA NO kosong",IF(K499="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H499&lt;&gt;K499,"CEK JENIS ZONA",IF(A499="","Zona STOCK",IF(B499="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17917,7 +17917,7 @@
         <v/>
       </c>
       <c r="M500" s="12">
-        <f>IF(AND(A500="",F500=""),"",IF(F500="","Belum ditempatkan",IF(I500="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G500="","CEK ZONA NO kosong",IF(K500="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H500&lt;&gt;K500,"CEK JENIS ZONA",IF(A500="","Zona kosong",IF(B500="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
+        <f>IF(AND(A500="",F500=""),"",IF(F500="","Belum ditempatkan",IF(I500="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(G500="","CEK ZONA NO kosong",IF(K500="zona tidak ada di layout","CEK ZONA NO di luar layout",IF(H500&lt;&gt;K500,"CEK JENIS ZONA",IF(A500="","Zona STOCK",IF(B500="","CEK SKU DESCRIPTION kosong","OK"))))))))</f>
         <v/>
       </c>
     </row>
@@ -17931,7 +17931,7 @@
       <formula>$M2="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>OR($M2="Zona kosong",$M2="Belum ditempatkan")</formula>
+      <formula>OR($M2="Zona STOCK",$M2="Belum ditempatkan")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">

</xml_diff>

<commit_message>
Faceted (interdependent) filters: options narrow by the other selected filters; Excel: remove LIST_GRUP sheet and its dropdowns (filters read only from DATA)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KGdyTJhm5K5VodWjT1gUuo
</commit_message>
<xml_diff>
--- a/data_planogram_terisi.xlsx
+++ b/data_planogram_terisi.xlsx
@@ -11,7 +11,6 @@
     <sheet name="DATA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="DAFTAR_FIXTURE" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="LAYOUT" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="LIST_GRUP" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="FIXTURE_IDS">OFFSET(DAFTAR_FIXTURE!$A$2,0,0,MAX(1,COUNTA(DAFTAR_FIXTURE!$A$2:$A$51)),1)</definedName>
@@ -679,7 +678,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Contoh: PENYIMPANAN, MAKAN, MASAK. Dropdown. Dipakai sebagai filter. Isi "X" dianggap kosong.</t>
+          <t>Contoh: PENYIMPANAN, MAKAN, MASAK. Dipakai sebagai filter. Isi "X" dianggap kosong.</t>
         </is>
       </c>
     </row>
@@ -691,7 +690,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Contoh: E4. CANISTER, A2. SERVINGWARE. Dropdown. Dipakai sebagai filter.</t>
+          <t>Contoh: E4. CANISTER, A2. SERVINGWARE. Dipakai sebagai filter.</t>
         </is>
       </c>
     </row>
@@ -27436,7 +27435,7 @@
       <formula>OR($Z2="Zona STOCK",$Z2="Belum ditempatkan")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
+  <dataValidations count="3">
     <dataValidation sqref="L2:L500 Q2:Q500 V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ID FIXTURE" error="Pilih ID dari daftar (kelola di sheet DAFTAR_FIXTURE)." type="list">
       <formula1>FIXTURE_IDS</formula1>
     </dataValidation>
@@ -27445,15 +27444,6 @@
     </dataValidation>
     <dataValidation sqref="N2:N500 S2:S500 X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Rak,Gantungan"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="GRUP DISPLAY" error="Nilai belum ada di LIST_GRUP. Tetap dipakai?" type="list" errorStyle="warning">
-      <formula1>LIST_GRUP!$A$2:$A$60</formula1>
-    </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="GRUP ADJACENCY" error="Nilai belum ada di LIST_GRUP. Tetap dipakai?" type="list" errorStyle="warning">
-      <formula1>LIST_GRUP!$B$2:$B$60</formula1>
-    </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="SERIES" error="Nilai belum ada di LIST_GRUP. Tetap dipakai?" type="list" errorStyle="warning">
-      <formula1>LIST_GRUP!$C$2:$C$60</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28665,191 +28655,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>GRUP DISPLAY</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>GRUP ADJACENCY</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>SERIES</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Daftar pilihan dropdown. Tambah nilai baru ke bawah kolom yang sesuai.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ALAT MASAK</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>A1. GLASSWARE</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ELAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MAKAN</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>A2. SERVINGWARE</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GLASS BASIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MASAK</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>B1. CASSEROLE</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GLASS FANCY</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>PENYIMPANAN</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>B2. COOKWARE</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GOLD MARBLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>C1. KITCHEN TOOLS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>INVERNESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>D11. KITCHEN PLASTICWARE</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KINGSTON</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>E4. CANISTER</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>KIRA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>MARBLE W/RACK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>POLLA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>SERVING SET MARBLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>TANTA NYLON</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>TANTA S/S</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>W/GOLD RACK GLASS</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Connected visuals limited to Wall/Gondola/Pallet (example picks one of each); sample workbook now fills every zone of all 12 fixture types
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KGdyTJhm5K5VodWjT1gUuo
</commit_message>
<xml_diff>
--- a/data_planogram_terisi.xlsx
+++ b/data_planogram_terisi.xlsx
@@ -1290,11 +1290,31 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="n"/>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Plates &amp; Bowls</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>238181</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>COUPE PLATE 16 CM SIMPLE PLUS</t>
+        </is>
+      </c>
       <c r="F2" s="10" t="n"/>
       <c r="G2" s="10" t="n"/>
       <c r="H2" s="10" t="n"/>
@@ -2386,15 +2406,47 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Glassware</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>10099887</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>ELAN WATER GLASS SET 414ML (6)</t>
+        </is>
+      </c>
       <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="n"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>A1. GLASSWARE</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>ELAN</t>
+        </is>
+      </c>
       <c r="J13" s="10" t="n"/>
       <c r="K13" s="10" t="n"/>
       <c r="L13" s="11" t="inlineStr">
@@ -3136,15 +3188,47 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n"/>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>10681571</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>SERVING GLASS SQR PLATER ZEVY GOLD</t>
+        </is>
+      </c>
       <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n"/>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>W/GOLD RACK GLASS</t>
+        </is>
+      </c>
       <c r="J21" s="10" t="n"/>
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="11" t="inlineStr">
@@ -3192,15 +3276,47 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>10470029</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET W/RACK OCTAGON MARBLE (4)</t>
+        </is>
+      </c>
       <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n"/>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET MARBLE</t>
+        </is>
+      </c>
       <c r="J22" s="10" t="n"/>
       <c r="K22" s="10" t="n"/>
       <c r="L22" s="11" t="inlineStr">
@@ -10078,20 +10194,50 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="10" t="n"/>
-      <c r="B97" s="10" t="n"/>
-      <c r="C97" s="10" t="n"/>
-      <c r="D97" s="10" t="n"/>
-      <c r="E97" s="10" t="n"/>
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>Plates &amp; Bowls</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="inlineStr">
+        <is>
+          <t>238182</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="inlineStr">
+        <is>
+          <t>COUPLE PLATE 27CM SIMPLE PLUS</t>
+        </is>
+      </c>
       <c r="F97" s="10" t="n"/>
       <c r="G97" s="10" t="n"/>
       <c r="H97" s="10" t="n"/>
       <c r="I97" s="10" t="n"/>
       <c r="J97" s="10" t="n"/>
       <c r="K97" s="10" t="n"/>
-      <c r="L97" s="11" t="n"/>
-      <c r="M97" s="11" t="n"/>
-      <c r="N97" s="11" t="n"/>
+      <c r="L97" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="M97" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N97" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O97" s="12">
         <f>IF(L97="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L97,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10124,20 +10270,50 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="10" t="n"/>
-      <c r="B98" s="10" t="n"/>
-      <c r="C98" s="10" t="n"/>
-      <c r="D98" s="10" t="n"/>
-      <c r="E98" s="10" t="n"/>
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>Plates &amp; Bowls</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>238187</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
+        <is>
+          <t>RECT PLATE 14.5CMX22CM SIMPLE PLUS</t>
+        </is>
+      </c>
       <c r="F98" s="10" t="n"/>
       <c r="G98" s="10" t="n"/>
       <c r="H98" s="10" t="n"/>
       <c r="I98" s="10" t="n"/>
       <c r="J98" s="10" t="n"/>
       <c r="K98" s="10" t="n"/>
-      <c r="L98" s="11" t="n"/>
-      <c r="M98" s="11" t="n"/>
-      <c r="N98" s="11" t="n"/>
+      <c r="L98" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="M98" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N98" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O98" s="12">
         <f>IF(L98="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L98,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10170,20 +10346,50 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="10" t="n"/>
-      <c r="B99" s="10" t="n"/>
-      <c r="C99" s="10" t="n"/>
-      <c r="D99" s="10" t="n"/>
-      <c r="E99" s="10" t="n"/>
+      <c r="A99" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C99" s="10" t="inlineStr">
+        <is>
+          <t>Plates &amp; Bowls</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="inlineStr">
+        <is>
+          <t>238192</t>
+        </is>
+      </c>
+      <c r="E99" s="10" t="inlineStr">
+        <is>
+          <t>LOW BOWL 17 CM SIMPLE PLUS</t>
+        </is>
+      </c>
       <c r="F99" s="10" t="n"/>
       <c r="G99" s="10" t="n"/>
       <c r="H99" s="10" t="n"/>
       <c r="I99" s="10" t="n"/>
       <c r="J99" s="10" t="n"/>
       <c r="K99" s="10" t="n"/>
-      <c r="L99" s="11" t="n"/>
-      <c r="M99" s="11" t="n"/>
-      <c r="N99" s="11" t="n"/>
+      <c r="L99" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="M99" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N99" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O99" s="12">
         <f>IF(L99="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L99,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10216,20 +10422,62 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="10" t="n"/>
-      <c r="B100" s="10" t="n"/>
-      <c r="C100" s="10" t="n"/>
-      <c r="D100" s="10" t="n"/>
-      <c r="E100" s="10" t="n"/>
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>Glassware</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>10099940</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>INVERNESS WATER GLASS SET 355ML (6)</t>
+        </is>
+      </c>
       <c r="F100" s="10" t="n"/>
-      <c r="G100" s="10" t="n"/>
-      <c r="H100" s="10" t="n"/>
-      <c r="I100" s="10" t="n"/>
+      <c r="G100" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H100" s="10" t="inlineStr">
+        <is>
+          <t>A1. GLASSWARE</t>
+        </is>
+      </c>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
+          <t>INVERNESS</t>
+        </is>
+      </c>
       <c r="J100" s="10" t="n"/>
       <c r="K100" s="10" t="n"/>
-      <c r="L100" s="11" t="n"/>
-      <c r="M100" s="11" t="n"/>
-      <c r="N100" s="11" t="n"/>
+      <c r="L100" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="M100" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N100" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O100" s="12">
         <f>IF(L100="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L100,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10262,20 +10510,50 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="10" t="n"/>
-      <c r="B101" s="10" t="n"/>
-      <c r="C101" s="10" t="n"/>
-      <c r="D101" s="10" t="n"/>
-      <c r="E101" s="10" t="n"/>
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>Cup &amp; Saucer</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="inlineStr">
+        <is>
+          <t>238190</t>
+        </is>
+      </c>
+      <c r="E101" s="10" t="inlineStr">
+        <is>
+          <t>CUP 100 CC W/SAUCER 12.5CM SIMPLE PLUS</t>
+        </is>
+      </c>
       <c r="F101" s="10" t="n"/>
       <c r="G101" s="10" t="n"/>
       <c r="H101" s="10" t="n"/>
       <c r="I101" s="10" t="n"/>
       <c r="J101" s="10" t="n"/>
       <c r="K101" s="10" t="n"/>
-      <c r="L101" s="11" t="n"/>
-      <c r="M101" s="11" t="n"/>
-      <c r="N101" s="11" t="n"/>
+      <c r="L101" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="M101" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N101" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O101" s="12">
         <f>IF(L101="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L101,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10308,20 +10586,50 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="10" t="n"/>
-      <c r="B102" s="10" t="n"/>
-      <c r="C102" s="10" t="n"/>
-      <c r="D102" s="10" t="n"/>
-      <c r="E102" s="10" t="n"/>
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>Cup &amp; Saucer</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>238191</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>CUP 200 CC W/SAUCER 15.5CM SIMPLE PLUS</t>
+        </is>
+      </c>
       <c r="F102" s="10" t="n"/>
       <c r="G102" s="10" t="n"/>
       <c r="H102" s="10" t="n"/>
       <c r="I102" s="10" t="n"/>
       <c r="J102" s="10" t="n"/>
       <c r="K102" s="10" t="n"/>
-      <c r="L102" s="11" t="n"/>
-      <c r="M102" s="11" t="n"/>
-      <c r="N102" s="11" t="n"/>
+      <c r="L102" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="M102" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N102" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O102" s="12">
         <f>IF(L102="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L102,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10354,20 +10662,62 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="10" t="n"/>
-      <c r="B103" s="10" t="n"/>
-      <c r="C103" s="10" t="n"/>
-      <c r="D103" s="10" t="n"/>
-      <c r="E103" s="10" t="n"/>
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>Food Storage</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>10680419</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr">
+        <is>
+          <t>MOSQUE DOME GLASS JAR SET OF 3 450ML</t>
+        </is>
+      </c>
       <c r="F103" s="10" t="n"/>
-      <c r="G103" s="10" t="n"/>
-      <c r="H103" s="10" t="n"/>
-      <c r="I103" s="10" t="n"/>
+      <c r="G103" s="10" t="inlineStr">
+        <is>
+          <t>PENYIMPANAN</t>
+        </is>
+      </c>
+      <c r="H103" s="10" t="inlineStr">
+        <is>
+          <t>E4. CANISTER</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t>GLASS FANCY</t>
+        </is>
+      </c>
       <c r="J103" s="10" t="n"/>
       <c r="K103" s="10" t="n"/>
-      <c r="L103" s="11" t="n"/>
-      <c r="M103" s="11" t="n"/>
-      <c r="N103" s="11" t="n"/>
+      <c r="L103" s="11" t="inlineStr">
+        <is>
+          <t>WLL-02</t>
+        </is>
+      </c>
+      <c r="M103" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N103" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O103" s="12">
         <f>IF(L103="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L103,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10400,20 +10750,62 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="10" t="n"/>
-      <c r="B104" s="10" t="n"/>
-      <c r="C104" s="10" t="n"/>
-      <c r="D104" s="10" t="n"/>
-      <c r="E104" s="10" t="n"/>
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>Food Storage</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>10682153</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>EID 2026 GLASS JAR SET OF 3 900ML</t>
+        </is>
+      </c>
       <c r="F104" s="10" t="n"/>
-      <c r="G104" s="10" t="n"/>
-      <c r="H104" s="10" t="n"/>
-      <c r="I104" s="10" t="n"/>
+      <c r="G104" s="10" t="inlineStr">
+        <is>
+          <t>PENYIMPANAN</t>
+        </is>
+      </c>
+      <c r="H104" s="10" t="inlineStr">
+        <is>
+          <t>E4. CANISTER</t>
+        </is>
+      </c>
+      <c r="I104" s="10" t="inlineStr">
+        <is>
+          <t>GLASS FANCY</t>
+        </is>
+      </c>
       <c r="J104" s="10" t="n"/>
       <c r="K104" s="10" t="n"/>
-      <c r="L104" s="11" t="n"/>
-      <c r="M104" s="11" t="n"/>
-      <c r="N104" s="11" t="n"/>
+      <c r="L104" s="11" t="inlineStr">
+        <is>
+          <t>WLL-02</t>
+        </is>
+      </c>
+      <c r="M104" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N104" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O104" s="12">
         <f>IF(L104="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L104,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10446,20 +10838,62 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="10" t="n"/>
-      <c r="B105" s="10" t="n"/>
-      <c r="C105" s="10" t="n"/>
-      <c r="D105" s="10" t="n"/>
-      <c r="E105" s="10" t="n"/>
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>Food Storage</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr">
+        <is>
+          <t>10682154</t>
+        </is>
+      </c>
+      <c r="E105" s="10" t="inlineStr">
+        <is>
+          <t>GRETTA GLASS JAR SET OF 4 WITH RACK</t>
+        </is>
+      </c>
       <c r="F105" s="10" t="n"/>
-      <c r="G105" s="10" t="n"/>
-      <c r="H105" s="10" t="n"/>
-      <c r="I105" s="10" t="n"/>
+      <c r="G105" s="10" t="inlineStr">
+        <is>
+          <t>PENYIMPANAN</t>
+        </is>
+      </c>
+      <c r="H105" s="10" t="inlineStr">
+        <is>
+          <t>E4. CANISTER</t>
+        </is>
+      </c>
+      <c r="I105" s="10" t="inlineStr">
+        <is>
+          <t>GLASS BASIC</t>
+        </is>
+      </c>
       <c r="J105" s="10" t="n"/>
       <c r="K105" s="10" t="n"/>
-      <c r="L105" s="11" t="n"/>
-      <c r="M105" s="11" t="n"/>
-      <c r="N105" s="11" t="n"/>
+      <c r="L105" s="11" t="inlineStr">
+        <is>
+          <t>WLL-02</t>
+        </is>
+      </c>
+      <c r="M105" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N105" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O105" s="12">
         <f>IF(L105="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L105,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10492,20 +10926,62 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="10" t="n"/>
-      <c r="B106" s="10" t="n"/>
-      <c r="C106" s="10" t="n"/>
-      <c r="D106" s="10" t="n"/>
-      <c r="E106" s="10" t="n"/>
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>Food Storage</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>10682155</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="inlineStr">
+        <is>
+          <t>GRETTA GLASS JAR SET OF 3 WITH RACK</t>
+        </is>
+      </c>
       <c r="F106" s="10" t="n"/>
-      <c r="G106" s="10" t="n"/>
-      <c r="H106" s="10" t="n"/>
-      <c r="I106" s="10" t="n"/>
+      <c r="G106" s="10" t="inlineStr">
+        <is>
+          <t>PENYIMPANAN</t>
+        </is>
+      </c>
+      <c r="H106" s="10" t="inlineStr">
+        <is>
+          <t>E4. CANISTER</t>
+        </is>
+      </c>
+      <c r="I106" s="10" t="inlineStr">
+        <is>
+          <t>GLASS BASIC</t>
+        </is>
+      </c>
       <c r="J106" s="10" t="n"/>
       <c r="K106" s="10" t="n"/>
-      <c r="L106" s="11" t="n"/>
-      <c r="M106" s="11" t="n"/>
-      <c r="N106" s="11" t="n"/>
+      <c r="L106" s="11" t="inlineStr">
+        <is>
+          <t>WLL-02</t>
+        </is>
+      </c>
+      <c r="M106" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N106" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O106" s="12">
         <f>IF(L106="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L106,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10538,20 +11014,62 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="n"/>
-      <c r="B107" s="10" t="n"/>
-      <c r="C107" s="10" t="n"/>
-      <c r="D107" s="10" t="n"/>
-      <c r="E107" s="10" t="n"/>
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="inlineStr">
+        <is>
+          <t>10681572</t>
+        </is>
+      </c>
+      <c r="E107" s="10" t="inlineStr">
+        <is>
+          <t>SERVING GLASS OVAL PLATER ZOE GOLD</t>
+        </is>
+      </c>
       <c r="F107" s="10" t="n"/>
-      <c r="G107" s="10" t="n"/>
-      <c r="H107" s="10" t="n"/>
-      <c r="I107" s="10" t="n"/>
+      <c r="G107" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H107" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I107" s="10" t="inlineStr">
+        <is>
+          <t>W/GOLD RACK GLASS</t>
+        </is>
+      </c>
       <c r="J107" s="10" t="n"/>
       <c r="K107" s="10" t="n"/>
-      <c r="L107" s="11" t="n"/>
-      <c r="M107" s="11" t="n"/>
-      <c r="N107" s="11" t="n"/>
+      <c r="L107" s="11" t="inlineStr">
+        <is>
+          <t>WLL-03</t>
+        </is>
+      </c>
+      <c r="M107" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N107" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O107" s="12">
         <f>IF(L107="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L107,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10584,20 +11102,62 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="10" t="n"/>
-      <c r="B108" s="10" t="n"/>
-      <c r="C108" s="10" t="n"/>
-      <c r="D108" s="10" t="n"/>
-      <c r="E108" s="10" t="n"/>
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="inlineStr">
+        <is>
+          <t>10681573</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="inlineStr">
+        <is>
+          <t>SERVING GLASS SQR TWO RACK ZENA GOLD</t>
+        </is>
+      </c>
       <c r="F108" s="10" t="n"/>
-      <c r="G108" s="10" t="n"/>
-      <c r="H108" s="10" t="n"/>
-      <c r="I108" s="10" t="n"/>
+      <c r="G108" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H108" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I108" s="10" t="inlineStr">
+        <is>
+          <t>W/GOLD RACK GLASS</t>
+        </is>
+      </c>
       <c r="J108" s="10" t="n"/>
       <c r="K108" s="10" t="n"/>
-      <c r="L108" s="11" t="n"/>
-      <c r="M108" s="11" t="n"/>
-      <c r="N108" s="11" t="n"/>
+      <c r="L108" s="11" t="inlineStr">
+        <is>
+          <t>WLL-03</t>
+        </is>
+      </c>
+      <c r="M108" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N108" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O108" s="12">
         <f>IF(L108="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L108,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10630,20 +11190,62 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="10" t="n"/>
-      <c r="B109" s="10" t="n"/>
-      <c r="C109" s="10" t="n"/>
-      <c r="D109" s="10" t="n"/>
-      <c r="E109" s="10" t="n"/>
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>10681574</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
+        <is>
+          <t>SERVING GLASS RND TWO RACK ZIA GOLD</t>
+        </is>
+      </c>
       <c r="F109" s="10" t="n"/>
-      <c r="G109" s="10" t="n"/>
-      <c r="H109" s="10" t="n"/>
-      <c r="I109" s="10" t="n"/>
+      <c r="G109" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H109" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t>W/GOLD RACK GLASS</t>
+        </is>
+      </c>
       <c r="J109" s="10" t="n"/>
       <c r="K109" s="10" t="n"/>
-      <c r="L109" s="11" t="n"/>
-      <c r="M109" s="11" t="n"/>
-      <c r="N109" s="11" t="n"/>
+      <c r="L109" s="11" t="inlineStr">
+        <is>
+          <t>WLL-03</t>
+        </is>
+      </c>
+      <c r="M109" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N109" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O109" s="12">
         <f>IF(L109="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L109,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10676,20 +11278,62 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="10" t="n"/>
-      <c r="B110" s="10" t="n"/>
-      <c r="C110" s="10" t="n"/>
-      <c r="D110" s="10" t="n"/>
-      <c r="E110" s="10" t="n"/>
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>10470030</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET RND DETACHABLE MARBLE (2)</t>
+        </is>
+      </c>
       <c r="F110" s="10" t="n"/>
-      <c r="G110" s="10" t="n"/>
-      <c r="H110" s="10" t="n"/>
-      <c r="I110" s="10" t="n"/>
+      <c r="G110" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H110" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I110" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET MARBLE</t>
+        </is>
+      </c>
       <c r="J110" s="10" t="n"/>
       <c r="K110" s="10" t="n"/>
-      <c r="L110" s="11" t="n"/>
-      <c r="M110" s="11" t="n"/>
-      <c r="N110" s="11" t="n"/>
+      <c r="L110" s="11" t="inlineStr">
+        <is>
+          <t>WLL-03</t>
+        </is>
+      </c>
+      <c r="M110" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N110" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O110" s="12">
         <f>IF(L110="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L110,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10722,20 +11366,62 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="10" t="n"/>
-      <c r="B111" s="10" t="n"/>
-      <c r="C111" s="10" t="n"/>
-      <c r="D111" s="10" t="n"/>
-      <c r="E111" s="10" t="n"/>
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>10470031</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET W/RACK SQR MARBLE BLACK (3)</t>
+        </is>
+      </c>
       <c r="F111" s="10" t="n"/>
-      <c r="G111" s="10" t="n"/>
-      <c r="H111" s="10" t="n"/>
-      <c r="I111" s="10" t="n"/>
+      <c r="G111" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H111" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I111" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET MARBLE</t>
+        </is>
+      </c>
       <c r="J111" s="10" t="n"/>
       <c r="K111" s="10" t="n"/>
-      <c r="L111" s="11" t="n"/>
-      <c r="M111" s="11" t="n"/>
-      <c r="N111" s="11" t="n"/>
+      <c r="L111" s="11" t="inlineStr">
+        <is>
+          <t>WLL-03</t>
+        </is>
+      </c>
+      <c r="M111" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N111" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O111" s="12">
         <f>IF(L111="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L111,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10768,20 +11454,62 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="10" t="n"/>
-      <c r="B112" s="10" t="n"/>
-      <c r="C112" s="10" t="n"/>
-      <c r="D112" s="10" t="n"/>
-      <c r="E112" s="10" t="n"/>
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t>Tableware</t>
+        </is>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>Serving Set</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>10470032</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET W/RACK STACK WHITE (3)</t>
+        </is>
+      </c>
       <c r="F112" s="10" t="n"/>
-      <c r="G112" s="10" t="n"/>
-      <c r="H112" s="10" t="n"/>
-      <c r="I112" s="10" t="n"/>
+      <c r="G112" s="10" t="inlineStr">
+        <is>
+          <t>MAKAN</t>
+        </is>
+      </c>
+      <c r="H112" s="10" t="inlineStr">
+        <is>
+          <t>A2. SERVINGWARE</t>
+        </is>
+      </c>
+      <c r="I112" s="10" t="inlineStr">
+        <is>
+          <t>SERVING SET MARBLE</t>
+        </is>
+      </c>
       <c r="J112" s="10" t="n"/>
       <c r="K112" s="10" t="n"/>
-      <c r="L112" s="11" t="n"/>
-      <c r="M112" s="11" t="n"/>
-      <c r="N112" s="11" t="n"/>
+      <c r="L112" s="11" t="inlineStr">
+        <is>
+          <t>WLL-03</t>
+        </is>
+      </c>
+      <c r="M112" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="N112" s="11" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
       <c r="O112" s="12">
         <f>IF(L112="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L112,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10814,20 +11542,62 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="10" t="n"/>
-      <c r="B113" s="10" t="n"/>
-      <c r="C113" s="10" t="n"/>
-      <c r="D113" s="10" t="n"/>
-      <c r="E113" s="10" t="n"/>
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>10198149</t>
+        </is>
+      </c>
+      <c r="E113" s="10" t="inlineStr">
+        <is>
+          <t>TANTA STRAINER DIA 10CM</t>
+        </is>
+      </c>
       <c r="F113" s="10" t="n"/>
-      <c r="G113" s="10" t="n"/>
-      <c r="H113" s="10" t="n"/>
-      <c r="I113" s="10" t="n"/>
+      <c r="G113" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H113" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I113" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S</t>
+        </is>
+      </c>
       <c r="J113" s="10" t="n"/>
       <c r="K113" s="10" t="n"/>
-      <c r="L113" s="11" t="n"/>
-      <c r="M113" s="11" t="n"/>
-      <c r="N113" s="11" t="n"/>
+      <c r="L113" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M113" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N113" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O113" s="12">
         <f>IF(L113="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L113,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10860,20 +11630,62 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="10" t="n"/>
-      <c r="B114" s="10" t="n"/>
-      <c r="C114" s="10" t="n"/>
-      <c r="D114" s="10" t="n"/>
-      <c r="E114" s="10" t="n"/>
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>10198150</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON TONGS 9 INCH</t>
+        </is>
+      </c>
       <c r="F114" s="10" t="n"/>
-      <c r="G114" s="10" t="n"/>
-      <c r="H114" s="10" t="n"/>
-      <c r="I114" s="10" t="n"/>
+      <c r="G114" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H114" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I114" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J114" s="10" t="n"/>
       <c r="K114" s="10" t="n"/>
-      <c r="L114" s="11" t="n"/>
-      <c r="M114" s="11" t="n"/>
-      <c r="N114" s="11" t="n"/>
+      <c r="L114" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M114" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N114" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O114" s="12">
         <f>IF(L114="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L114,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10906,20 +11718,62 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="10" t="n"/>
-      <c r="B115" s="10" t="n"/>
-      <c r="C115" s="10" t="n"/>
-      <c r="D115" s="10" t="n"/>
-      <c r="E115" s="10" t="n"/>
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>10198151</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON TONGS 12 INCH</t>
+        </is>
+      </c>
       <c r="F115" s="10" t="n"/>
-      <c r="G115" s="10" t="n"/>
-      <c r="H115" s="10" t="n"/>
-      <c r="I115" s="10" t="n"/>
+      <c r="G115" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H115" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I115" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J115" s="10" t="n"/>
       <c r="K115" s="10" t="n"/>
-      <c r="L115" s="11" t="n"/>
-      <c r="M115" s="11" t="n"/>
-      <c r="N115" s="11" t="n"/>
+      <c r="L115" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M115" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N115" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O115" s="12">
         <f>IF(L115="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L115,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10952,20 +11806,62 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="10" t="n"/>
-      <c r="B116" s="10" t="n"/>
-      <c r="C116" s="10" t="n"/>
-      <c r="D116" s="10" t="n"/>
-      <c r="E116" s="10" t="n"/>
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>10198152</t>
+        </is>
+      </c>
+      <c r="E116" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S SOLID TURNER M</t>
+        </is>
+      </c>
       <c r="F116" s="10" t="n"/>
-      <c r="G116" s="10" t="n"/>
-      <c r="H116" s="10" t="n"/>
-      <c r="I116" s="10" t="n"/>
+      <c r="G116" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H116" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I116" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S</t>
+        </is>
+      </c>
       <c r="J116" s="10" t="n"/>
       <c r="K116" s="10" t="n"/>
-      <c r="L116" s="11" t="n"/>
-      <c r="M116" s="11" t="n"/>
-      <c r="N116" s="11" t="n"/>
+      <c r="L116" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M116" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N116" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O116" s="12">
         <f>IF(L116="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L116,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -10998,20 +11894,62 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="10" t="n"/>
-      <c r="B117" s="10" t="n"/>
-      <c r="C117" s="10" t="n"/>
-      <c r="D117" s="10" t="n"/>
-      <c r="E117" s="10" t="n"/>
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>10198154</t>
+        </is>
+      </c>
+      <c r="E117" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S LADLE</t>
+        </is>
+      </c>
       <c r="F117" s="10" t="n"/>
-      <c r="G117" s="10" t="n"/>
-      <c r="H117" s="10" t="n"/>
-      <c r="I117" s="10" t="n"/>
+      <c r="G117" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H117" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I117" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S</t>
+        </is>
+      </c>
       <c r="J117" s="10" t="n"/>
       <c r="K117" s="10" t="n"/>
-      <c r="L117" s="11" t="n"/>
-      <c r="M117" s="11" t="n"/>
-      <c r="N117" s="11" t="n"/>
+      <c r="L117" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M117" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N117" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O117" s="12">
         <f>IF(L117="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L117,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11044,20 +11982,62 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="10" t="n"/>
-      <c r="B118" s="10" t="n"/>
-      <c r="C118" s="10" t="n"/>
-      <c r="D118" s="10" t="n"/>
-      <c r="E118" s="10" t="n"/>
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>10198156</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON SLOTTED TURNER M</t>
+        </is>
+      </c>
       <c r="F118" s="10" t="n"/>
-      <c r="G118" s="10" t="n"/>
-      <c r="H118" s="10" t="n"/>
-      <c r="I118" s="10" t="n"/>
+      <c r="G118" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J118" s="10" t="n"/>
       <c r="K118" s="10" t="n"/>
-      <c r="L118" s="11" t="n"/>
-      <c r="M118" s="11" t="n"/>
-      <c r="N118" s="11" t="n"/>
+      <c r="L118" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M118" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N118" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O118" s="12">
         <f>IF(L118="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L118,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11090,20 +12070,62 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="10" t="n"/>
-      <c r="B119" s="10" t="n"/>
-      <c r="C119" s="10" t="n"/>
-      <c r="D119" s="10" t="n"/>
-      <c r="E119" s="10" t="n"/>
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>10198157</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON SOLID TURNER L</t>
+        </is>
+      </c>
       <c r="F119" s="10" t="n"/>
-      <c r="G119" s="10" t="n"/>
-      <c r="H119" s="10" t="n"/>
-      <c r="I119" s="10" t="n"/>
+      <c r="G119" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H119" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J119" s="10" t="n"/>
       <c r="K119" s="10" t="n"/>
-      <c r="L119" s="11" t="n"/>
-      <c r="M119" s="11" t="n"/>
-      <c r="N119" s="11" t="n"/>
+      <c r="L119" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M119" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N119" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O119" s="12">
         <f>IF(L119="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L119,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11136,20 +12158,62 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="10" t="n"/>
-      <c r="B120" s="10" t="n"/>
-      <c r="C120" s="10" t="n"/>
-      <c r="D120" s="10" t="n"/>
-      <c r="E120" s="10" t="n"/>
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>10198159</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON LADLE</t>
+        </is>
+      </c>
       <c r="F120" s="10" t="n"/>
-      <c r="G120" s="10" t="n"/>
-      <c r="H120" s="10" t="n"/>
-      <c r="I120" s="10" t="n"/>
+      <c r="G120" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H120" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I120" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J120" s="10" t="n"/>
       <c r="K120" s="10" t="n"/>
-      <c r="L120" s="11" t="n"/>
-      <c r="M120" s="11" t="n"/>
-      <c r="N120" s="11" t="n"/>
+      <c r="L120" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M120" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N120" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O120" s="12">
         <f>IF(L120="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L120,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11182,20 +12246,62 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="10" t="n"/>
-      <c r="B121" s="10" t="n"/>
-      <c r="C121" s="10" t="n"/>
-      <c r="D121" s="10" t="n"/>
-      <c r="E121" s="10" t="n"/>
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>10198160</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON WHISK</t>
+        </is>
+      </c>
       <c r="F121" s="10" t="n"/>
-      <c r="G121" s="10" t="n"/>
-      <c r="H121" s="10" t="n"/>
-      <c r="I121" s="10" t="n"/>
+      <c r="G121" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H121" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I121" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J121" s="10" t="n"/>
       <c r="K121" s="10" t="n"/>
-      <c r="L121" s="11" t="n"/>
-      <c r="M121" s="11" t="n"/>
-      <c r="N121" s="11" t="n"/>
+      <c r="L121" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M121" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N121" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O121" s="12">
         <f>IF(L121="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L121,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11228,20 +12334,62 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="10" t="n"/>
-      <c r="B122" s="10" t="n"/>
-      <c r="C122" s="10" t="n"/>
-      <c r="D122" s="10" t="n"/>
-      <c r="E122" s="10" t="n"/>
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>10198149</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="inlineStr">
+        <is>
+          <t>TANTA STRAINER DIA 10CM</t>
+        </is>
+      </c>
       <c r="F122" s="10" t="n"/>
-      <c r="G122" s="10" t="n"/>
-      <c r="H122" s="10" t="n"/>
-      <c r="I122" s="10" t="n"/>
+      <c r="G122" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H122" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S</t>
+        </is>
+      </c>
       <c r="J122" s="10" t="n"/>
       <c r="K122" s="10" t="n"/>
-      <c r="L122" s="11" t="n"/>
-      <c r="M122" s="11" t="n"/>
-      <c r="N122" s="11" t="n"/>
+      <c r="L122" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M122" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N122" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O122" s="12">
         <f>IF(L122="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L122,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11274,20 +12422,62 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="10" t="n"/>
-      <c r="B123" s="10" t="n"/>
-      <c r="C123" s="10" t="n"/>
-      <c r="D123" s="10" t="n"/>
-      <c r="E123" s="10" t="n"/>
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>10198150</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON TONGS 9 INCH</t>
+        </is>
+      </c>
       <c r="F123" s="10" t="n"/>
-      <c r="G123" s="10" t="n"/>
-      <c r="H123" s="10" t="n"/>
-      <c r="I123" s="10" t="n"/>
+      <c r="G123" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H123" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I123" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J123" s="10" t="n"/>
       <c r="K123" s="10" t="n"/>
-      <c r="L123" s="11" t="n"/>
-      <c r="M123" s="11" t="n"/>
-      <c r="N123" s="11" t="n"/>
+      <c r="L123" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M123" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N123" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O123" s="12">
         <f>IF(L123="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L123,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11320,20 +12510,62 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="10" t="n"/>
-      <c r="B124" s="10" t="n"/>
-      <c r="C124" s="10" t="n"/>
-      <c r="D124" s="10" t="n"/>
-      <c r="E124" s="10" t="n"/>
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>10198151</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON TONGS 12 INCH</t>
+        </is>
+      </c>
       <c r="F124" s="10" t="n"/>
-      <c r="G124" s="10" t="n"/>
-      <c r="H124" s="10" t="n"/>
-      <c r="I124" s="10" t="n"/>
+      <c r="G124" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H124" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I124" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J124" s="10" t="n"/>
       <c r="K124" s="10" t="n"/>
-      <c r="L124" s="11" t="n"/>
-      <c r="M124" s="11" t="n"/>
-      <c r="N124" s="11" t="n"/>
+      <c r="L124" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M124" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N124" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O124" s="12">
         <f>IF(L124="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L124,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11366,20 +12598,62 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="10" t="n"/>
-      <c r="B125" s="10" t="n"/>
-      <c r="C125" s="10" t="n"/>
-      <c r="D125" s="10" t="n"/>
-      <c r="E125" s="10" t="n"/>
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>10198152</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S SOLID TURNER M</t>
+        </is>
+      </c>
       <c r="F125" s="10" t="n"/>
-      <c r="G125" s="10" t="n"/>
-      <c r="H125" s="10" t="n"/>
-      <c r="I125" s="10" t="n"/>
+      <c r="G125" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H125" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I125" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S</t>
+        </is>
+      </c>
       <c r="J125" s="10" t="n"/>
       <c r="K125" s="10" t="n"/>
-      <c r="L125" s="11" t="n"/>
-      <c r="M125" s="11" t="n"/>
-      <c r="N125" s="11" t="n"/>
+      <c r="L125" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M125" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N125" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O125" s="12">
         <f>IF(L125="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L125,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11412,20 +12686,62 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="10" t="n"/>
-      <c r="B126" s="10" t="n"/>
-      <c r="C126" s="10" t="n"/>
-      <c r="D126" s="10" t="n"/>
-      <c r="E126" s="10" t="n"/>
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>10198154</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S LADLE</t>
+        </is>
+      </c>
       <c r="F126" s="10" t="n"/>
-      <c r="G126" s="10" t="n"/>
-      <c r="H126" s="10" t="n"/>
-      <c r="I126" s="10" t="n"/>
+      <c r="G126" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H126" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I126" s="10" t="inlineStr">
+        <is>
+          <t>TANTA S/S</t>
+        </is>
+      </c>
       <c r="J126" s="10" t="n"/>
       <c r="K126" s="10" t="n"/>
-      <c r="L126" s="11" t="n"/>
-      <c r="M126" s="11" t="n"/>
-      <c r="N126" s="11" t="n"/>
+      <c r="L126" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M126" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N126" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O126" s="12">
         <f>IF(L126="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L126,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11458,20 +12774,62 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="10" t="n"/>
-      <c r="B127" s="10" t="n"/>
-      <c r="C127" s="10" t="n"/>
-      <c r="D127" s="10" t="n"/>
-      <c r="E127" s="10" t="n"/>
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>10198156</t>
+        </is>
+      </c>
+      <c r="E127" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON SLOTTED TURNER M</t>
+        </is>
+      </c>
       <c r="F127" s="10" t="n"/>
-      <c r="G127" s="10" t="n"/>
-      <c r="H127" s="10" t="n"/>
-      <c r="I127" s="10" t="n"/>
+      <c r="G127" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H127" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I127" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J127" s="10" t="n"/>
       <c r="K127" s="10" t="n"/>
-      <c r="L127" s="11" t="n"/>
-      <c r="M127" s="11" t="n"/>
-      <c r="N127" s="11" t="n"/>
+      <c r="L127" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M127" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N127" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O127" s="12">
         <f>IF(L127="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L127,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11504,20 +12862,62 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="10" t="n"/>
-      <c r="B128" s="10" t="n"/>
-      <c r="C128" s="10" t="n"/>
-      <c r="D128" s="10" t="n"/>
-      <c r="E128" s="10" t="n"/>
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="inlineStr">
+        <is>
+          <t>10198157</t>
+        </is>
+      </c>
+      <c r="E128" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON SOLID TURNER L</t>
+        </is>
+      </c>
       <c r="F128" s="10" t="n"/>
-      <c r="G128" s="10" t="n"/>
-      <c r="H128" s="10" t="n"/>
-      <c r="I128" s="10" t="n"/>
+      <c r="G128" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H128" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I128" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J128" s="10" t="n"/>
       <c r="K128" s="10" t="n"/>
-      <c r="L128" s="11" t="n"/>
-      <c r="M128" s="11" t="n"/>
-      <c r="N128" s="11" t="n"/>
+      <c r="L128" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M128" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N128" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O128" s="12">
         <f>IF(L128="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L128,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11550,20 +12950,62 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="10" t="n"/>
-      <c r="B129" s="10" t="n"/>
-      <c r="C129" s="10" t="n"/>
-      <c r="D129" s="10" t="n"/>
-      <c r="E129" s="10" t="n"/>
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B129" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>10198159</t>
+        </is>
+      </c>
+      <c r="E129" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON LADLE</t>
+        </is>
+      </c>
       <c r="F129" s="10" t="n"/>
-      <c r="G129" s="10" t="n"/>
-      <c r="H129" s="10" t="n"/>
-      <c r="I129" s="10" t="n"/>
+      <c r="G129" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H129" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I129" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J129" s="10" t="n"/>
       <c r="K129" s="10" t="n"/>
-      <c r="L129" s="11" t="n"/>
-      <c r="M129" s="11" t="n"/>
-      <c r="N129" s="11" t="n"/>
+      <c r="L129" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M129" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N129" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O129" s="12">
         <f>IF(L129="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L129,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>
@@ -11596,20 +13038,62 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="10" t="n"/>
-      <c r="B130" s="10" t="n"/>
-      <c r="C130" s="10" t="n"/>
-      <c r="D130" s="10" t="n"/>
-      <c r="E130" s="10" t="n"/>
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>Homeware</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>Kitchenware</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen Tools</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="inlineStr">
+        <is>
+          <t>10198160</t>
+        </is>
+      </c>
+      <c r="E130" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON WHISK</t>
+        </is>
+      </c>
       <c r="F130" s="10" t="n"/>
-      <c r="G130" s="10" t="n"/>
-      <c r="H130" s="10" t="n"/>
-      <c r="I130" s="10" t="n"/>
+      <c r="G130" s="10" t="inlineStr">
+        <is>
+          <t>ALAT MASAK</t>
+        </is>
+      </c>
+      <c r="H130" s="10" t="inlineStr">
+        <is>
+          <t>C1. KITCHEN TOOLS</t>
+        </is>
+      </c>
+      <c r="I130" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
       <c r="J130" s="10" t="n"/>
       <c r="K130" s="10" t="n"/>
-      <c r="L130" s="11" t="n"/>
-      <c r="M130" s="11" t="n"/>
-      <c r="N130" s="11" t="n"/>
+      <c r="L130" s="11" t="inlineStr">
+        <is>
+          <t>GND-03</t>
+        </is>
+      </c>
+      <c r="M130" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N130" s="11" t="inlineStr">
+        <is>
+          <t>Gantungan</t>
+        </is>
+      </c>
       <c r="O130" s="12">
         <f>IF(L130="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(L130,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
         <v/>

</xml_diff>